<commit_message>
Add scraped businesses data and update clients spreadsheet
- Introduced a new JSON file `scraped_businesses.json` containing detailed information about various hospitals, clinics, hotels, and restaurants sourced from Google.
- Updated the `clients.xlsx` file to reflect changes in the client data.
</commit_message>
<xml_diff>
--- a/job_hunter_agent/data/clients.xlsx
+++ b/job_hunter_agent/data/clients.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N89"/>
+  <dimension ref="A1:N95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -997,60 +997,72 @@
       <c r="N9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Aster Hospital: Best Multispeciality Hospital - Top Hospital in ...</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>hospital</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Dubai</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>https://www.asterhospitals.ae/</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>info@asterhospital.com</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>+971) 44 400 500</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Dr. Azad Moopen</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr"/>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Proposal: Custom Hospital CRM/ERP for Aster Hospital</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:13</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr"/>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 14:06</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>google_search</t>
         </is>
       </c>
-      <c r="M10" s="4" t="inlineStr"/>
-      <c r="N10" s="4" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1105,60 +1117,72 @@
       <c r="N11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Private hospitals | Ramsay Health Care UK</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>hospital</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>London</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>https://www.ramsayhealth.co.uk/</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Media.Enquiries@ramsayhealth.co.uk</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>0808 223 0500</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Mr Amir Sriemevan</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr"/>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Custom Hospital CRM/ERP Proposal for Ramsay Health Care UK</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:13</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr"/>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 14:08</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>google_search</t>
         </is>
       </c>
-      <c r="M12" s="4" t="inlineStr"/>
-      <c r="N12" s="4" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1357,52 +1381,64 @@
       <c r="N16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Your Private Practice in Berlin.</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>clinic</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Berlin</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>https://www.meoclinic.de/en/</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>info@meoclinic.de</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr"/>
-      <c r="G17" s="4" t="inlineStr"/>
-      <c r="H17" s="4" t="inlineStr"/>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Custom Clinic Management Web App Proposal</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:15</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr"/>
-      <c r="L17" s="4" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 14:10</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>google_search</t>
         </is>
       </c>
-      <c r="M17" s="4" t="inlineStr"/>
-      <c r="N17" s="4" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -2273,7 +2309,7 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>sales.hospitality@tfghospitality.com</t>
+          <t>reservations.businessbay@thefirstcollection.ae</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
@@ -3807,472 +3843,400 @@
       <c r="N67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="4" t="inlineStr">
+      <c r="A68" s="3" t="inlineStr">
         <is>
           <t>The British School of Amsterdam</t>
         </is>
       </c>
-      <c r="B68" s="4" t="inlineStr">
+      <c r="B68" s="3" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C68" s="4" t="inlineStr">
+      <c r="C68" s="3" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D68" s="4" t="inlineStr">
-        <is>
-          <t>https://www.britams.nl/</t>
-        </is>
-      </c>
-      <c r="E68" s="4" t="inlineStr">
-        <is>
-          <t>principal@britams.nl</t>
-        </is>
-      </c>
-      <c r="F68" s="4" t="inlineStr">
+      <c r="D68" s="3" t="inlineStr"/>
+      <c r="E68" s="3" t="inlineStr"/>
+      <c r="F68" s="3" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
         </is>
       </c>
-      <c r="G68" s="4" t="inlineStr"/>
-      <c r="H68" s="4" t="inlineStr"/>
-      <c r="I68" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J68" s="4" t="inlineStr">
+      <c r="G68" s="3" t="inlineStr"/>
+      <c r="H68" s="3" t="inlineStr"/>
+      <c r="I68" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J68" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K68" s="4" t="inlineStr"/>
-      <c r="L68" s="4" t="inlineStr">
-        <is>
-          <t>google_maps</t>
-        </is>
-      </c>
-      <c r="M68" s="4" t="inlineStr"/>
-      <c r="N68" s="4" t="inlineStr"/>
+      <c r="K68" s="3" t="inlineStr"/>
+      <c r="L68" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M68" s="3" t="inlineStr"/>
+      <c r="N68" s="3" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="4" t="inlineStr">
+      <c r="A69" s="3" t="inlineStr">
         <is>
           <t>Amsterdam International Community School (AICS South campus)</t>
         </is>
       </c>
-      <c r="B69" s="4" t="inlineStr">
+      <c r="B69" s="3" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C69" s="4" t="inlineStr">
+      <c r="C69" s="3" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D69" s="4" t="inlineStr">
-        <is>
-          <t>https://www.britams.nl/</t>
-        </is>
-      </c>
-      <c r="E69" s="4" t="inlineStr">
-        <is>
-          <t>principal@britams.nl</t>
-        </is>
-      </c>
-      <c r="F69" s="4" t="inlineStr">
+      <c r="D69" s="3" t="inlineStr"/>
+      <c r="E69" s="3" t="inlineStr"/>
+      <c r="F69" s="3" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
         </is>
       </c>
-      <c r="G69" s="4" t="inlineStr"/>
-      <c r="H69" s="4" t="inlineStr"/>
-      <c r="I69" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J69" s="4" t="inlineStr">
+      <c r="G69" s="3" t="inlineStr"/>
+      <c r="H69" s="3" t="inlineStr"/>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K69" s="4" t="inlineStr"/>
-      <c r="L69" s="4" t="inlineStr">
-        <is>
-          <t>google_maps</t>
-        </is>
-      </c>
-      <c r="M69" s="4" t="inlineStr"/>
-      <c r="N69" s="4" t="inlineStr"/>
+      <c r="K69" s="3" t="inlineStr"/>
+      <c r="L69" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M69" s="3" t="inlineStr"/>
+      <c r="N69" s="3" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="4" t="inlineStr">
+      <c r="A70" s="3" t="inlineStr">
         <is>
           <t>Amity International School, Amsterdam</t>
         </is>
       </c>
-      <c r="B70" s="4" t="inlineStr">
+      <c r="B70" s="3" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C70" s="4" t="inlineStr">
+      <c r="C70" s="3" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D70" s="4" t="inlineStr">
-        <is>
-          <t>https://www.britams.nl/</t>
-        </is>
-      </c>
-      <c r="E70" s="4" t="inlineStr">
-        <is>
-          <t>principal@britams.nl</t>
-        </is>
-      </c>
-      <c r="F70" s="4" t="inlineStr">
+      <c r="D70" s="3" t="inlineStr"/>
+      <c r="E70" s="3" t="inlineStr"/>
+      <c r="F70" s="3" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
         </is>
       </c>
-      <c r="G70" s="4" t="inlineStr"/>
-      <c r="H70" s="4" t="inlineStr"/>
-      <c r="I70" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J70" s="4" t="inlineStr">
+      <c r="G70" s="3" t="inlineStr"/>
+      <c r="H70" s="3" t="inlineStr"/>
+      <c r="I70" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J70" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K70" s="4" t="inlineStr"/>
-      <c r="L70" s="4" t="inlineStr">
-        <is>
-          <t>google_maps</t>
-        </is>
-      </c>
-      <c r="M70" s="4" t="inlineStr"/>
-      <c r="N70" s="4" t="inlineStr"/>
+      <c r="K70" s="3" t="inlineStr"/>
+      <c r="L70" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M70" s="3" t="inlineStr"/>
+      <c r="N70" s="3" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="4" t="inlineStr">
+      <c r="A71" s="3" t="inlineStr">
         <is>
           <t>Public Elementary School De Burght</t>
         </is>
       </c>
-      <c r="B71" s="4" t="inlineStr">
+      <c r="B71" s="3" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C71" s="4" t="inlineStr">
+      <c r="C71" s="3" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D71" s="4" t="inlineStr">
-        <is>
-          <t>https://www.britams.nl/</t>
-        </is>
-      </c>
-      <c r="E71" s="4" t="inlineStr">
-        <is>
-          <t>principal@britams.nl</t>
-        </is>
-      </c>
-      <c r="F71" s="4" t="inlineStr">
+      <c r="D71" s="3" t="inlineStr"/>
+      <c r="E71" s="3" t="inlineStr"/>
+      <c r="F71" s="3" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
         </is>
       </c>
-      <c r="G71" s="4" t="inlineStr"/>
-      <c r="H71" s="4" t="inlineStr"/>
-      <c r="I71" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J71" s="4" t="inlineStr">
+      <c r="G71" s="3" t="inlineStr"/>
+      <c r="H71" s="3" t="inlineStr"/>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J71" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K71" s="4" t="inlineStr"/>
-      <c r="L71" s="4" t="inlineStr">
-        <is>
-          <t>google_maps</t>
-        </is>
-      </c>
-      <c r="M71" s="4" t="inlineStr"/>
-      <c r="N71" s="4" t="inlineStr"/>
+      <c r="K71" s="3" t="inlineStr"/>
+      <c r="L71" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M71" s="3" t="inlineStr"/>
+      <c r="N71" s="3" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="4" t="inlineStr">
+      <c r="A72" s="3" t="inlineStr">
         <is>
           <t>International French School d'Amsterdam</t>
         </is>
       </c>
-      <c r="B72" s="4" t="inlineStr">
+      <c r="B72" s="3" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C72" s="4" t="inlineStr">
+      <c r="C72" s="3" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D72" s="4" t="inlineStr">
-        <is>
-          <t>https://www.britams.nl/</t>
-        </is>
-      </c>
-      <c r="E72" s="4" t="inlineStr">
-        <is>
-          <t>principal@britams.nl</t>
-        </is>
-      </c>
-      <c r="F72" s="4" t="inlineStr">
+      <c r="D72" s="3" t="inlineStr"/>
+      <c r="E72" s="3" t="inlineStr"/>
+      <c r="F72" s="3" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
         </is>
       </c>
-      <c r="G72" s="4" t="inlineStr"/>
-      <c r="H72" s="4" t="inlineStr"/>
-      <c r="I72" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J72" s="4" t="inlineStr">
+      <c r="G72" s="3" t="inlineStr"/>
+      <c r="H72" s="3" t="inlineStr"/>
+      <c r="I72" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J72" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K72" s="4" t="inlineStr"/>
-      <c r="L72" s="4" t="inlineStr">
-        <is>
-          <t>google_maps</t>
-        </is>
-      </c>
-      <c r="M72" s="4" t="inlineStr"/>
-      <c r="N72" s="4" t="inlineStr"/>
+      <c r="K72" s="3" t="inlineStr"/>
+      <c r="L72" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M72" s="3" t="inlineStr"/>
+      <c r="N72" s="3" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="4" t="inlineStr">
+      <c r="A73" s="3" t="inlineStr">
         <is>
           <t>Onze Amsterdamse School</t>
         </is>
       </c>
-      <c r="B73" s="4" t="inlineStr">
+      <c r="B73" s="3" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C73" s="4" t="inlineStr">
+      <c r="C73" s="3" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D73" s="4" t="inlineStr">
-        <is>
-          <t>https://www.britams.nl/</t>
-        </is>
-      </c>
-      <c r="E73" s="4" t="inlineStr">
-        <is>
-          <t>principal@britams.nl</t>
-        </is>
-      </c>
-      <c r="F73" s="4" t="inlineStr">
+      <c r="D73" s="3" t="inlineStr"/>
+      <c r="E73" s="3" t="inlineStr"/>
+      <c r="F73" s="3" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
         </is>
       </c>
-      <c r="G73" s="4" t="inlineStr"/>
-      <c r="H73" s="4" t="inlineStr"/>
-      <c r="I73" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J73" s="4" t="inlineStr">
+      <c r="G73" s="3" t="inlineStr"/>
+      <c r="H73" s="3" t="inlineStr"/>
+      <c r="I73" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J73" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K73" s="4" t="inlineStr"/>
-      <c r="L73" s="4" t="inlineStr">
-        <is>
-          <t>google_maps</t>
-        </is>
-      </c>
-      <c r="M73" s="4" t="inlineStr"/>
-      <c r="N73" s="4" t="inlineStr"/>
+      <c r="K73" s="3" t="inlineStr"/>
+      <c r="L73" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M73" s="3" t="inlineStr"/>
+      <c r="N73" s="3" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="4" t="inlineStr">
+      <c r="A74" s="3" t="inlineStr">
         <is>
           <t>New International School Esprit (DENISE)</t>
         </is>
       </c>
-      <c r="B74" s="4" t="inlineStr">
+      <c r="B74" s="3" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C74" s="4" t="inlineStr">
+      <c r="C74" s="3" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D74" s="4" t="inlineStr">
-        <is>
-          <t>https://www.britams.nl/</t>
-        </is>
-      </c>
-      <c r="E74" s="4" t="inlineStr">
-        <is>
-          <t>principal@britams.nl</t>
-        </is>
-      </c>
-      <c r="F74" s="4" t="inlineStr">
+      <c r="D74" s="3" t="inlineStr"/>
+      <c r="E74" s="3" t="inlineStr"/>
+      <c r="F74" s="3" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
         </is>
       </c>
-      <c r="G74" s="4" t="inlineStr"/>
-      <c r="H74" s="4" t="inlineStr"/>
-      <c r="I74" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J74" s="4" t="inlineStr">
+      <c r="G74" s="3" t="inlineStr"/>
+      <c r="H74" s="3" t="inlineStr"/>
+      <c r="I74" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J74" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K74" s="4" t="inlineStr"/>
-      <c r="L74" s="4" t="inlineStr">
-        <is>
-          <t>google_maps</t>
-        </is>
-      </c>
-      <c r="M74" s="4" t="inlineStr"/>
-      <c r="N74" s="4" t="inlineStr"/>
+      <c r="K74" s="3" t="inlineStr"/>
+      <c r="L74" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M74" s="3" t="inlineStr"/>
+      <c r="N74" s="3" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="4" t="inlineStr">
+      <c r="A75" s="3" t="inlineStr">
         <is>
           <t>Foundation The Japanese School of Amsterdam</t>
         </is>
       </c>
-      <c r="B75" s="4" t="inlineStr">
+      <c r="B75" s="3" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C75" s="4" t="inlineStr">
+      <c r="C75" s="3" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D75" s="4" t="inlineStr">
-        <is>
-          <t>https://www.britams.nl/</t>
-        </is>
-      </c>
-      <c r="E75" s="4" t="inlineStr">
-        <is>
-          <t>principal@britams.nl</t>
-        </is>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
+      <c r="D75" s="3" t="inlineStr"/>
+      <c r="E75" s="3" t="inlineStr"/>
+      <c r="F75" s="3" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
         </is>
       </c>
-      <c r="G75" s="4" t="inlineStr"/>
-      <c r="H75" s="4" t="inlineStr"/>
-      <c r="I75" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J75" s="4" t="inlineStr">
+      <c r="G75" s="3" t="inlineStr"/>
+      <c r="H75" s="3" t="inlineStr"/>
+      <c r="I75" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J75" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K75" s="4" t="inlineStr"/>
-      <c r="L75" s="4" t="inlineStr">
-        <is>
-          <t>google_maps</t>
-        </is>
-      </c>
-      <c r="M75" s="4" t="inlineStr"/>
-      <c r="N75" s="4" t="inlineStr"/>
+      <c r="K75" s="3" t="inlineStr"/>
+      <c r="L75" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M75" s="3" t="inlineStr"/>
+      <c r="N75" s="3" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="4" t="inlineStr">
+      <c r="A76" s="3" t="inlineStr">
         <is>
           <t>Private Education, Winford Amsterdam</t>
         </is>
       </c>
-      <c r="B76" s="4" t="inlineStr">
+      <c r="B76" s="3" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C76" s="4" t="inlineStr">
+      <c r="C76" s="3" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D76" s="4" t="inlineStr">
-        <is>
-          <t>https://www.britams.nl/</t>
-        </is>
-      </c>
-      <c r="E76" s="4" t="inlineStr">
-        <is>
-          <t>principal@britams.nl</t>
-        </is>
-      </c>
-      <c r="F76" s="4" t="inlineStr">
+      <c r="D76" s="3" t="inlineStr"/>
+      <c r="E76" s="3" t="inlineStr"/>
+      <c r="F76" s="3" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
         </is>
       </c>
-      <c r="G76" s="4" t="inlineStr"/>
-      <c r="H76" s="4" t="inlineStr"/>
-      <c r="I76" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J76" s="4" t="inlineStr">
+      <c r="G76" s="3" t="inlineStr"/>
+      <c r="H76" s="3" t="inlineStr"/>
+      <c r="I76" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J76" s="3" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K76" s="4" t="inlineStr"/>
-      <c r="L76" s="4" t="inlineStr">
-        <is>
-          <t>google_maps</t>
-        </is>
-      </c>
-      <c r="M76" s="4" t="inlineStr"/>
-      <c r="N76" s="4" t="inlineStr"/>
+      <c r="K76" s="3" t="inlineStr"/>
+      <c r="L76" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M76" s="3" t="inlineStr"/>
+      <c r="N76" s="3" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
@@ -4290,16 +4254,8 @@
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D77" s="4" t="inlineStr">
-        <is>
-          <t>https://www.britams.nl/</t>
-        </is>
-      </c>
-      <c r="E77" s="4" t="inlineStr">
-        <is>
-          <t>principal@britams.nl</t>
-        </is>
-      </c>
+      <c r="D77" s="4" t="inlineStr"/>
+      <c r="E77" s="4" t="inlineStr"/>
       <c r="F77" s="4" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
@@ -4342,16 +4298,8 @@
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D78" s="4" t="inlineStr">
-        <is>
-          <t>https://www.britams.nl/</t>
-        </is>
-      </c>
-      <c r="E78" s="4" t="inlineStr">
-        <is>
-          <t>principal@britams.nl</t>
-        </is>
-      </c>
+      <c r="D78" s="4" t="inlineStr"/>
+      <c r="E78" s="4" t="inlineStr"/>
       <c r="F78" s="4" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
@@ -4861,6 +4809,274 @@
       </c>
       <c r="M89" s="3" t="inlineStr"/>
       <c r="N89" s="3" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>Acibadem International Medical Center</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>https://www.amsterdamumc.nl/nl/locatie-vumc/adres.htm</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr"/>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>1117 1081</t>
+        </is>
+      </c>
+      <c r="G90" s="3" t="inlineStr"/>
+      <c r="H90" s="3" t="inlineStr"/>
+      <c r="I90" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J90" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 14:02</t>
+        </is>
+      </c>
+      <c r="K90" s="3" t="inlineStr"/>
+      <c r="L90" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M90" s="3" t="inlineStr"/>
+      <c r="N90" s="3" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>ZenDXB: Polyclinic focussed on Health, Wellness, and Home-care</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>clinic</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>private clinics Dubai</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr"/>
+      <c r="E91" s="3" t="inlineStr"/>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G91" s="3" t="inlineStr"/>
+      <c r="H91" s="3" t="inlineStr"/>
+      <c r="I91" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J91" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 14:03</t>
+        </is>
+      </c>
+      <c r="K91" s="3" t="inlineStr"/>
+      <c r="L91" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M91" s="3" t="inlineStr"/>
+      <c r="N91" s="3" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>Leman Locke Aldgate</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>hotels London</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr"/>
+      <c r="E92" s="3" t="inlineStr"/>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>+44 20 3327 7140</t>
+        </is>
+      </c>
+      <c r="G92" s="3" t="inlineStr"/>
+      <c r="H92" s="3" t="inlineStr"/>
+      <c r="I92" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J92" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 14:03</t>
+        </is>
+      </c>
+      <c r="K92" s="3" t="inlineStr"/>
+      <c r="L92" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M92" s="3" t="inlineStr"/>
+      <c r="N92" s="3" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>Gem Langham Court Hotel</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>hotels London</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr"/>
+      <c r="E93" s="3" t="inlineStr"/>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>+44 20 7436 6622</t>
+        </is>
+      </c>
+      <c r="G93" s="3" t="inlineStr"/>
+      <c r="H93" s="3" t="inlineStr"/>
+      <c r="I93" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J93" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 14:03</t>
+        </is>
+      </c>
+      <c r="K93" s="3" t="inlineStr"/>
+      <c r="L93" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M93" s="3" t="inlineStr"/>
+      <c r="N93" s="3" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>Rijksmuseum</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>school</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>schools Amsterdam</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr"/>
+      <c r="E94" s="3" t="inlineStr"/>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G94" s="3" t="inlineStr"/>
+      <c r="H94" s="3" t="inlineStr"/>
+      <c r="I94" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J94" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 14:03</t>
+        </is>
+      </c>
+      <c r="K94" s="3" t="inlineStr"/>
+      <c r="L94" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M94" s="3" t="inlineStr"/>
+      <c r="N94" s="3" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>HYVN REALTY LLC</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>real estate agencies Dubai</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr"/>
+      <c r="E95" s="3" t="inlineStr"/>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G95" s="3" t="inlineStr"/>
+      <c r="H95" s="3" t="inlineStr"/>
+      <c r="I95" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J95" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 14:04</t>
+        </is>
+      </c>
+      <c r="K95" s="3" t="inlineStr"/>
+      <c r="L95" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M95" s="3" t="inlineStr"/>
+      <c r="N95" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update job proposals, enhance emailer functionality, and add run_all script
- Increased score for Senior Frontend Developer proposal.
- Updated URL for Senior React Native Developer proposal.
- Modified scraped businesses data, including updates to snippets and removal of outdated entries.
- Improved emailer.py to handle Google API imports gracefully and refactored Gmail service authentication.
- Implemented IMAP fallback for reading replies and enhanced reply filtering.
- Added run_all.py script to streamline execution of both Job Hunter and Client Hunter bots with various options.
</commit_message>
<xml_diff>
--- a/job_hunter_agent/data/clients.xlsx
+++ b/job_hunter_agent/data/clients.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N95"/>
+  <dimension ref="A1:N122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -578,7 +578,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Elevate Patient Care with Customized Hospital Solution</t>
+          <t>Propose Custom Hospital CRM/ERP Solution</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -593,7 +593,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07 13:29</t>
+          <t>2026-05-07 17:27</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>jciquality@jcrinc.com</t>
+          <t>hr@zulekhahospitals.com</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -834,7 +834,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Transforming Patient Care with Customized Hospital Solutions</t>
+          <t>Propose Custom CRM/ERP Solution for Zulekha Hospital</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -849,7 +849,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07 13:32</t>
+          <t>2026-05-07 17:32</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Streamline Your Operations with Custom Healthcare Solutions</t>
+          <t>Custom Hospital CRM/ERP Proposal for Dubai Health Network</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07 13:34</t>
+          <t>2026-05-07 17:35</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -961,12 +961,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Prof. Dr</t>
+          <t>Dr. Tariq Aslam</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Streamline Your Hospital Operations with Customized Solution</t>
+          <t>Custom Hospital CRM/ERP Proposal - Al Zahra Hospital</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -981,7 +981,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07 13:36</t>
+          <t>2026-05-07 20:03</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1034,7 +1034,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Proposal: Custom Hospital CRM/ERP for Aster Hospital</t>
+          <t>Propose Custom Hospital CRM/ERP Solution for Aster Hospital</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1049,7 +1049,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07 14:06</t>
+          <t>2026-05-07 18:11</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07 14:08</t>
+          <t>2026-05-07 18:15</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -1425,7 +1425,7 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-07 14:10</t>
+          <t>2026-05-07 18:19</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -1441,117 +1441,141 @@
       <c r="N17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>PRIVATE CLINIC HOURS</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>clinic</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Berlin</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>https://familycareberlin.de/en/private-clinic-hours/</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>allgemeinmedizin@familycareberlin.de</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>+49 30 29 77 897 0</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Dr. Bernhard</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr"/>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J18" s="4" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Custom Clinic Management App Proposal</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:15</t>
         </is>
       </c>
-      <c r="K18" s="4" t="inlineStr"/>
-      <c r="L18" s="4" t="inlineStr">
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 18:23</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>google_search</t>
         </is>
       </c>
-      <c r="M18" s="4" t="inlineStr"/>
-      <c r="N18" s="4" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Dental Clinics</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>clinic</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Toronto</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>https://www.toronto.ca/community-people/health-wellness-care/health-programs-advice/dental-and-oral-health-services/dental-clinics/</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>supplychain@toronto.ca</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>416-338-7600</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Dr 
 Suite</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr"/>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Revolutionize Your Practice: Custom Clinic Management App</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:15</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr"/>
-      <c r="L19" s="4" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 18:32</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>google_search</t>
         </is>
       </c>
-      <c r="M19" s="4" t="inlineStr"/>
-      <c r="N19" s="4" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1794,109 +1818,133 @@
       <c r="N24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>De Pijp Boutique Hotel Amsterdam | Official website</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>hotel</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>https://www.depijpboutiquehotel.nl/</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>info@depijpboutiquehotel.nl</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>+31 (0) 20 676 031</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr"/>
-      <c r="H25" s="4" t="inlineStr"/>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Proposal: Custom Hotel Management System for De Pijp Boutique Hotel</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:18</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr"/>
-      <c r="L25" s="4" t="inlineStr">
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 18:36</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
         <is>
           <t>google_search</t>
         </is>
       </c>
-      <c r="M25" s="4" t="inlineStr"/>
-      <c r="N25" s="4" t="inlineStr"/>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>The Hendrick's | Boutique Hotel Amsterdam | Official Website</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>hotel</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>https://www.thehendrickshotel.com/</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>info@thehendrickshotel.com</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>139 
  1011</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr"/>
-      <c r="H26" s="4" t="inlineStr"/>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J26" s="4" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Proposal: Custom Hotel Management System</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:18</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr"/>
-      <c r="L26" s="4" t="inlineStr">
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 18:39</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>google_search</t>
         </is>
       </c>
-      <c r="M26" s="4" t="inlineStr"/>
-      <c r="N26" s="4" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1943,212 +1991,260 @@
       <c r="N27" s="3" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Hotel Notting Hill Amsterdam | City Centre Hotel - Official ...</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>hotel</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>https://www.hotelnottinghill.nl/</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>reservation@hotelnottinghill.nl</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>+31 (0) 20 523 10</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr"/>
-      <c r="H28" s="4" t="inlineStr"/>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J28" s="4" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom Hotel Management System Solution</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:18</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr"/>
-      <c r="L28" s="4" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 18:49</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
         <is>
           <t>google_search</t>
         </is>
       </c>
-      <c r="M28" s="4" t="inlineStr"/>
-      <c r="N28" s="4" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Boutique Hotel | Boutique Hotel View | Amsterdam</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>hotel</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>https://www.boutiquehotelview.nl/</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>info@boutiquehotelview.nl</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>+31205289668</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr"/>
-      <c r="H29" s="4" t="inlineStr"/>
-      <c r="I29" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J29" s="4" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom Hotel Management System</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:19</t>
         </is>
       </c>
-      <c r="K29" s="4" t="inlineStr"/>
-      <c r="L29" s="4" t="inlineStr">
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:10</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
         <is>
           <t>google_search</t>
         </is>
       </c>
-      <c r="M29" s="4" t="inlineStr"/>
-      <c r="N29" s="4" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>The Albus Boutique Hotel Amsterdam Centre</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>hotel</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>https://www.albushotel.com/</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>welcome@albushotel.com</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>+31 (0)20 530 6200</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr"/>
-      <c r="H30" s="4" t="inlineStr"/>
-      <c r="I30" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J30" s="4" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom Hotel Management System</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:19</t>
         </is>
       </c>
-      <c r="K30" s="4" t="inlineStr"/>
-      <c r="L30" s="4" t="inlineStr">
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 18:42</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
         <is>
           <t>google_search</t>
         </is>
       </c>
-      <c r="M30" s="4" t="inlineStr"/>
-      <c r="N30" s="4" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Park Regis Business Bay (Dubai)</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>hotel</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>Dubai</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>https://www.parkregisbusinessbay.com/</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>info@parkregisbusinessbay.com</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>2487486593</t>
         </is>
       </c>
-      <c r="G31" s="4" t="inlineStr"/>
-      <c r="H31" s="4" t="inlineStr"/>
-      <c r="I31" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J31" s="4" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Proposal: Custom Hotel Management System</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:19</t>
         </is>
       </c>
-      <c r="K31" s="4" t="inlineStr"/>
-      <c r="L31" s="4" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 18:53</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
         <is>
           <t>google_search</t>
         </is>
       </c>
-      <c r="M31" s="4" t="inlineStr"/>
-      <c r="N31" s="4" t="inlineStr"/>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -2287,56 +2383,68 @@
       <c r="N34" s="3" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Hotel in Dubai Business Bay</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>hotel</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>Dubai</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>https://www.thefirstcollection.ae/business-bay/</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>reservations.businessbay@thefirstcollection.ae</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>+971 4 873 4444</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr"/>
-      <c r="H35" s="4" t="inlineStr"/>
-      <c r="I35" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J35" s="4" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom Hotel Management System</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:20</t>
         </is>
       </c>
-      <c r="K35" s="4" t="inlineStr"/>
-      <c r="L35" s="4" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 18:57</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
         <is>
           <t>google_search</t>
         </is>
       </c>
-      <c r="M35" s="4" t="inlineStr"/>
-      <c r="N35" s="4" t="inlineStr"/>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2439,56 +2547,68 @@
       <c r="N37" s="3" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>St. JOHN Restaurant</t>
         </is>
       </c>
-      <c r="B38" s="4" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>restaurant</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>London</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>https://stjohnrestaurant.com/</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>reservations@stjohnrestaurant.com</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>020 7251 0848</t>
         </is>
       </c>
-      <c r="G38" s="4" t="inlineStr"/>
-      <c r="H38" s="4" t="inlineStr"/>
-      <c r="I38" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J38" s="4" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Custom Mobile-Friendly App for St. John's Restaurant</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:20</t>
         </is>
       </c>
-      <c r="K38" s="4" t="inlineStr"/>
-      <c r="L38" s="4" t="inlineStr">
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:15</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
         <is>
           <t>google_search</t>
         </is>
       </c>
-      <c r="M38" s="4" t="inlineStr"/>
-      <c r="N38" s="4" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -2543,52 +2663,64 @@
       <c r="N39" s="4" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>Fallow - Restaurant London - Creative Cooking Sustainable ...</t>
         </is>
       </c>
-      <c r="B40" s="4" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>restaurant</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>London</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>https://fallowrestaurant.com/</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>info@fallowrestaurant.com</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr"/>
-      <c r="G40" s="4" t="inlineStr"/>
-      <c r="H40" s="4" t="inlineStr"/>
-      <c r="I40" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J40" s="4" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Build Your Sustainable Restaurant App: Mobile Solution Proposal</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:20</t>
         </is>
       </c>
-      <c r="K40" s="4" t="inlineStr"/>
-      <c r="L40" s="4" t="inlineStr">
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:17</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
         <is>
           <t>google_search</t>
         </is>
       </c>
-      <c r="M40" s="4" t="inlineStr"/>
-      <c r="N40" s="4" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -3626,7 +3758,7 @@
       <c r="E63" s="3" t="inlineStr"/>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>0333 234 6605</t>
+          <t>+44 20 7603 3355</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr"/>
@@ -3722,7 +3854,7 @@
       <c r="E65" s="3" t="inlineStr"/>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>+44 (0) 20 78 70 6</t>
+          <t>46263680613</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr"/>
@@ -3747,540 +3879,780 @@
       <c r="N65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="inlineStr">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>The Rose &amp; Crown, London Bridge (PUBLOVE)</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>hotel</t>
         </is>
       </c>
-      <c r="C66" s="3" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>hotels London</t>
         </is>
       </c>
-      <c r="D66" s="3" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>https://zedwellhotels.com/locations/london/piccadilly-circus/piccadilly-circus-hotel</t>
         </is>
       </c>
-      <c r="E66" s="3" t="inlineStr"/>
-      <c r="F66" s="3" t="inlineStr">
-        <is>
-          <t>+44 (0) 20 78 70 6</t>
-        </is>
-      </c>
-      <c r="G66" s="3" t="inlineStr"/>
-      <c r="H66" s="3" t="inlineStr"/>
-      <c r="I66" s="3" t="inlineStr">
-        <is>
-          <t>no_email</t>
-        </is>
-      </c>
-      <c r="J66" s="3" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>reservations@publove.co.uk</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>+44 20 7407 7090</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Head Clerkenwell  View</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>Proposal: Custom Hotel Management System</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:24</t>
         </is>
       </c>
-      <c r="K66" s="3" t="inlineStr"/>
-      <c r="L66" s="3" t="inlineStr">
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:30</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr">
         <is>
           <t>google_maps</t>
         </is>
       </c>
-      <c r="M66" s="3" t="inlineStr"/>
-      <c r="N66" s="3" t="inlineStr"/>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="3" t="inlineStr">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>The Steam Engine, Waterloo (PUBLOVE)</t>
         </is>
       </c>
-      <c r="B67" s="3" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
         <is>
           <t>hotel</t>
         </is>
       </c>
-      <c r="C67" s="3" t="inlineStr">
+      <c r="C67" s="2" t="inlineStr">
         <is>
           <t>hotels London</t>
         </is>
       </c>
-      <c r="D67" s="3" t="inlineStr">
+      <c r="D67" s="2" t="inlineStr">
         <is>
           <t>https://zedwellhotels.com/locations/london/piccadilly-circus/piccadilly-circus-hotel</t>
         </is>
       </c>
-      <c r="E67" s="3" t="inlineStr"/>
-      <c r="F67" s="3" t="inlineStr">
-        <is>
-          <t>+44 (0) 20 78 70 6</t>
-        </is>
-      </c>
-      <c r="G67" s="3" t="inlineStr"/>
-      <c r="H67" s="3" t="inlineStr"/>
-      <c r="I67" s="3" t="inlineStr">
-        <is>
-          <t>no_email</t>
-        </is>
-      </c>
-      <c r="J67" s="3" t="inlineStr">
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>reservations@publove.co.uk</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>+44 20 7407 7090</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>Head Clerkenwell  View</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>Proposal: Custom Hotel Management System</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K67" s="3" t="inlineStr"/>
-      <c r="L67" s="3" t="inlineStr">
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:32</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr">
         <is>
           <t>google_maps</t>
         </is>
       </c>
-      <c r="M67" s="3" t="inlineStr"/>
-      <c r="N67" s="3" t="inlineStr"/>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="3" t="inlineStr">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>The British School of Amsterdam</t>
         </is>
       </c>
-      <c r="B68" s="3" t="inlineStr">
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C68" s="3" t="inlineStr">
+      <c r="C68" s="2" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D68" s="3" t="inlineStr"/>
-      <c r="E68" s="3" t="inlineStr"/>
-      <c r="F68" s="3" t="inlineStr">
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>https://www.britams.nl/</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>principal@britams.nl</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
         </is>
       </c>
-      <c r="G68" s="3" t="inlineStr"/>
-      <c r="H68" s="3" t="inlineStr"/>
-      <c r="I68" s="3" t="inlineStr">
-        <is>
-          <t>no_email</t>
-        </is>
-      </c>
-      <c r="J68" s="3" t="inlineStr">
+      <c r="G68" s="2" t="inlineStr"/>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Proposal: Custom College CRM Solution for The British School of Amsterdam</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K68" s="3" t="inlineStr"/>
-      <c r="L68" s="3" t="inlineStr">
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:28</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr">
         <is>
           <t>google_maps</t>
         </is>
       </c>
-      <c r="M68" s="3" t="inlineStr"/>
-      <c r="N68" s="3" t="inlineStr"/>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="3" t="inlineStr">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>Amsterdam International Community School (AICS South campus)</t>
         </is>
       </c>
-      <c r="B69" s="3" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C69" s="3" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D69" s="3" t="inlineStr"/>
-      <c r="E69" s="3" t="inlineStr"/>
-      <c r="F69" s="3" t="inlineStr">
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>https://www.britams.nl/</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>principal@britams.nl</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
         </is>
       </c>
-      <c r="G69" s="3" t="inlineStr"/>
-      <c r="H69" s="3" t="inlineStr"/>
-      <c r="I69" s="3" t="inlineStr">
-        <is>
-          <t>no_email</t>
-        </is>
-      </c>
-      <c r="J69" s="3" t="inlineStr">
+      <c r="G69" s="2" t="inlineStr"/>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>Proposal: Custom CRM Solution for AICS South Campus</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K69" s="3" t="inlineStr"/>
-      <c r="L69" s="3" t="inlineStr">
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:32</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
         <is>
           <t>google_maps</t>
         </is>
       </c>
-      <c r="M69" s="3" t="inlineStr"/>
-      <c r="N69" s="3" t="inlineStr"/>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="3" t="inlineStr">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t>Amity International School, Amsterdam</t>
         </is>
       </c>
-      <c r="B70" s="3" t="inlineStr">
+      <c r="B70" s="2" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C70" s="3" t="inlineStr">
+      <c r="C70" s="2" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D70" s="3" t="inlineStr"/>
-      <c r="E70" s="3" t="inlineStr"/>
-      <c r="F70" s="3" t="inlineStr">
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>https://www.britams.nl/</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>principal@britams.nl</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
         </is>
       </c>
-      <c r="G70" s="3" t="inlineStr"/>
-      <c r="H70" s="3" t="inlineStr"/>
-      <c r="I70" s="3" t="inlineStr">
-        <is>
-          <t>no_email</t>
-        </is>
-      </c>
-      <c r="J70" s="3" t="inlineStr">
+      <c r="G70" s="2" t="inlineStr"/>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom College CRM Solution for Amity International School</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K70" s="3" t="inlineStr"/>
-      <c r="L70" s="3" t="inlineStr">
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:34</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
         <is>
           <t>google_maps</t>
         </is>
       </c>
-      <c r="M70" s="3" t="inlineStr"/>
-      <c r="N70" s="3" t="inlineStr"/>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="3" t="inlineStr">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>Public Elementary School De Burght</t>
         </is>
       </c>
-      <c r="B71" s="3" t="inlineStr">
+      <c r="B71" s="2" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C71" s="3" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D71" s="3" t="inlineStr"/>
-      <c r="E71" s="3" t="inlineStr"/>
-      <c r="F71" s="3" t="inlineStr">
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>https://www.britams.nl/</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>principal@britams.nl</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
         </is>
       </c>
-      <c r="G71" s="3" t="inlineStr"/>
-      <c r="H71" s="3" t="inlineStr"/>
-      <c r="I71" s="3" t="inlineStr">
-        <is>
-          <t>no_email</t>
-        </is>
-      </c>
-      <c r="J71" s="3" t="inlineStr">
+      <c r="G71" s="2" t="inlineStr"/>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>Custom College/School CRM Proposal: Public Elementary School de Burght</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K71" s="3" t="inlineStr"/>
-      <c r="L71" s="3" t="inlineStr">
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:39</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="inlineStr">
         <is>
           <t>google_maps</t>
         </is>
       </c>
-      <c r="M71" s="3" t="inlineStr"/>
-      <c r="N71" s="3" t="inlineStr"/>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="3" t="inlineStr">
+      <c r="A72" s="2" t="inlineStr">
         <is>
           <t>International French School d'Amsterdam</t>
         </is>
       </c>
-      <c r="B72" s="3" t="inlineStr">
+      <c r="B72" s="2" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C72" s="3" t="inlineStr">
+      <c r="C72" s="2" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D72" s="3" t="inlineStr"/>
-      <c r="E72" s="3" t="inlineStr"/>
-      <c r="F72" s="3" t="inlineStr">
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.britams.nl/</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>principal@britams.nl</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
         </is>
       </c>
-      <c r="G72" s="3" t="inlineStr"/>
-      <c r="H72" s="3" t="inlineStr"/>
-      <c r="I72" s="3" t="inlineStr">
-        <is>
-          <t>no_email</t>
-        </is>
-      </c>
-      <c r="J72" s="3" t="inlineStr">
+      <c r="G72" s="2" t="inlineStr"/>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>Proposal: Customized College/School CRM Solution</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K72" s="3" t="inlineStr"/>
-      <c r="L72" s="3" t="inlineStr">
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:36</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="inlineStr">
         <is>
           <t>google_maps</t>
         </is>
       </c>
-      <c r="M72" s="3" t="inlineStr"/>
-      <c r="N72" s="3" t="inlineStr"/>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="3" t="inlineStr">
+      <c r="A73" s="2" t="inlineStr">
         <is>
           <t>Onze Amsterdamse School</t>
         </is>
       </c>
-      <c r="B73" s="3" t="inlineStr">
+      <c r="B73" s="2" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C73" s="3" t="inlineStr">
+      <c r="C73" s="2" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D73" s="3" t="inlineStr"/>
-      <c r="E73" s="3" t="inlineStr"/>
-      <c r="F73" s="3" t="inlineStr">
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>https://www.britams.nl/</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>principal@britams.nl</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
         </is>
       </c>
-      <c r="G73" s="3" t="inlineStr"/>
-      <c r="H73" s="3" t="inlineStr"/>
-      <c r="I73" s="3" t="inlineStr">
-        <is>
-          <t>no_email</t>
-        </is>
-      </c>
-      <c r="J73" s="3" t="inlineStr">
+      <c r="G73" s="2" t="inlineStr"/>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>Propose: Custom College CRM Solution for Onze Amsterdamse School</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K73" s="3" t="inlineStr"/>
-      <c r="L73" s="3" t="inlineStr">
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:36</t>
+        </is>
+      </c>
+      <c r="L73" s="2" t="inlineStr">
         <is>
           <t>google_maps</t>
         </is>
       </c>
-      <c r="M73" s="3" t="inlineStr"/>
-      <c r="N73" s="3" t="inlineStr"/>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="3" t="inlineStr">
+      <c r="A74" s="2" t="inlineStr">
         <is>
           <t>New International School Esprit (DENISE)</t>
         </is>
       </c>
-      <c r="B74" s="3" t="inlineStr">
+      <c r="B74" s="2" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C74" s="3" t="inlineStr">
+      <c r="C74" s="2" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D74" s="3" t="inlineStr"/>
-      <c r="E74" s="3" t="inlineStr"/>
-      <c r="F74" s="3" t="inlineStr">
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>https://www.britams.nl/</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>principal@britams.nl</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
         </is>
       </c>
-      <c r="G74" s="3" t="inlineStr"/>
-      <c r="H74" s="3" t="inlineStr"/>
-      <c r="I74" s="3" t="inlineStr">
-        <is>
-          <t>no_email</t>
-        </is>
-      </c>
-      <c r="J74" s="3" t="inlineStr">
+      <c r="G74" s="2" t="inlineStr"/>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>Custom College CRM Proposal for New International School Esprit - DENISE</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K74" s="3" t="inlineStr"/>
-      <c r="L74" s="3" t="inlineStr">
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:41</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="inlineStr">
         <is>
           <t>google_maps</t>
         </is>
       </c>
-      <c r="M74" s="3" t="inlineStr"/>
-      <c r="N74" s="3" t="inlineStr"/>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N74" s="2" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="3" t="inlineStr">
+      <c r="A75" s="2" t="inlineStr">
         <is>
           <t>Foundation The Japanese School of Amsterdam</t>
         </is>
       </c>
-      <c r="B75" s="3" t="inlineStr">
+      <c r="B75" s="2" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C75" s="3" t="inlineStr">
+      <c r="C75" s="2" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D75" s="3" t="inlineStr"/>
-      <c r="E75" s="3" t="inlineStr"/>
-      <c r="F75" s="3" t="inlineStr">
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>https://www.britams.nl/</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>principal@britams.nl</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
         </is>
       </c>
-      <c r="G75" s="3" t="inlineStr"/>
-      <c r="H75" s="3" t="inlineStr"/>
-      <c r="I75" s="3" t="inlineStr">
-        <is>
-          <t>no_email</t>
-        </is>
-      </c>
-      <c r="J75" s="3" t="inlineStr">
+      <c r="G75" s="2" t="inlineStr"/>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>Proposal: Custom CRM Solution for TJSA College Management</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K75" s="3" t="inlineStr"/>
-      <c r="L75" s="3" t="inlineStr">
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:47</t>
+        </is>
+      </c>
+      <c r="L75" s="2" t="inlineStr">
         <is>
           <t>google_maps</t>
         </is>
       </c>
-      <c r="M75" s="3" t="inlineStr"/>
-      <c r="N75" s="3" t="inlineStr"/>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N75" s="2" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="3" t="inlineStr">
+      <c r="A76" s="2" t="inlineStr">
         <is>
           <t>Private Education, Winford Amsterdam</t>
         </is>
       </c>
-      <c r="B76" s="3" t="inlineStr">
+      <c r="B76" s="2" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C76" s="3" t="inlineStr">
+      <c r="C76" s="2" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D76" s="3" t="inlineStr"/>
-      <c r="E76" s="3" t="inlineStr"/>
-      <c r="F76" s="3" t="inlineStr">
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>https://www.britams.nl/</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>principal@britams.nl</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
         </is>
       </c>
-      <c r="G76" s="3" t="inlineStr"/>
-      <c r="H76" s="3" t="inlineStr"/>
-      <c r="I76" s="3" t="inlineStr">
-        <is>
-          <t>no_email</t>
-        </is>
-      </c>
-      <c r="J76" s="3" t="inlineStr">
+      <c r="G76" s="2" t="inlineStr"/>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>Custom College CRM Proposal for Winford Amsterdam</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K76" s="3" t="inlineStr"/>
-      <c r="L76" s="3" t="inlineStr">
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:44</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="inlineStr">
         <is>
           <t>google_maps</t>
         </is>
       </c>
-      <c r="M76" s="3" t="inlineStr"/>
-      <c r="N76" s="3" t="inlineStr"/>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="4" t="inlineStr">
+      <c r="A77" s="2" t="inlineStr">
         <is>
           <t>Winford Bilingual Primary School</t>
         </is>
       </c>
-      <c r="B77" s="4" t="inlineStr">
+      <c r="B77" s="2" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C77" s="4" t="inlineStr">
+      <c r="C77" s="2" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D77" s="4" t="inlineStr"/>
-      <c r="E77" s="4" t="inlineStr"/>
-      <c r="F77" s="4" t="inlineStr">
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>https://www.britams.nl/</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>principal@britams.nl</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
         <is>
           <t>+31 (0) 20 67 97 8</t>
         </is>
       </c>
-      <c r="G77" s="4" t="inlineStr"/>
-      <c r="H77" s="4" t="inlineStr"/>
-      <c r="I77" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J77" s="4" t="inlineStr">
+      <c r="G77" s="2" t="inlineStr"/>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom CRM Solution for Winford Bilingual Primary School</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K77" s="4" t="inlineStr"/>
-      <c r="L77" s="4" t="inlineStr">
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:49</t>
+        </is>
+      </c>
+      <c r="L77" s="2" t="inlineStr">
         <is>
           <t>google_maps</t>
         </is>
       </c>
-      <c r="M77" s="4" t="inlineStr"/>
-      <c r="N77" s="4" t="inlineStr"/>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
@@ -4430,14 +4802,22 @@
           <t>real estate agencies Dubai</t>
         </is>
       </c>
-      <c r="D81" s="3" t="inlineStr"/>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>https://www.exclusive-links.com/?utm_source=localmaps&amp;utm_medium=gbp&amp;utm_campaign=Dubaimarina&amp;utm_term=listing</t>
+        </is>
+      </c>
       <c r="E81" s="3" t="inlineStr"/>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>Send to phone</t>
-        </is>
-      </c>
-      <c r="G81" s="3" t="inlineStr"/>
+          <t>+971 4 399 4937</t>
+        </is>
+      </c>
+      <c r="G81" s="3" t="inlineStr">
+        <is>
+          <t>Head Office</t>
+        </is>
+      </c>
       <c r="H81" s="3" t="inlineStr"/>
       <c r="I81" s="3" t="inlineStr">
         <is>
@@ -4474,14 +4854,22 @@
           <t>real estate agencies Dubai</t>
         </is>
       </c>
-      <c r="D82" s="3" t="inlineStr"/>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>https://www.exclusive-links.com/?utm_source=localmaps&amp;utm_medium=gbp&amp;utm_campaign=Dubaimarina&amp;utm_term=listing</t>
+        </is>
+      </c>
       <c r="E82" s="3" t="inlineStr"/>
       <c r="F82" s="3" t="inlineStr">
         <is>
-          <t>Send to phone</t>
-        </is>
-      </c>
-      <c r="G82" s="3" t="inlineStr"/>
+          <t>+971 4 399 4937</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>Head Office</t>
+        </is>
+      </c>
       <c r="H82" s="3" t="inlineStr"/>
       <c r="I82" s="3" t="inlineStr">
         <is>
@@ -4518,14 +4906,22 @@
           <t>real estate agencies Dubai</t>
         </is>
       </c>
-      <c r="D83" s="3" t="inlineStr"/>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>https://www.exclusive-links.com/?utm_source=localmaps&amp;utm_medium=gbp&amp;utm_campaign=Dubaimarina&amp;utm_term=listing</t>
+        </is>
+      </c>
       <c r="E83" s="3" t="inlineStr"/>
       <c r="F83" s="3" t="inlineStr">
         <is>
-          <t>Send to phone</t>
-        </is>
-      </c>
-      <c r="G83" s="3" t="inlineStr"/>
+          <t>+971 4 399 4937</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>Head Office</t>
+        </is>
+      </c>
       <c r="H83" s="3" t="inlineStr"/>
       <c r="I83" s="3" t="inlineStr">
         <is>
@@ -4562,14 +4958,22 @@
           <t>real estate agencies Dubai</t>
         </is>
       </c>
-      <c r="D84" s="3" t="inlineStr"/>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>https://www.exclusive-links.com/?utm_source=localmaps&amp;utm_medium=gbp&amp;utm_campaign=Dubaimarina&amp;utm_term=listing</t>
+        </is>
+      </c>
       <c r="E84" s="3" t="inlineStr"/>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>Send to phone</t>
-        </is>
-      </c>
-      <c r="G84" s="3" t="inlineStr"/>
+          <t>+971 4 399 4937</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>Head Office</t>
+        </is>
+      </c>
       <c r="H84" s="3" t="inlineStr"/>
       <c r="I84" s="3" t="inlineStr">
         <is>
@@ -4606,14 +5010,22 @@
           <t>real estate agencies Dubai</t>
         </is>
       </c>
-      <c r="D85" s="3" t="inlineStr"/>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>https://www.exclusive-links.com/?utm_source=localmaps&amp;utm_medium=gbp&amp;utm_campaign=Dubaimarina&amp;utm_term=listing</t>
+        </is>
+      </c>
       <c r="E85" s="3" t="inlineStr"/>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>Send to phone</t>
-        </is>
-      </c>
-      <c r="G85" s="3" t="inlineStr"/>
+          <t>+971 4 399 4937</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>Head Office</t>
+        </is>
+      </c>
       <c r="H85" s="3" t="inlineStr"/>
       <c r="I85" s="3" t="inlineStr">
         <is>
@@ -4650,14 +5062,22 @@
           <t>real estate agencies Dubai</t>
         </is>
       </c>
-      <c r="D86" s="3" t="inlineStr"/>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>https://www.exclusive-links.com/?utm_source=localmaps&amp;utm_medium=gbp&amp;utm_campaign=Dubaimarina&amp;utm_term=listing</t>
+        </is>
+      </c>
       <c r="E86" s="3" t="inlineStr"/>
       <c r="F86" s="3" t="inlineStr">
         <is>
-          <t>Send to phone</t>
-        </is>
-      </c>
-      <c r="G86" s="3" t="inlineStr"/>
+          <t>+971 4 399 4937</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>Head Office</t>
+        </is>
+      </c>
       <c r="H86" s="3" t="inlineStr"/>
       <c r="I86" s="3" t="inlineStr">
         <is>
@@ -4694,14 +5114,22 @@
           <t>real estate agencies Dubai</t>
         </is>
       </c>
-      <c r="D87" s="3" t="inlineStr"/>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>https://www.exclusive-links.com/?utm_source=localmaps&amp;utm_medium=gbp&amp;utm_campaign=Dubaimarina&amp;utm_term=listing</t>
+        </is>
+      </c>
       <c r="E87" s="3" t="inlineStr"/>
       <c r="F87" s="3" t="inlineStr">
         <is>
-          <t>Send to phone</t>
-        </is>
-      </c>
-      <c r="G87" s="3" t="inlineStr"/>
+          <t>+971 4 399 4937</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>Head Office</t>
+        </is>
+      </c>
       <c r="H87" s="3" t="inlineStr"/>
       <c r="I87" s="3" t="inlineStr">
         <is>
@@ -4738,14 +5166,22 @@
           <t>real estate agencies Dubai</t>
         </is>
       </c>
-      <c r="D88" s="3" t="inlineStr"/>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>https://www.exclusive-links.com/?utm_source=localmaps&amp;utm_medium=gbp&amp;utm_campaign=Dubaimarina&amp;utm_term=listing</t>
+        </is>
+      </c>
       <c r="E88" s="3" t="inlineStr"/>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>Send to phone</t>
-        </is>
-      </c>
-      <c r="G88" s="3" t="inlineStr"/>
+          <t>+971 4 399 4937</t>
+        </is>
+      </c>
+      <c r="G88" s="3" t="inlineStr">
+        <is>
+          <t>Head Office</t>
+        </is>
+      </c>
       <c r="H88" s="3" t="inlineStr"/>
       <c r="I88" s="3" t="inlineStr">
         <is>
@@ -5077,6 +5513,1416 @@
       </c>
       <c r="M95" s="3" t="inlineStr"/>
       <c r="N95" s="3" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>MEOCLINIC Berlin | Private Hospital &amp; Specialist Care</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>clinic</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>https://www.berlin-health-excellence.com/medical-facilities-berlin/meoclinic</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>health@visitBerlin.de</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>+49 (0) 30 - 2094</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>Prof. Dr</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom Hospital CRM/ERP Solution for MEOCLINIC Berlin</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 18:24</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 18:29</t>
+        </is>
+      </c>
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>google_search</t>
+        </is>
+      </c>
+      <c r="M96" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N96" s="2" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>Grand Canal Boutique Hotel | 4-Star Amsterdam Canal Stay</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>https://www.grandcanalhotelamsterdam.com/</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>info@amsterdamcanalhotels.com</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>+31 (0)20 787 07 4</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr"/>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>Proposal: Custom Hotel Management System for Grand Canal Boutique Hotel</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 18:43</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 18:45</t>
+        </is>
+      </c>
+      <c r="L97" s="2" t="inlineStr">
+        <is>
+          <t>google_search</t>
+        </is>
+      </c>
+      <c r="M97" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N97" s="2" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>The Dylan Amsterdam: Luxury 5 Star Boutique Hotel in ...</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>https://www.dylanamsterdam.com/</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr"/>
+      <c r="F98" s="3" t="inlineStr"/>
+      <c r="G98" s="3" t="inlineStr"/>
+      <c r="H98" s="3" t="inlineStr"/>
+      <c r="I98" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J98" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 18:50</t>
+        </is>
+      </c>
+      <c r="K98" s="3" t="inlineStr"/>
+      <c r="L98" s="3" t="inlineStr">
+        <is>
+          <t>google_search</t>
+        </is>
+      </c>
+      <c r="M98" s="3" t="inlineStr"/>
+      <c r="N98" s="3" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>The First Collection Business Bay, Dubai | Stylish Hotel ...</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>https://www.marriott.com/en-us/hotels/dxbtb-the-first-collection-business-bay-dubai-a-tribute-portfolio-hotel/overview/</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr"/>
+      <c r="F99" s="3" t="inlineStr"/>
+      <c r="G99" s="3" t="inlineStr"/>
+      <c r="H99" s="3" t="inlineStr"/>
+      <c r="I99" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J99" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 18:54</t>
+        </is>
+      </c>
+      <c r="K99" s="3" t="inlineStr"/>
+      <c r="L99" s="3" t="inlineStr">
+        <is>
+          <t>google_search</t>
+        </is>
+      </c>
+      <c r="M99" s="3" t="inlineStr"/>
+      <c r="N99" s="3" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>Grand Millennium Business Bay - Dubai Hotels</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>https://www.millenniumhotels.com/en/dubai/grand-millennium-business-bay/</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr"/>
+      <c r="F100" s="3" t="inlineStr">
+        <is>
+          <t>+971 4 545 2100</t>
+        </is>
+      </c>
+      <c r="G100" s="3" t="inlineStr"/>
+      <c r="H100" s="3" t="inlineStr"/>
+      <c r="I100" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J100" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 18:58</t>
+        </is>
+      </c>
+      <c r="K100" s="3" t="inlineStr"/>
+      <c r="L100" s="3" t="inlineStr">
+        <is>
+          <t>google_search</t>
+        </is>
+      </c>
+      <c r="M100" s="3" t="inlineStr"/>
+      <c r="N100" s="3" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>Gordon Ramsay Restaurants</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gordonramsayrestaurants.com/</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>guestrelations@gordonramsay.com</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr"/>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>Mr 
+ Mrs 
+ Miss</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>Custom Mobile App Solution for Enhancing Your Dining Experience</t>
+        </is>
+      </c>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 18:58</t>
+        </is>
+      </c>
+      <c r="K101" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:01</t>
+        </is>
+      </c>
+      <c r="L101" s="2" t="inlineStr">
+        <is>
+          <t>google_search</t>
+        </is>
+      </c>
+      <c r="M101" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N101" s="2" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>Dishoom | Indian Restaurants | From Bombay with Love</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>https://www.dishoom.com/</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr"/>
+      <c r="F102" s="3" t="inlineStr"/>
+      <c r="G102" s="3" t="inlineStr"/>
+      <c r="H102" s="3" t="inlineStr"/>
+      <c r="I102" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J102" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:02</t>
+        </is>
+      </c>
+      <c r="K102" s="3" t="inlineStr"/>
+      <c r="L102" s="3" t="inlineStr">
+        <is>
+          <t>google_search</t>
+        </is>
+      </c>
+      <c r="M102" s="3" t="inlineStr"/>
+      <c r="N102" s="3" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>Zizzi | Italian Restaurants in the UK and Ireland</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>https://www.zizzi.co.uk/</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>recruitment@zizzi.co.uk</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr"/>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>Head Office</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>Building Custom Mobile App for Zizzi Italian Restaurants</t>
+        </is>
+      </c>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:02</t>
+        </is>
+      </c>
+      <c r="K103" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:05</t>
+        </is>
+      </c>
+      <c r="L103" s="2" t="inlineStr">
+        <is>
+          <t>google_search</t>
+        </is>
+      </c>
+      <c r="M103" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N103" s="2" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>Carluccio's</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>https://www.carluccios.com/</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>orders@carluccios.com</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr"/>
+      <c r="G104" s="2" t="inlineStr"/>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>Build Custom Mobile-Friendly App for Carluccio's</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:06</t>
+        </is>
+      </c>
+      <c r="K104" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:09</t>
+        </is>
+      </c>
+      <c r="L104" s="2" t="inlineStr">
+        <is>
+          <t>google_search</t>
+        </is>
+      </c>
+      <c r="M104" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N104" s="2" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>DNA Health &amp; Wellness - Al Wasl</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>clinic</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>private clinics Dubai</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr"/>
+      <c r="E105" s="3" t="inlineStr"/>
+      <c r="F105" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G105" s="3" t="inlineStr"/>
+      <c r="H105" s="3" t="inlineStr"/>
+      <c r="I105" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J105" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:11</t>
+        </is>
+      </c>
+      <c r="K105" s="3" t="inlineStr"/>
+      <c r="L105" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M105" s="3" t="inlineStr"/>
+      <c r="N105" s="3" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>Trucare Plus Home Healthcare – Doctor at Home &amp; IV Drips Dubai</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>clinic</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>private clinics Dubai</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr"/>
+      <c r="E106" s="3" t="inlineStr"/>
+      <c r="F106" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G106" s="3" t="inlineStr"/>
+      <c r="H106" s="3" t="inlineStr"/>
+      <c r="I106" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J106" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:11</t>
+        </is>
+      </c>
+      <c r="K106" s="3" t="inlineStr"/>
+      <c r="L106" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M106" s="3" t="inlineStr"/>
+      <c r="N106" s="3" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>The Parlour at Bloomsbury</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>hotels London</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr"/>
+      <c r="E107" s="3" t="inlineStr"/>
+      <c r="F107" s="3" t="inlineStr"/>
+      <c r="G107" s="3" t="inlineStr"/>
+      <c r="H107" s="3" t="inlineStr"/>
+      <c r="I107" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J107" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:11</t>
+        </is>
+      </c>
+      <c r="K107" s="3" t="inlineStr"/>
+      <c r="L107" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M107" s="3" t="inlineStr"/>
+      <c r="N107" s="3" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>Crown &amp; Sceptre</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>hotels London</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>https://thezetter.com/bloomsbury/the-parlour/</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>press@thezetter.com</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>2025-05-30 10</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>Head Chef</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>Proposal: Custom Hotel Management System</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:11</t>
+        </is>
+      </c>
+      <c r="K108" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:13</t>
+        </is>
+      </c>
+      <c r="L108" s="2" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M108" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N108" s="2" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>International School of Amsterdam</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>school</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>schools Amsterdam</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>https://www.britams.nl/</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>principal@britams.nl</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>+31 (0) 20 67 97 8</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr"/>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>Proposal: Custom CRM Solution for ISA College Management</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:50</t>
+        </is>
+      </c>
+      <c r="K109" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:53</t>
+        </is>
+      </c>
+      <c r="L109" s="2" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M109" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N109" s="2" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>Baytify Real Estate Dubai | Global</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>real estate agencies Dubai</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr"/>
+      <c r="E110" s="3" t="inlineStr"/>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G110" s="3" t="inlineStr"/>
+      <c r="H110" s="3" t="inlineStr"/>
+      <c r="I110" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J110" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:53</t>
+        </is>
+      </c>
+      <c r="K110" s="3" t="inlineStr"/>
+      <c r="L110" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M110" s="3" t="inlineStr"/>
+      <c r="N110" s="3" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>Espace</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>real estate agencies Dubai</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr"/>
+      <c r="E111" s="3" t="inlineStr"/>
+      <c r="F111" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G111" s="3" t="inlineStr"/>
+      <c r="H111" s="3" t="inlineStr"/>
+      <c r="I111" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J111" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 19:54</t>
+        </is>
+      </c>
+      <c r="K111" s="3" t="inlineStr"/>
+      <c r="L111" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M111" s="3" t="inlineStr"/>
+      <c r="N111" s="3" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>فقيه مركز الخصوبة والتوليد - دبي</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>clinic</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>private clinics Dubai</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr"/>
+      <c r="E112" s="3" t="inlineStr"/>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G112" s="3" t="inlineStr"/>
+      <c r="H112" s="3" t="inlineStr"/>
+      <c r="I112" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J112" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:20</t>
+        </is>
+      </c>
+      <c r="K112" s="3" t="inlineStr"/>
+      <c r="L112" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M112" s="3" t="inlineStr"/>
+      <c r="N112" s="3" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
+        <is>
+          <t>Algebra Healthcare ( Polyclinic &amp; Home Health care center )</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>clinic</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>private clinics Dubai</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr"/>
+      <c r="E113" s="3" t="inlineStr"/>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="inlineStr"/>
+      <c r="H113" s="3" t="inlineStr"/>
+      <c r="I113" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J113" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:20</t>
+        </is>
+      </c>
+      <c r="K113" s="3" t="inlineStr"/>
+      <c r="L113" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M113" s="3" t="inlineStr"/>
+      <c r="N113" s="3" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="inlineStr">
+        <is>
+          <t>Mueller Medical Clinic FZ LLC – ENT, Sleep Apnea &amp; Psychology Specialist Center In Dubai</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>clinic</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>private clinics Dubai</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr"/>
+      <c r="E114" s="3" t="inlineStr"/>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="inlineStr"/>
+      <c r="H114" s="3" t="inlineStr"/>
+      <c r="I114" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J114" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:20</t>
+        </is>
+      </c>
+      <c r="K114" s="3" t="inlineStr"/>
+      <c r="L114" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M114" s="3" t="inlineStr"/>
+      <c r="N114" s="3" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="inlineStr">
+        <is>
+          <t>DoubleTree by Hilton London - Victoria</t>
+        </is>
+      </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr">
+        <is>
+          <t>hotels London</t>
+        </is>
+      </c>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>https://www.hilton.com/en/hotels/lonvcdi-doubletree-london-victoria/?SEO_id=GMB-EMEA-DI-LONVCDI</t>
+        </is>
+      </c>
+      <c r="E115" s="3" t="inlineStr"/>
+      <c r="F115" s="3" t="inlineStr">
+        <is>
+          <t>+44 20 7834 8123</t>
+        </is>
+      </c>
+      <c r="G115" s="3" t="inlineStr"/>
+      <c r="H115" s="3" t="inlineStr"/>
+      <c r="I115" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J115" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:20</t>
+        </is>
+      </c>
+      <c r="K115" s="3" t="inlineStr"/>
+      <c r="L115" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M115" s="3" t="inlineStr"/>
+      <c r="N115" s="3" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="3" t="inlineStr">
+        <is>
+          <t>Hilton London Angel Islington</t>
+        </is>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>hotels London</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>https://www.hilton.com/en/hotels/lonishn-hilton-london-angel-islington/?SEO_id=GMB-EMEA-HN-LONISHN</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="inlineStr"/>
+      <c r="F116" s="3" t="inlineStr">
+        <is>
+          <t>+44 20 7354 7700</t>
+        </is>
+      </c>
+      <c r="G116" s="3" t="inlineStr"/>
+      <c r="H116" s="3" t="inlineStr"/>
+      <c r="I116" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J116" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:23</t>
+        </is>
+      </c>
+      <c r="K116" s="3" t="inlineStr"/>
+      <c r="L116" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M116" s="3" t="inlineStr"/>
+      <c r="N116" s="3" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>Montessori Lyceum Amsterdam</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>school</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>schools Amsterdam</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>https://www.britams.nl/</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>principal@britams.nl</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>+31 (0) 20 67 97 8</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="inlineStr"/>
+      <c r="H117" s="2" t="inlineStr">
+        <is>
+          <t>Custom CRM Proposal for Montessori Lyceum Amsterdam</t>
+        </is>
+      </c>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J117" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:33</t>
+        </is>
+      </c>
+      <c r="K117" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:34</t>
+        </is>
+      </c>
+      <c r="L117" s="2" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M117" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N117" s="2" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>Next Level Real Estate - Award Winning Real Estate Agency in Dubai</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>real estate agencies Dubai</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>https://www.exclusive-links.com/?utm_source=localmaps&amp;utm_medium=gbp&amp;utm_campaign=Dubaimarina&amp;utm_term=listing</t>
+        </is>
+      </c>
+      <c r="E118" s="3" t="inlineStr"/>
+      <c r="F118" s="3" t="inlineStr">
+        <is>
+          <t>+971 4 399 4937</t>
+        </is>
+      </c>
+      <c r="G118" s="3" t="inlineStr">
+        <is>
+          <t>Head Office</t>
+        </is>
+      </c>
+      <c r="H118" s="3" t="inlineStr"/>
+      <c r="I118" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J118" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:38</t>
+        </is>
+      </c>
+      <c r="K118" s="3" t="inlineStr"/>
+      <c r="L118" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M118" s="3" t="inlineStr"/>
+      <c r="N118" s="3" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>Al Ayan Real Estate Broker LLC</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>real estate agencies Dubai</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>https://www.exclusive-links.com/?utm_source=localmaps&amp;utm_medium=gbp&amp;utm_campaign=Dubaimarina&amp;utm_term=listing</t>
+        </is>
+      </c>
+      <c r="E119" s="3" t="inlineStr"/>
+      <c r="F119" s="3" t="inlineStr">
+        <is>
+          <t>+971 4 399 4937</t>
+        </is>
+      </c>
+      <c r="G119" s="3" t="inlineStr">
+        <is>
+          <t>Head Office</t>
+        </is>
+      </c>
+      <c r="H119" s="3" t="inlineStr"/>
+      <c r="I119" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J119" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:39</t>
+        </is>
+      </c>
+      <c r="K119" s="3" t="inlineStr"/>
+      <c r="L119" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M119" s="3" t="inlineStr"/>
+      <c r="N119" s="3" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="inlineStr">
+        <is>
+          <t>Xperience​ Realty Real Estate</t>
+        </is>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>real estate agencies Dubai</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>https://www.exclusive-links.com/?utm_source=localmaps&amp;utm_medium=gbp&amp;utm_campaign=Dubaimarina&amp;utm_term=listing</t>
+        </is>
+      </c>
+      <c r="E120" s="3" t="inlineStr"/>
+      <c r="F120" s="3" t="inlineStr">
+        <is>
+          <t>+971 4 399 4937</t>
+        </is>
+      </c>
+      <c r="G120" s="3" t="inlineStr">
+        <is>
+          <t>Head Office</t>
+        </is>
+      </c>
+      <c r="H120" s="3" t="inlineStr"/>
+      <c r="I120" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J120" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:40</t>
+        </is>
+      </c>
+      <c r="K120" s="3" t="inlineStr"/>
+      <c r="L120" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M120" s="3" t="inlineStr"/>
+      <c r="N120" s="3" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>Boutique Hotel The Noblemen Amsterdam</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>https://hotelthenoblemen.com/</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>info@hotelthenoblemen.com</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>020 215 6131</t>
+        </is>
+      </c>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>Director Stef</t>
+        </is>
+      </c>
+      <c r="H121" s="2" t="inlineStr">
+        <is>
+          <t>Proposal: Custom Hotel Management System for The Noblemen Amsterdam</t>
+        </is>
+      </c>
+      <c r="I121" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J121" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:51</t>
+        </is>
+      </c>
+      <c r="K121" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:52</t>
+        </is>
+      </c>
+      <c r="L121" s="2" t="inlineStr">
+        <is>
+          <t>google_search</t>
+        </is>
+      </c>
+      <c r="M121" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N121" s="2" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="4" t="inlineStr">
+        <is>
+          <t>Welcome to The Restaurant Group - The Restaurant Group ltd</t>
+        </is>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="C122" s="4" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>https://trggroupltd.com/</t>
+        </is>
+      </c>
+      <c r="E122" s="4" t="inlineStr"/>
+      <c r="F122" s="4" t="inlineStr"/>
+      <c r="G122" s="4" t="inlineStr"/>
+      <c r="H122" s="4" t="inlineStr"/>
+      <c r="I122" s="4" t="inlineStr">
+        <is>
+          <t>found</t>
+        </is>
+      </c>
+      <c r="J122" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:55</t>
+        </is>
+      </c>
+      <c r="K122" s="4" t="inlineStr"/>
+      <c r="L122" s="4" t="inlineStr">
+        <is>
+          <t>google_search</t>
+        </is>
+      </c>
+      <c r="M122" s="4" t="inlineStr"/>
+      <c r="N122" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Refactor pitch and email template for improved clarity and focus on client needs; updated profile details and industry-specific pain points, solutions, and CTAs.
</commit_message>
<xml_diff>
--- a/job_hunter_agent/data/clients.xlsx
+++ b/job_hunter_agent/data/clients.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N122"/>
+  <dimension ref="A1:N138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2447,60 +2447,72 @@
       <c r="N35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Citymax Hotel Business Bay | 4 star Hotel Dubai</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>hotel</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Dubai</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>https://www.citymaxhotels.com/uae/dubai/citymax-hotels-business-bay/</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>reservations@citymaxhotels.com</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>14774221887</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>Mr. Manmeet</t>
         </is>
       </c>
-      <c r="H36" s="4" t="inlineStr"/>
-      <c r="I36" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J36" s="4" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Proposal: Custom Hotel Management System for Citymax Business Bay</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:20</t>
         </is>
       </c>
-      <c r="K36" s="4" t="inlineStr"/>
-      <c r="L36" s="4" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:49</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
         <is>
           <t>google_search</t>
         </is>
       </c>
-      <c r="M36" s="4" t="inlineStr"/>
-      <c r="N36" s="4" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -4655,48 +4667,68 @@
       <c r="N77" s="2" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="4" t="inlineStr">
+      <c r="A78" s="2" t="inlineStr">
         <is>
           <t>Public Elementary School De Witte Olifant</t>
         </is>
       </c>
-      <c r="B78" s="4" t="inlineStr">
+      <c r="B78" s="2" t="inlineStr">
         <is>
           <t>school</t>
         </is>
       </c>
-      <c r="C78" s="4" t="inlineStr">
+      <c r="C78" s="2" t="inlineStr">
         <is>
           <t>schools Amsterdam</t>
         </is>
       </c>
-      <c r="D78" s="4" t="inlineStr"/>
-      <c r="E78" s="4" t="inlineStr"/>
-      <c r="F78" s="4" t="inlineStr">
-        <is>
-          <t>+31 (0) 20 67 97 8</t>
-        </is>
-      </c>
-      <c r="G78" s="4" t="inlineStr"/>
-      <c r="H78" s="4" t="inlineStr"/>
-      <c r="I78" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J78" s="4" t="inlineStr">
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>http://www.amityschool.nl/</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>ENQUIRIES@AMITYAMSTERDAM.NL</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>204   1182</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr"/>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>Custom College CRM Proposal: De Witte Olifant</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 13:25</t>
         </is>
       </c>
-      <c r="K78" s="4" t="inlineStr"/>
-      <c r="L78" s="4" t="inlineStr">
-        <is>
-          <t>google_maps</t>
-        </is>
-      </c>
-      <c r="M78" s="4" t="inlineStr"/>
-      <c r="N78" s="4" t="inlineStr"/>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:30</t>
+        </is>
+      </c>
+      <c r="L78" s="2" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
@@ -6881,48 +6913,889 @@
       <c r="N121" s="2" t="inlineStr"/>
     </row>
     <row r="122">
-      <c r="A122" s="4" t="inlineStr">
+      <c r="A122" s="2" t="inlineStr">
         <is>
           <t>Welcome to The Restaurant Group - The Restaurant Group ltd</t>
         </is>
       </c>
-      <c r="B122" s="4" t="inlineStr">
+      <c r="B122" s="2" t="inlineStr">
         <is>
           <t>restaurant</t>
         </is>
       </c>
-      <c r="C122" s="4" t="inlineStr">
+      <c r="C122" s="2" t="inlineStr">
         <is>
           <t>London</t>
         </is>
       </c>
-      <c r="D122" s="4" t="inlineStr">
+      <c r="D122" s="2" t="inlineStr">
         <is>
           <t>https://trggroupltd.com/</t>
         </is>
       </c>
-      <c r="E122" s="4" t="inlineStr"/>
-      <c r="F122" s="4" t="inlineStr"/>
-      <c r="G122" s="4" t="inlineStr"/>
-      <c r="H122" s="4" t="inlineStr"/>
-      <c r="I122" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J122" s="4" t="inlineStr">
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>supplierinfo@trggroupltd.com</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>0203 117 5001</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>Head Office 
+ Address</t>
+        </is>
+      </c>
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>Build Your Custom Mobile Restaurant App</t>
+        </is>
+      </c>
+      <c r="I122" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J122" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 20:55</t>
         </is>
       </c>
-      <c r="K122" s="4" t="inlineStr"/>
-      <c r="L122" s="4" t="inlineStr">
+      <c r="K122" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:56</t>
+        </is>
+      </c>
+      <c r="L122" s="2" t="inlineStr">
         <is>
           <t>google_search</t>
         </is>
       </c>
-      <c r="M122" s="4" t="inlineStr"/>
-      <c r="N122" s="4" t="inlineStr"/>
+      <c r="M122" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N122" s="2" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="inlineStr">
+        <is>
+          <t>Queens Medical Center Al Satwa</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>clinic</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr">
+        <is>
+          <t>private clinics Dubai</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="inlineStr"/>
+      <c r="E123" s="3" t="inlineStr"/>
+      <c r="F123" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G123" s="3" t="inlineStr"/>
+      <c r="H123" s="3" t="inlineStr"/>
+      <c r="I123" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J123" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 20:59</t>
+        </is>
+      </c>
+      <c r="K123" s="3" t="inlineStr"/>
+      <c r="L123" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M123" s="3" t="inlineStr"/>
+      <c r="N123" s="3" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
+          <t>Travelodge London Central City Road</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>hotels London</t>
+        </is>
+      </c>
+      <c r="D124" s="3" t="inlineStr">
+        <is>
+          <t>https://www.travelodge.co.uk/hotels/340/London-Central-City-Road-hotel?utm_source=google&amp;utm_medium=GHA_Organic&amp;utm_campaign=GHA_London%20Central%20City%20Road</t>
+        </is>
+      </c>
+      <c r="E124" s="3" t="inlineStr"/>
+      <c r="F124" s="3" t="inlineStr">
+        <is>
+          <t>08719 846333</t>
+        </is>
+      </c>
+      <c r="G124" s="3" t="inlineStr"/>
+      <c r="H124" s="3" t="inlineStr"/>
+      <c r="I124" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J124" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:00</t>
+        </is>
+      </c>
+      <c r="K124" s="3" t="inlineStr"/>
+      <c r="L124" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M124" s="3" t="inlineStr"/>
+      <c r="N124" s="3" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="3" t="inlineStr">
+        <is>
+          <t>Travelodge London City</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>hotels London</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="inlineStr">
+        <is>
+          <t>https://www.travelodge.co.uk/hotels/639/London-City?utm_source=google&amp;utm_medium=GHA_Organic&amp;utm_campaign=GHA_London%20City</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="inlineStr"/>
+      <c r="F125" s="3" t="inlineStr">
+        <is>
+          <t>08719 846534</t>
+        </is>
+      </c>
+      <c r="G125" s="3" t="inlineStr"/>
+      <c r="H125" s="3" t="inlineStr"/>
+      <c r="I125" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J125" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:01</t>
+        </is>
+      </c>
+      <c r="K125" s="3" t="inlineStr"/>
+      <c r="L125" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M125" s="3" t="inlineStr"/>
+      <c r="N125" s="3" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="inlineStr">
+        <is>
+          <t>Terra Nova</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>real estate agencies Dubai</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="inlineStr"/>
+      <c r="E126" s="3" t="inlineStr"/>
+      <c r="F126" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G126" s="3" t="inlineStr"/>
+      <c r="H126" s="3" t="inlineStr"/>
+      <c r="I126" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J126" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:01</t>
+        </is>
+      </c>
+      <c r="K126" s="3" t="inlineStr"/>
+      <c r="L126" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M126" s="3" t="inlineStr"/>
+      <c r="N126" s="3" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>Best Hospital in Dubai | Top-Rated Hospital in Dubai-King's</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>https://kingscollegehospitaldubai.com/</t>
+        </is>
+      </c>
+      <c r="E127" s="3" t="inlineStr"/>
+      <c r="F127" s="3" t="inlineStr"/>
+      <c r="G127" s="3" t="inlineStr"/>
+      <c r="H127" s="3" t="inlineStr"/>
+      <c r="I127" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J127" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:09</t>
+        </is>
+      </c>
+      <c r="K127" s="3" t="inlineStr"/>
+      <c r="L127" s="3" t="inlineStr">
+        <is>
+          <t>google_search</t>
+        </is>
+      </c>
+      <c r="M127" s="3" t="inlineStr"/>
+      <c r="N127" s="3" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Helios International — Official Helios Website for International ...</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>clinic</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>https://www.helios-international.com/</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>info@helios-international.com</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>+49 30 6832 3885</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Horst Schmidt</t>
+        </is>
+      </c>
+      <c r="H128" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom Clinic Management Web App Solution</t>
+        </is>
+      </c>
+      <c r="I128" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J128" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:11</t>
+        </is>
+      </c>
+      <c r="K128" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:12</t>
+        </is>
+      </c>
+      <c r="L128" s="2" t="inlineStr">
+        <is>
+          <t>google_search</t>
+        </is>
+      </c>
+      <c r="M128" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N128" s="2" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="3" t="inlineStr">
+        <is>
+          <t>Go Dental Clinic, Bur Dubai</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>clinic</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>private clinics Dubai</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr"/>
+      <c r="E129" s="3" t="inlineStr"/>
+      <c r="F129" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G129" s="3" t="inlineStr"/>
+      <c r="H129" s="3" t="inlineStr"/>
+      <c r="I129" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J129" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:21</t>
+        </is>
+      </c>
+      <c r="K129" s="3" t="inlineStr"/>
+      <c r="L129" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M129" s="3" t="inlineStr"/>
+      <c r="N129" s="3" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
+          <t>Ember Locke Kensington</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>hotels London</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>https://www.lockeliving.com/en/london/ember-locke</t>
+        </is>
+      </c>
+      <c r="E130" s="3" t="inlineStr"/>
+      <c r="F130" s="3" t="inlineStr">
+        <is>
+          <t>+44 20 7052 7175</t>
+        </is>
+      </c>
+      <c r="G130" s="3" t="inlineStr"/>
+      <c r="H130" s="3" t="inlineStr"/>
+      <c r="I130" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J130" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:21</t>
+        </is>
+      </c>
+      <c r="K130" s="3" t="inlineStr"/>
+      <c r="L130" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M130" s="3" t="inlineStr"/>
+      <c r="N130" s="3" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>The Chesterfield Mayfair</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>hotels London</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>https://www.chesterfieldmayfair.com/?utm_source=google&amp;utm_medium=local&amp;utm_campaign=hotel-the-chesterfield-mayfair</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>alake@chesterfieldmayfair.com</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>+44 20 7491 2622</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>Manager Adam Lake</t>
+        </is>
+      </c>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom Hotel Management System</t>
+        </is>
+      </c>
+      <c r="I131" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J131" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:21</t>
+        </is>
+      </c>
+      <c r="K131" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:23</t>
+        </is>
+      </c>
+      <c r="L131" s="2" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M131" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N131" s="2" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>The Tower Hotel, by Thistle</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>hotel</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>hotels London</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>http://www.publove.co.uk/</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>reservations@publove.co.uk</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>+44 20 7928 0720</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>Head Clerkenwell  View</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>Proposal: Custom Hotel Management System</t>
+        </is>
+      </c>
+      <c r="I132" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J132" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:27</t>
+        </is>
+      </c>
+      <c r="K132" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:28</t>
+        </is>
+      </c>
+      <c r="L132" s="2" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M132" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N132" s="2" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>KAYE &amp; CO REAL ESTATE L.L.C.</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>business</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>real estate agencies Dubai</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="inlineStr">
+        <is>
+          <t>https://www.exclusive-links.com/?utm_source=localmaps&amp;utm_medium=gbp&amp;utm_campaign=Dubai&amp;utm_term=listing</t>
+        </is>
+      </c>
+      <c r="E133" s="3" t="inlineStr"/>
+      <c r="F133" s="3" t="inlineStr">
+        <is>
+          <t>+971 4 399 4937</t>
+        </is>
+      </c>
+      <c r="G133" s="3" t="inlineStr">
+        <is>
+          <t>Head Office</t>
+        </is>
+      </c>
+      <c r="H133" s="3" t="inlineStr"/>
+      <c r="I133" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J133" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:33</t>
+        </is>
+      </c>
+      <c r="K133" s="3" t="inlineStr"/>
+      <c r="L133" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M133" s="3" t="inlineStr"/>
+      <c r="N133" s="3" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>King Edward VII's Hospital | Premier Private Hospital</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kingedwardvii.co.uk/</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>enquiries@kingedwardvii.co.uk</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>020 7467 3221</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr"/>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
+          <t>Custom CRM/ERP Proposal for King Edward VII's Hospital</t>
+        </is>
+      </c>
+      <c r="I134" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J134" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:42</t>
+        </is>
+      </c>
+      <c r="K134" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:44</t>
+        </is>
+      </c>
+      <c r="L134" s="2" t="inlineStr">
+        <is>
+          <t>google_search</t>
+        </is>
+      </c>
+      <c r="M134" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N134" s="2" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="3" t="inlineStr">
+        <is>
+          <t>Contact Us - Dental Clinic Toronto</t>
+        </is>
+      </c>
+      <c r="B135" s="3" t="inlineStr">
+        <is>
+          <t>clinic</t>
+        </is>
+      </c>
+      <c r="C135" s="3" t="inlineStr">
+        <is>
+          <t>Toronto</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="inlineStr">
+        <is>
+          <t>https://dentalclinictoronto.dentist/contact-us/</t>
+        </is>
+      </c>
+      <c r="E135" s="3" t="inlineStr"/>
+      <c r="F135" s="3" t="inlineStr"/>
+      <c r="G135" s="3" t="inlineStr"/>
+      <c r="H135" s="3" t="inlineStr"/>
+      <c r="I135" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J135" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:45</t>
+        </is>
+      </c>
+      <c r="K135" s="3" t="inlineStr"/>
+      <c r="L135" s="3" t="inlineStr">
+        <is>
+          <t>google_search</t>
+        </is>
+      </c>
+      <c r="M135" s="3" t="inlineStr"/>
+      <c r="N135" s="3" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="3" t="inlineStr">
+        <is>
+          <t>Bill's Restaurants | All Day Dining | Famous Burgers</t>
+        </is>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="inlineStr">
+        <is>
+          <t>https://bills-website.co.uk/</t>
+        </is>
+      </c>
+      <c r="E136" s="3" t="inlineStr"/>
+      <c r="F136" s="3" t="inlineStr"/>
+      <c r="G136" s="3" t="inlineStr"/>
+      <c r="H136" s="3" t="inlineStr"/>
+      <c r="I136" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J136" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:51</t>
+        </is>
+      </c>
+      <c r="K136" s="3" t="inlineStr"/>
+      <c r="L136" s="3" t="inlineStr">
+        <is>
+          <t>google_search</t>
+        </is>
+      </c>
+      <c r="M136" s="3" t="inlineStr"/>
+      <c r="N136" s="3" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Joy Dental Clinic, Jumeirah Al Wasl Road</t>
+        </is>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>clinic</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>private clinics Dubai</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="inlineStr"/>
+      <c r="E137" s="3" t="inlineStr"/>
+      <c r="F137" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G137" s="3" t="inlineStr"/>
+      <c r="H137" s="3" t="inlineStr"/>
+      <c r="I137" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J137" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:54</t>
+        </is>
+      </c>
+      <c r="K137" s="3" t="inlineStr"/>
+      <c r="L137" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M137" s="3" t="inlineStr"/>
+      <c r="N137" s="3" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="3" t="inlineStr">
+        <is>
+          <t>Oral Implantology Medical Center</t>
+        </is>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>clinic</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>private clinics Dubai</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="inlineStr"/>
+      <c r="E138" s="3" t="inlineStr"/>
+      <c r="F138" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G138" s="3" t="inlineStr"/>
+      <c r="H138" s="3" t="inlineStr"/>
+      <c r="I138" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J138" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 21:54</t>
+        </is>
+      </c>
+      <c r="K138" s="3" t="inlineStr"/>
+      <c r="L138" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M138" s="3" t="inlineStr"/>
+      <c r="N138" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: Add new client entry for Dentons and update status in clients data
</commit_message>
<xml_diff>
--- a/job_hunter_agent/data/clients.xlsx
+++ b/job_hunter_agent/data/clients.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N150"/>
+  <dimension ref="A1:N151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -8430,48 +8430,92 @@
       <c r="N149" s="3" t="inlineStr"/>
     </row>
     <row r="150">
-      <c r="A150" s="4" t="inlineStr">
+      <c r="A150" s="3" t="inlineStr">
         <is>
           <t>Amity University – Leading Private University in India | World ...</t>
         </is>
       </c>
-      <c r="B150" s="4" t="inlineStr">
+      <c r="B150" s="3" t="inlineStr">
         <is>
           <t>hospital</t>
         </is>
       </c>
-      <c r="C150" s="4" t="inlineStr">
+      <c r="C150" s="3" t="inlineStr">
         <is>
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="D150" s="4" t="inlineStr">
+      <c r="D150" s="3" t="inlineStr">
         <is>
           <t>https://www.amity.edu/</t>
         </is>
       </c>
-      <c r="E150" s="4" t="inlineStr"/>
-      <c r="F150" s="4" t="inlineStr"/>
-      <c r="G150" s="4" t="inlineStr"/>
-      <c r="H150" s="4" t="inlineStr"/>
-      <c r="I150" s="4" t="inlineStr">
+      <c r="E150" s="3" t="inlineStr"/>
+      <c r="F150" s="3" t="inlineStr"/>
+      <c r="G150" s="3" t="inlineStr"/>
+      <c r="H150" s="3" t="inlineStr"/>
+      <c r="I150" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J150" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 23:03</t>
+        </is>
+      </c>
+      <c r="K150" s="3" t="inlineStr"/>
+      <c r="L150" s="3" t="inlineStr">
+        <is>
+          <t>google_p4</t>
+        </is>
+      </c>
+      <c r="M150" s="3" t="inlineStr"/>
+      <c r="N150" s="3" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="4" t="inlineStr">
+        <is>
+          <t>Dentons advises on US$300 million PPP hospital project in ...</t>
+        </is>
+      </c>
+      <c r="B151" s="4" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C151" s="4" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D151" s="4" t="inlineStr">
+        <is>
+          <t>https://www.dentons.com/en/about-dentons/news-events-and-awards/news/2026/april/dentons-advises-on-us-300-million-ppp-hospital-project-in-uzbekistan</t>
+        </is>
+      </c>
+      <c r="E151" s="4" t="inlineStr"/>
+      <c r="F151" s="4" t="inlineStr"/>
+      <c r="G151" s="4" t="inlineStr"/>
+      <c r="H151" s="4" t="inlineStr"/>
+      <c r="I151" s="4" t="inlineStr">
         <is>
           <t>found</t>
         </is>
       </c>
-      <c r="J150" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-07 23:03</t>
-        </is>
-      </c>
-      <c r="K150" s="4" t="inlineStr"/>
-      <c r="L150" s="4" t="inlineStr">
+      <c r="J151" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-07 23:04</t>
+        </is>
+      </c>
+      <c r="K151" s="4" t="inlineStr"/>
+      <c r="L151" s="4" t="inlineStr">
         <is>
           <t>google_p4</t>
         </is>
       </c>
-      <c r="M150" s="4" t="inlineStr"/>
-      <c r="N150" s="4" t="inlineStr"/>
+      <c r="M151" s="4" t="inlineStr"/>
+      <c r="N151" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Enhance job_hunter_agent functionality: - Update autorun.log and client_hunter.log to log email interactions with hospitals. - Modify clients.json to reflect email statuses and add new hospital entries. - Sync all data to Supabase, including leads and clients, with improved error handling. - Implement reply checking from Gmail to update client statuses and notes. - Add follow-up candidate retrieval for leads needing follow-up.
</commit_message>
<xml_diff>
--- a/job_hunter_agent/data/clients.xlsx
+++ b/job_hunter_agent/data/clients.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -57,6 +57,11 @@
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CCE5FF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -70,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -82,6 +87,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -449,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N151"/>
+  <dimension ref="A1:N163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -7994,72 +8002,76 @@
       <c r="N141" s="2" t="inlineStr"/>
     </row>
     <row r="142">
-      <c r="A142" s="2" t="inlineStr">
+      <c r="A142" s="5" t="inlineStr">
         <is>
           <t>Netherlands: list of medical facilities</t>
         </is>
       </c>
-      <c r="B142" s="2" t="inlineStr">
+      <c r="B142" s="5" t="inlineStr">
         <is>
           <t>hospital</t>
         </is>
       </c>
-      <c r="C142" s="2" t="inlineStr">
+      <c r="C142" s="5" t="inlineStr">
         <is>
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="D142" s="2" t="inlineStr">
+      <c r="D142" s="5" t="inlineStr">
         <is>
           <t>https://www.gov.uk/government/publications/the-netherlands-list-of-medical-facilitiespractitioners/netherlands-list-of-medical-facilities</t>
         </is>
       </c>
-      <c r="E142" s="2" t="inlineStr">
+      <c r="E142" s="5" t="inlineStr">
         <is>
           <t>ukinnl@fcdo.gov.uk</t>
         </is>
       </c>
-      <c r="F142" s="2" t="inlineStr">
+      <c r="F142" s="5" t="inlineStr">
         <is>
           <t>0031 (0) 20 566 9</t>
         </is>
       </c>
-      <c r="G142" s="2" t="inlineStr">
+      <c r="G142" s="5" t="inlineStr">
         <is>
           <t>Dr. Molewaterplein</t>
         </is>
       </c>
-      <c r="H142" s="2" t="inlineStr">
+      <c r="H142" s="5" t="inlineStr">
         <is>
           <t>Revolutionize Your Medical Facility Operations</t>
         </is>
       </c>
-      <c r="I142" s="2" t="inlineStr">
-        <is>
-          <t>email_sent</t>
-        </is>
-      </c>
-      <c r="J142" s="2" t="inlineStr">
+      <c r="I142" s="5" t="inlineStr">
+        <is>
+          <t>replied</t>
+        </is>
+      </c>
+      <c r="J142" s="5" t="inlineStr">
         <is>
           <t>2026-05-07 22:53</t>
         </is>
       </c>
-      <c r="K142" s="2" t="inlineStr">
+      <c r="K142" s="5" t="inlineStr">
         <is>
           <t>2026-05-07T22:55:44.804660</t>
         </is>
       </c>
-      <c r="L142" s="2" t="inlineStr">
+      <c r="L142" s="5" t="inlineStr">
         <is>
           <t>google_p2</t>
         </is>
       </c>
-      <c r="M142" s="2" t="inlineStr">
+      <c r="M142" s="5" t="inlineStr">
         <is>
           <t>True</t>
         </is>
       </c>
-      <c r="N142" s="2" t="inlineStr"/>
+      <c r="N142" s="5" t="inlineStr">
+        <is>
+          <t>Reply received 2026-05-07</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
@@ -8474,48 +8486,700 @@
       <c r="N150" s="3" t="inlineStr"/>
     </row>
     <row r="151">
-      <c r="A151" s="4" t="inlineStr">
+      <c r="A151" s="2" t="inlineStr">
         <is>
           <t>Dentons advises on US$300 million PPP hospital project in ...</t>
         </is>
       </c>
-      <c r="B151" s="4" t="inlineStr">
+      <c r="B151" s="2" t="inlineStr">
         <is>
           <t>hospital</t>
         </is>
       </c>
-      <c r="C151" s="4" t="inlineStr">
+      <c r="C151" s="2" t="inlineStr">
         <is>
           <t>Amsterdam</t>
         </is>
       </c>
-      <c r="D151" s="4" t="inlineStr">
+      <c r="D151" s="2" t="inlineStr">
         <is>
           <t>https://www.dentons.com/en/about-dentons/news-events-and-awards/news/2026/april/dentons-advises-on-us-300-million-ppp-hospital-project-in-uzbekistan</t>
         </is>
       </c>
-      <c r="E151" s="4" t="inlineStr"/>
-      <c r="F151" s="4" t="inlineStr"/>
-      <c r="G151" s="4" t="inlineStr"/>
-      <c r="H151" s="4" t="inlineStr"/>
-      <c r="I151" s="4" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="J151" s="4" t="inlineStr">
+      <c r="E151" s="2" t="inlineStr">
+        <is>
+          <t>amanda.lowe@dentons.com</t>
+        </is>
+      </c>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>9 9   8 7 8   1 5</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr"/>
+      <c r="H151" s="2" t="inlineStr">
+        <is>
+          <t>Streamline PPP Hospital Operations: Custom Digital Solution Proposal</t>
+        </is>
+      </c>
+      <c r="I151" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J151" s="2" t="inlineStr">
         <is>
           <t>2026-05-07 23:04</t>
         </is>
       </c>
-      <c r="K151" s="4" t="inlineStr"/>
-      <c r="L151" s="4" t="inlineStr">
+      <c r="K151" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07T23:06:16.924998</t>
+        </is>
+      </c>
+      <c r="L151" s="2" t="inlineStr">
         <is>
           <t>google_p4</t>
         </is>
       </c>
-      <c r="M151" s="4" t="inlineStr"/>
-      <c r="N151" s="4" t="inlineStr"/>
+      <c r="M151" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N151" s="2" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t>Equans : a world leader in energy and services</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="inlineStr">
+        <is>
+          <t>https://www.equans.com/</t>
+        </is>
+      </c>
+      <c r="E152" s="3" t="inlineStr"/>
+      <c r="F152" s="3" t="inlineStr"/>
+      <c r="G152" s="3" t="inlineStr"/>
+      <c r="H152" s="3" t="inlineStr"/>
+      <c r="I152" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J152" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 23:07</t>
+        </is>
+      </c>
+      <c r="K152" s="3" t="inlineStr"/>
+      <c r="L152" s="3" t="inlineStr">
+        <is>
+          <t>google_p4</t>
+        </is>
+      </c>
+      <c r="M152" s="3" t="inlineStr"/>
+      <c r="N152" s="3" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="3" t="inlineStr">
+        <is>
+          <t>Global management consulting | McKinsey &amp; Company</t>
+        </is>
+      </c>
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D153" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mckinsey.com/</t>
+        </is>
+      </c>
+      <c r="E153" s="3" t="inlineStr"/>
+      <c r="F153" s="3" t="inlineStr"/>
+      <c r="G153" s="3" t="inlineStr"/>
+      <c r="H153" s="3" t="inlineStr"/>
+      <c r="I153" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J153" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 23:07</t>
+        </is>
+      </c>
+      <c r="K153" s="3" t="inlineStr"/>
+      <c r="L153" s="3" t="inlineStr">
+        <is>
+          <t>google_p4</t>
+        </is>
+      </c>
+      <c r="M153" s="3" t="inlineStr"/>
+      <c r="N153" s="3" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>Burjeel Hospital</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>https://burjeel.com/</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>%20dataprotectionofficer@burjeelholdings.com</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr"/>
+      <c r="G154" s="2" t="inlineStr"/>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
+          <t>Streamline Operations: Custom Digital Solution Proposal</t>
+        </is>
+      </c>
+      <c r="I154" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J154" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 23:11</t>
+        </is>
+      </c>
+      <c r="K154" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07T23:13:35.978141</t>
+        </is>
+      </c>
+      <c r="L154" s="2" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M154" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N154" s="2" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="3" t="inlineStr">
+        <is>
+          <t>HMS Al Garhoud Hospital: Best hospitals in Dubai - Top Rated ...</t>
+        </is>
+      </c>
+      <c r="B155" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="D155" s="3" t="inlineStr">
+        <is>
+          <t>https://www.gph.ae/</t>
+        </is>
+      </c>
+      <c r="E155" s="3" t="inlineStr"/>
+      <c r="F155" s="3" t="inlineStr"/>
+      <c r="G155" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Ahmed Ghanem</t>
+        </is>
+      </c>
+      <c r="H155" s="3" t="inlineStr"/>
+      <c r="I155" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J155" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 23:14</t>
+        </is>
+      </c>
+      <c r="K155" s="3" t="inlineStr"/>
+      <c r="L155" s="3" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M155" s="3" t="inlineStr"/>
+      <c r="N155" s="3" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>Canadian Specialist Hospital | The Best Hospital in Dubai</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>https://csh.ae/</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>info@csh.ae</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>+97147072222</t>
+        </is>
+      </c>
+      <c r="G156" s="2" t="inlineStr"/>
+      <c r="H156" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom Digital Solution for Optimizing Operations at Canadian Specialist Hospital</t>
+        </is>
+      </c>
+      <c r="I156" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J156" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 23:14</t>
+        </is>
+      </c>
+      <c r="K156" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07T23:16:32.158477</t>
+        </is>
+      </c>
+      <c r="L156" s="2" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M156" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N156" s="2" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="3" t="inlineStr">
+        <is>
+          <t>Dubai London Clinics &amp; Hospitals</t>
+        </is>
+      </c>
+      <c r="B157" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="D157" s="3" t="inlineStr">
+        <is>
+          <t>https://dubailondonhospital.com/</t>
+        </is>
+      </c>
+      <c r="E157" s="3" t="inlineStr"/>
+      <c r="F157" s="3" t="inlineStr"/>
+      <c r="G157" s="3" t="inlineStr"/>
+      <c r="H157" s="3" t="inlineStr"/>
+      <c r="I157" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J157" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 23:17</t>
+        </is>
+      </c>
+      <c r="K157" s="3" t="inlineStr"/>
+      <c r="L157" s="3" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M157" s="3" t="inlineStr"/>
+      <c r="N157" s="3" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>Medcare Appointment Booking - Dubai</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="inlineStr">
+        <is>
+          <t>https://www.medcare.ae/en/appointments.html</t>
+        </is>
+      </c>
+      <c r="E158" s="3" t="inlineStr"/>
+      <c r="F158" s="3" t="inlineStr">
+        <is>
+          <t>800 633 2273</t>
+        </is>
+      </c>
+      <c r="G158" s="3" t="inlineStr">
+        <is>
+          <t>Dr Saeed Al</t>
+        </is>
+      </c>
+      <c r="H158" s="3" t="inlineStr"/>
+      <c r="I158" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J158" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 23:17</t>
+        </is>
+      </c>
+      <c r="K158" s="3" t="inlineStr"/>
+      <c r="L158" s="3" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M158" s="3" t="inlineStr"/>
+      <c r="N158" s="3" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="3" t="inlineStr">
+        <is>
+          <t>1 Private Hospital in Dubai</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="inlineStr">
+        <is>
+          <t>https://saudigerman.com/dubai/</t>
+        </is>
+      </c>
+      <c r="E159" s="3" t="inlineStr"/>
+      <c r="F159" s="3" t="inlineStr">
+        <is>
+          <t>+971 4389 0002</t>
+        </is>
+      </c>
+      <c r="G159" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Bushra</t>
+        </is>
+      </c>
+      <c r="H159" s="3" t="inlineStr"/>
+      <c r="I159" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J159" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 23:17</t>
+        </is>
+      </c>
+      <c r="K159" s="3" t="inlineStr"/>
+      <c r="L159" s="3" t="inlineStr">
+        <is>
+          <t>google_p3</t>
+        </is>
+      </c>
+      <c r="M159" s="3" t="inlineStr"/>
+      <c r="N159" s="3" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="3" t="inlineStr">
+        <is>
+          <t>NMC Hospitals and Clinics – A Leading Healthcare Provider ...</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="D160" s="3" t="inlineStr">
+        <is>
+          <t>https://nmc.ae/en</t>
+        </is>
+      </c>
+      <c r="E160" s="3" t="inlineStr"/>
+      <c r="F160" s="3" t="inlineStr">
+        <is>
+          <t>30-04-2026</t>
+        </is>
+      </c>
+      <c r="G160" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Tatyana Avsyanskaya</t>
+        </is>
+      </c>
+      <c r="H160" s="3" t="inlineStr"/>
+      <c r="I160" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J160" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 23:18</t>
+        </is>
+      </c>
+      <c r="K160" s="3" t="inlineStr"/>
+      <c r="L160" s="3" t="inlineStr">
+        <is>
+          <t>google_p3</t>
+        </is>
+      </c>
+      <c r="M160" s="3" t="inlineStr"/>
+      <c r="N160" s="3" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>Best Hospital in Dubai | Top Healthcare in UAE</t>
+        </is>
+      </c>
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>https://www.hmsmirdifhospital.ae/en/</t>
+        </is>
+      </c>
+      <c r="E161" s="2" t="inlineStr">
+        <is>
+          <t>info_mph@hmsco.ae</t>
+        </is>
+      </c>
+      <c r="F161" s="2" t="inlineStr"/>
+      <c r="G161" s="2" t="inlineStr"/>
+      <c r="H161" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom Digital Solution for Optimized Operations</t>
+        </is>
+      </c>
+      <c r="I161" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J161" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 23:19</t>
+        </is>
+      </c>
+      <c r="K161" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07T23:20:48.355298</t>
+        </is>
+      </c>
+      <c r="L161" s="2" t="inlineStr">
+        <is>
+          <t>google_p3</t>
+        </is>
+      </c>
+      <c r="M161" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N161" s="2" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="3" t="inlineStr">
+        <is>
+          <t>Al Tadawi Specialty Hospital - Best Hospital In Dubai</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="D162" s="3" t="inlineStr">
+        <is>
+          <t>https://tadawi.ae/</t>
+        </is>
+      </c>
+      <c r="E162" s="3" t="inlineStr"/>
+      <c r="F162" s="3" t="inlineStr"/>
+      <c r="G162" s="3" t="inlineStr"/>
+      <c r="H162" s="3" t="inlineStr"/>
+      <c r="I162" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J162" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 23:21</t>
+        </is>
+      </c>
+      <c r="K162" s="3" t="inlineStr"/>
+      <c r="L162" s="3" t="inlineStr">
+        <is>
+          <t>google_p4</t>
+        </is>
+      </c>
+      <c r="M162" s="3" t="inlineStr"/>
+      <c r="N162" s="3" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>Thumbay University Hospital - Largest Private Academic ...</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>Dubai</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>https://thumbayuniversityhospital.com/</t>
+        </is>
+      </c>
+      <c r="E163" s="2" t="inlineStr">
+        <is>
+          <t>info@thumbayuniversityhospital.com</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>600515555</t>
+        </is>
+      </c>
+      <c r="G163" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Abdulsalam Al</t>
+        </is>
+      </c>
+      <c r="H163" s="2" t="inlineStr">
+        <is>
+          <t>Solve Operations Challenges: Custom Digital Solution for Thumbay University Hospital</t>
+        </is>
+      </c>
+      <c r="I163" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J163" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07 23:21</t>
+        </is>
+      </c>
+      <c r="K163" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-07T23:23:34.040926</t>
+        </is>
+      </c>
+      <c r="L163" s="2" t="inlineStr">
+        <is>
+          <t>google_p4</t>
+        </is>
+      </c>
+      <c r="M163" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N163" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: Enhance bilingual email generation in Ollama writer
- Added support for generating cold outreach emails in multiple languages, including Japanese, Russian, Korean, Chinese, French, German, Spanish, Portuguese, Dutch, Turkish, Thai, Arabic, Indonesian, Czech, Italian, Polish, Swedish, Norwegian, and Finnish.
- Implemented a city-to-language mapping to determine the appropriate language based on the client's location.
- Updated email structure to include a local language section above the English version.
- Refactored email generation logic to utilize Ollama for both local and English email bodies, with fallbacks to templates if Ollama is not running.
- Enhanced logging to indicate whether emails are generated using AI or templates.
</commit_message>
<xml_diff>
--- a/job_hunter_agent/data/clients.xlsx
+++ b/job_hunter_agent/data/clients.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N331"/>
+  <dimension ref="A1:N418"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -18719,48 +18719,4743 @@
       <c r="N330" s="2" t="inlineStr"/>
     </row>
     <row r="331">
-      <c r="A331" s="4" t="inlineStr">
+      <c r="A331" s="2" t="inlineStr">
         <is>
           <t>Apollo Hospitals: Best Hospital in India | Best Multispeciality ...</t>
         </is>
       </c>
-      <c r="B331" s="4" t="inlineStr">
-        <is>
-          <t>hospital</t>
-        </is>
-      </c>
-      <c r="C331" s="4" t="inlineStr">
+      <c r="B331" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C331" s="2" t="inlineStr">
         <is>
           <t>Bangalore</t>
         </is>
       </c>
-      <c r="D331" s="4" t="inlineStr">
+      <c r="D331" s="2" t="inlineStr">
         <is>
           <t>https://www.apollohospitals.com/</t>
         </is>
       </c>
-      <c r="E331" s="4" t="inlineStr"/>
-      <c r="F331" s="4" t="inlineStr"/>
-      <c r="G331" s="4" t="inlineStr"/>
-      <c r="H331" s="4" t="inlineStr"/>
-      <c r="I331" s="4" t="inlineStr">
+      <c r="E331" s="2" t="inlineStr">
+        <is>
+          <t>dranjali_a@apollohospitals.com</t>
+        </is>
+      </c>
+      <c r="F331" s="2" t="inlineStr">
+        <is>
+          <t>+91 4043441066</t>
+        </is>
+      </c>
+      <c r="G331" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Prathap</t>
+        </is>
+      </c>
+      <c r="H331" s="2" t="inlineStr">
+        <is>
+          <t>Custom Digital Solution for Streamlining Apollo Hospitals Operations</t>
+        </is>
+      </c>
+      <c r="I331" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J331" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 11:44</t>
+        </is>
+      </c>
+      <c r="K331" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T11:46:32.424282</t>
+        </is>
+      </c>
+      <c r="L331" s="2" t="inlineStr">
+        <is>
+          <t>google_p1</t>
+        </is>
+      </c>
+      <c r="M331" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N331" s="2" t="inlineStr"/>
+    </row>
+    <row r="332">
+      <c r="A332" s="3" t="inlineStr">
+        <is>
+          <t>SPARSH Hospital: Best Hospital in Bangalore | MultiSpeciality ...</t>
+        </is>
+      </c>
+      <c r="B332" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C332" s="3" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D332" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sparshhospital.com/</t>
+        </is>
+      </c>
+      <c r="E332" s="3" t="inlineStr"/>
+      <c r="F332" s="3" t="inlineStr">
+        <is>
+          <t>080 61 222 000</t>
+        </is>
+      </c>
+      <c r="G332" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Sharan Shivaraj</t>
+        </is>
+      </c>
+      <c r="H332" s="3" t="inlineStr"/>
+      <c r="I332" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J332" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 11:47</t>
+        </is>
+      </c>
+      <c r="K332" s="3" t="inlineStr"/>
+      <c r="L332" s="3" t="inlineStr">
+        <is>
+          <t>google_p1</t>
+        </is>
+      </c>
+      <c r="M332" s="3" t="inlineStr"/>
+      <c r="N332" s="3" t="inlineStr"/>
+    </row>
+    <row r="333">
+      <c r="A333" s="2" t="inlineStr">
+        <is>
+          <t>St John's National Academy of Health Sciences</t>
+        </is>
+      </c>
+      <c r="B333" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C333" s="2" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D333" s="2" t="inlineStr">
+        <is>
+          <t>https://www.stjohns.in/</t>
+        </is>
+      </c>
+      <c r="E333" s="2" t="inlineStr">
+        <is>
+          <t>sjmch.infodesk@stjohns.in</t>
+        </is>
+      </c>
+      <c r="F333" s="2" t="inlineStr">
+        <is>
+          <t>+91 080 22065000</t>
+        </is>
+      </c>
+      <c r="G333" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Anura Kurpad</t>
+        </is>
+      </c>
+      <c r="H333" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom Digital Solution for Enhanced Hospital Operations</t>
+        </is>
+      </c>
+      <c r="I333" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J333" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 11:47</t>
+        </is>
+      </c>
+      <c r="K333" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T11:49:26.148097</t>
+        </is>
+      </c>
+      <c r="L333" s="2" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M333" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N333" s="2" t="inlineStr"/>
+    </row>
+    <row r="334">
+      <c r="A334" s="3" t="inlineStr">
+        <is>
+          <t>Fortis Hospital BG Road, Bangalore</t>
+        </is>
+      </c>
+      <c r="B334" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C334" s="3" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D334" s="3" t="inlineStr">
+        <is>
+          <t>https://www.fortishealthcare.com/location/fortis-hospital-bg-road-bangalore</t>
+        </is>
+      </c>
+      <c r="E334" s="3" t="inlineStr"/>
+      <c r="F334" s="3" t="inlineStr">
+        <is>
+          <t>9205 010 100</t>
+        </is>
+      </c>
+      <c r="G334" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Mohan  Keshavamurthy</t>
+        </is>
+      </c>
+      <c r="H334" s="3" t="inlineStr"/>
+      <c r="I334" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J334" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 11:50</t>
+        </is>
+      </c>
+      <c r="K334" s="3" t="inlineStr"/>
+      <c r="L334" s="3" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M334" s="3" t="inlineStr"/>
+      <c r="N334" s="3" t="inlineStr"/>
+    </row>
+    <row r="335">
+      <c r="A335" s="2" t="inlineStr">
+        <is>
+          <t>HOSMAT Hospitals: Best Orthopaedic &amp; Multispecialty ...</t>
+        </is>
+      </c>
+      <c r="B335" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C335" s="2" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D335" s="2" t="inlineStr">
+        <is>
+          <t>https://hosmathospitals.com/</t>
+        </is>
+      </c>
+      <c r="E335" s="2" t="inlineStr">
+        <is>
+          <t>info@hosmathospitals.com</t>
+        </is>
+      </c>
+      <c r="F335" s="2" t="inlineStr">
+        <is>
+          <t>+91 9796197961</t>
+        </is>
+      </c>
+      <c r="G335" s="2" t="inlineStr">
+        <is>
+          <t>Dr Thomas</t>
+        </is>
+      </c>
+      <c r="H335" s="2" t="inlineStr">
+        <is>
+          <t>Streamline Operations: Custom Digital Solution Proposal</t>
+        </is>
+      </c>
+      <c r="I335" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J335" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 11:50</t>
+        </is>
+      </c>
+      <c r="K335" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T11:52:17.141635</t>
+        </is>
+      </c>
+      <c r="L335" s="2" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M335" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N335" s="2" t="inlineStr"/>
+    </row>
+    <row r="336">
+      <c r="A336" s="2" t="inlineStr">
+        <is>
+          <t>St. Philomena's Hospital | Multi-Specialty Hospital in ...</t>
+        </is>
+      </c>
+      <c r="B336" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C336" s="2" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D336" s="2" t="inlineStr">
+        <is>
+          <t>https://stphilomenashospital.com/</t>
+        </is>
+      </c>
+      <c r="E336" s="2" t="inlineStr">
+        <is>
+          <t>pro@stphilomenashospital.com</t>
+        </is>
+      </c>
+      <c r="F336" s="2" t="inlineStr">
+        <is>
+          <t>080- 24491449</t>
+        </is>
+      </c>
+      <c r="G336" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Sangeetha</t>
+        </is>
+      </c>
+      <c r="H336" s="2" t="inlineStr">
+        <is>
+          <t>Streamline Operations: Custom Digital Solution Proposal for St. Philomena's Hospital</t>
+        </is>
+      </c>
+      <c r="I336" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J336" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 11:53</t>
+        </is>
+      </c>
+      <c r="K336" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T11:55:02.887434</t>
+        </is>
+      </c>
+      <c r="L336" s="2" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M336" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N336" s="2" t="inlineStr"/>
+    </row>
+    <row r="337">
+      <c r="A337" s="2" t="inlineStr">
+        <is>
+          <t>Mallige Hospital: Discover the Best Multi-Speciality Hospital in ...</t>
+        </is>
+      </c>
+      <c r="B337" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C337" s="2" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D337" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mallige.com/</t>
+        </is>
+      </c>
+      <c r="E337" s="2" t="inlineStr">
+        <is>
+          <t>feedback@mallige.com</t>
+        </is>
+      </c>
+      <c r="F337" s="2" t="inlineStr">
+        <is>
+          <t>+91-80-67165555</t>
+        </is>
+      </c>
+      <c r="G337" s="2" t="inlineStr"/>
+      <c r="H337" s="2" t="inlineStr">
+        <is>
+          <t>Revolutionize Operations at Mallige Hospital: Custom Digital Solution Proposal</t>
+        </is>
+      </c>
+      <c r="I337" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J337" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 11:55</t>
+        </is>
+      </c>
+      <c r="K337" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T11:57:43.854153</t>
+        </is>
+      </c>
+      <c r="L337" s="2" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M337" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N337" s="2" t="inlineStr"/>
+    </row>
+    <row r="338">
+      <c r="A338" s="3" t="inlineStr">
+        <is>
+          <t>Best Multispeciality Hospital in Bangalore</t>
+        </is>
+      </c>
+      <c r="B338" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C338" s="3" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D338" s="3" t="inlineStr">
+        <is>
+          <t>https://vims.ac.in/vims-hospital/</t>
+        </is>
+      </c>
+      <c r="E338" s="3" t="inlineStr"/>
+      <c r="F338" s="3" t="inlineStr">
+        <is>
+          <t>+91-80-4125 9032</t>
+        </is>
+      </c>
+      <c r="G338" s="3" t="inlineStr">
+        <is>
+          <t>Dr. Sharan Prakash</t>
+        </is>
+      </c>
+      <c r="H338" s="3" t="inlineStr"/>
+      <c r="I338" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J338" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 11:58</t>
+        </is>
+      </c>
+      <c r="K338" s="3" t="inlineStr"/>
+      <c r="L338" s="3" t="inlineStr">
+        <is>
+          <t>google_p3</t>
+        </is>
+      </c>
+      <c r="M338" s="3" t="inlineStr"/>
+      <c r="N338" s="3" t="inlineStr"/>
+    </row>
+    <row r="339">
+      <c r="A339" s="3" t="inlineStr">
+        <is>
+          <t>Home - Chinmaya Mission Hospital - Bangalore</t>
+        </is>
+      </c>
+      <c r="B339" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C339" s="3" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D339" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cmhblr.com/</t>
+        </is>
+      </c>
+      <c r="E339" s="3" t="inlineStr"/>
+      <c r="F339" s="3" t="inlineStr">
+        <is>
+          <t>080-25026100</t>
+        </is>
+      </c>
+      <c r="G339" s="3" t="inlineStr"/>
+      <c r="H339" s="3" t="inlineStr"/>
+      <c r="I339" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J339" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 11:58</t>
+        </is>
+      </c>
+      <c r="K339" s="3" t="inlineStr"/>
+      <c r="L339" s="3" t="inlineStr">
+        <is>
+          <t>google_p3</t>
+        </is>
+      </c>
+      <c r="M339" s="3" t="inlineStr"/>
+      <c r="N339" s="3" t="inlineStr"/>
+    </row>
+    <row r="340">
+      <c r="A340" s="6" t="inlineStr">
+        <is>
+          <t>Sagar Hospitals: Best Multispeciality Hospital in Bangalore</t>
+        </is>
+      </c>
+      <c r="B340" s="6" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C340" s="6" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D340" s="6" t="inlineStr">
+        <is>
+          <t>https://www.sagarhospitals.in/</t>
+        </is>
+      </c>
+      <c r="E340" s="6" t="inlineStr">
+        <is>
+          <t>infobsk®sagarhospitals.in</t>
+        </is>
+      </c>
+      <c r="F340" s="6" t="inlineStr">
+        <is>
+          <t>080 69555555</t>
+        </is>
+      </c>
+      <c r="G340" s="6" t="inlineStr">
+        <is>
+          <t>Dr. Nikhil</t>
+        </is>
+      </c>
+      <c r="H340" s="6" t="inlineStr"/>
+      <c r="I340" s="6" t="inlineStr">
+        <is>
+          <t>bounced</t>
+        </is>
+      </c>
+      <c r="J340" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-08 11:58</t>
+        </is>
+      </c>
+      <c r="K340" s="6" t="inlineStr"/>
+      <c r="L340" s="6" t="inlineStr">
+        <is>
+          <t>google_p3</t>
+        </is>
+      </c>
+      <c r="M340" s="6" t="inlineStr"/>
+      <c r="N340" s="6" t="inlineStr"/>
+    </row>
+    <row r="341">
+      <c r="A341" s="2" t="inlineStr">
+        <is>
+          <t>Prakriya Hospitals: Best Hospital in Nagasandra, Bangalore ...</t>
+        </is>
+      </c>
+      <c r="B341" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C341" s="2" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D341" s="2" t="inlineStr">
+        <is>
+          <t>https://www.prakriyahospitals.com/</t>
+        </is>
+      </c>
+      <c r="E341" s="2" t="inlineStr">
+        <is>
+          <t>life@prakriyahospitals.com</t>
+        </is>
+      </c>
+      <c r="F341" s="2" t="inlineStr">
+        <is>
+          <t>080 3737 5555</t>
+        </is>
+      </c>
+      <c r="G341" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Srinivas</t>
+        </is>
+      </c>
+      <c r="H341" s="2" t="inlineStr">
+        <is>
+          <t>Transform Operations at Prakriya Hospitals: Custom Digital Solution Proposal</t>
+        </is>
+      </c>
+      <c r="I341" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J341" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:01</t>
+        </is>
+      </c>
+      <c r="K341" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T12:03:47.955856</t>
+        </is>
+      </c>
+      <c r="L341" s="2" t="inlineStr">
+        <is>
+          <t>google_p3</t>
+        </is>
+      </c>
+      <c r="M341" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N341" s="2" t="inlineStr"/>
+    </row>
+    <row r="342">
+      <c r="A342" s="3" t="inlineStr">
+        <is>
+          <t>Vasavi Hospitals</t>
+        </is>
+      </c>
+      <c r="B342" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C342" s="3" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D342" s="3" t="inlineStr">
+        <is>
+          <t>https://www.vasavihospitals.com/</t>
+        </is>
+      </c>
+      <c r="E342" s="3" t="inlineStr"/>
+      <c r="F342" s="3" t="inlineStr"/>
+      <c r="G342" s="3" t="inlineStr"/>
+      <c r="H342" s="3" t="inlineStr"/>
+      <c r="I342" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J342" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:04</t>
+        </is>
+      </c>
+      <c r="K342" s="3" t="inlineStr"/>
+      <c r="L342" s="3" t="inlineStr">
+        <is>
+          <t>google_p3</t>
+        </is>
+      </c>
+      <c r="M342" s="3" t="inlineStr"/>
+      <c r="N342" s="3" t="inlineStr"/>
+    </row>
+    <row r="343">
+      <c r="A343" s="3" t="inlineStr">
+        <is>
+          <t>Sanjeevini Hospital: Best Cardiac Care and Multi-Specialty ...</t>
+        </is>
+      </c>
+      <c r="B343" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C343" s="3" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D343" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sanjeevinihospital.com/</t>
+        </is>
+      </c>
+      <c r="E343" s="3" t="inlineStr"/>
+      <c r="F343" s="3" t="inlineStr"/>
+      <c r="G343" s="3" t="inlineStr"/>
+      <c r="H343" s="3" t="inlineStr"/>
+      <c r="I343" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J343" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:05</t>
+        </is>
+      </c>
+      <c r="K343" s="3" t="inlineStr"/>
+      <c r="L343" s="3" t="inlineStr">
+        <is>
+          <t>google_p4</t>
+        </is>
+      </c>
+      <c r="M343" s="3" t="inlineStr"/>
+      <c r="N343" s="3" t="inlineStr"/>
+    </row>
+    <row r="344">
+      <c r="A344" s="3" t="inlineStr">
+        <is>
+          <t>BMJH | Home</t>
+        </is>
+      </c>
+      <c r="B344" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C344" s="3" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D344" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bmjh.org/</t>
+        </is>
+      </c>
+      <c r="E344" s="3" t="inlineStr"/>
+      <c r="F344" s="3" t="inlineStr"/>
+      <c r="G344" s="3" t="inlineStr"/>
+      <c r="H344" s="3" t="inlineStr"/>
+      <c r="I344" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J344" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:05</t>
+        </is>
+      </c>
+      <c r="K344" s="3" t="inlineStr"/>
+      <c r="L344" s="3" t="inlineStr">
+        <is>
+          <t>google_p4</t>
+        </is>
+      </c>
+      <c r="M344" s="3" t="inlineStr"/>
+      <c r="N344" s="3" t="inlineStr"/>
+    </row>
+    <row r="345">
+      <c r="A345" s="2" t="inlineStr">
+        <is>
+          <t>St. Theresas Hospital</t>
+        </is>
+      </c>
+      <c r="B345" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C345" s="2" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D345" s="2" t="inlineStr">
+        <is>
+          <t>https://sttheresas.co.in/</t>
+        </is>
+      </c>
+      <c r="E345" s="2" t="inlineStr">
+        <is>
+          <t>theresahospital@gmail.com</t>
+        </is>
+      </c>
+      <c r="F345" s="2" t="inlineStr">
+        <is>
+          <t>080 23472772</t>
+        </is>
+      </c>
+      <c r="G345" s="2" t="inlineStr"/>
+      <c r="H345" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom Digital Solution for Enhanced Hospital Operations</t>
+        </is>
+      </c>
+      <c r="I345" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J345" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:05</t>
+        </is>
+      </c>
+      <c r="K345" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T12:07:36.756450</t>
+        </is>
+      </c>
+      <c r="L345" s="2" t="inlineStr">
+        <is>
+          <t>google_p4</t>
+        </is>
+      </c>
+      <c r="M345" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N345" s="2" t="inlineStr"/>
+    </row>
+    <row r="346">
+      <c r="A346" s="6" t="inlineStr">
+        <is>
+          <t>Bengaluru PPN List of Hospitals | National Insurance</t>
+        </is>
+      </c>
+      <c r="B346" s="6" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C346" s="6" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D346" s="6" t="inlineStr">
+        <is>
+          <t>https://nationalinsurance.nic.co.in/sites/default/files/Bengaluru%20PPN%20List%20of%20Hospitals.pdf</t>
+        </is>
+      </c>
+      <c r="E346" s="6" t="inlineStr">
+        <is>
+          <t>agent[dot]portal[at]nic[dot]co[dot]in</t>
+        </is>
+      </c>
+      <c r="F346" s="6" t="inlineStr">
+        <is>
+          <t>2020-01-29</t>
+        </is>
+      </c>
+      <c r="G346" s="6" t="inlineStr">
+        <is>
+          <t>Head Office Premises</t>
+        </is>
+      </c>
+      <c r="H346" s="6" t="inlineStr"/>
+      <c r="I346" s="6" t="inlineStr">
+        <is>
+          <t>bounced</t>
+        </is>
+      </c>
+      <c r="J346" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:08</t>
+        </is>
+      </c>
+      <c r="K346" s="6" t="inlineStr"/>
+      <c r="L346" s="6" t="inlineStr">
+        <is>
+          <t>google_p4</t>
+        </is>
+      </c>
+      <c r="M346" s="6" t="inlineStr"/>
+      <c r="N346" s="6" t="inlineStr"/>
+    </row>
+    <row r="347">
+      <c r="A347" s="2" t="inlineStr">
+        <is>
+          <t>Sri Sathya Sai Institute of Higher Medical Sciences - Sri ...</t>
+        </is>
+      </c>
+      <c r="B347" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C347" s="2" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D347" s="2" t="inlineStr">
+        <is>
+          <t>https://sssihms.org/</t>
+        </is>
+      </c>
+      <c r="E347" s="2" t="inlineStr">
+        <is>
+          <t>publicrelationspg@sssihms.org.in</t>
+        </is>
+      </c>
+      <c r="F347" s="2" t="inlineStr">
+        <is>
+          <t>+91 (08555) 287388</t>
+        </is>
+      </c>
+      <c r="G347" s="2" t="inlineStr"/>
+      <c r="H347" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom Digital Solution for Enhanced Hospital Operations</t>
+        </is>
+      </c>
+      <c r="I347" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J347" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:10</t>
+        </is>
+      </c>
+      <c r="K347" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T12:12:01.791850</t>
+        </is>
+      </c>
+      <c r="L347" s="2" t="inlineStr">
+        <is>
+          <t>google_p4</t>
+        </is>
+      </c>
+      <c r="M347" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N347" s="2" t="inlineStr"/>
+    </row>
+    <row r="348">
+      <c r="A348" s="2" t="inlineStr">
+        <is>
+          <t>Yashoda Hospitals: Best Hospital in Hyderabad | Multi ...</t>
+        </is>
+      </c>
+      <c r="B348" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C348" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="D348" s="2" t="inlineStr">
+        <is>
+          <t>https://www.yashodahospitals.com/</t>
+        </is>
+      </c>
+      <c r="E348" s="2" t="inlineStr">
+        <is>
+          <t>query@yashodamail.com</t>
+        </is>
+      </c>
+      <c r="F348" s="2" t="inlineStr">
+        <is>
+          <t>+91 40 4567 4567</t>
+        </is>
+      </c>
+      <c r="G348" s="2" t="inlineStr">
+        <is>
+          <t>Mr. Pankaj Das</t>
+        </is>
+      </c>
+      <c r="H348" s="2" t="inlineStr">
+        <is>
+          <t>Optimize Operations at Yashoda Hospitals: Custom Digital Solution Proposal</t>
+        </is>
+      </c>
+      <c r="I348" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J348" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:12</t>
+        </is>
+      </c>
+      <c r="K348" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T12:14:38.772702</t>
+        </is>
+      </c>
+      <c r="L348" s="2" t="inlineStr">
+        <is>
+          <t>google_p1</t>
+        </is>
+      </c>
+      <c r="M348" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N348" s="2" t="inlineStr"/>
+    </row>
+    <row r="349">
+      <c r="A349" s="3" t="inlineStr">
+        <is>
+          <t>CARE Hospitals: Best Hospital in Hyderabad | Best ...</t>
+        </is>
+      </c>
+      <c r="B349" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C349" s="3" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="D349" s="3" t="inlineStr">
+        <is>
+          <t>https://www.carehospitals.com/</t>
+        </is>
+      </c>
+      <c r="E349" s="3" t="inlineStr"/>
+      <c r="F349" s="3" t="inlineStr">
+        <is>
+          <t>+91-4068106587</t>
+        </is>
+      </c>
+      <c r="G349" s="3" t="inlineStr">
+        <is>
+          <t>Mr. Varun Khanna</t>
+        </is>
+      </c>
+      <c r="H349" s="3" t="inlineStr"/>
+      <c r="I349" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J349" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:15</t>
+        </is>
+      </c>
+      <c r="K349" s="3" t="inlineStr"/>
+      <c r="L349" s="3" t="inlineStr">
+        <is>
+          <t>google_p1</t>
+        </is>
+      </c>
+      <c r="M349" s="3" t="inlineStr"/>
+      <c r="N349" s="3" t="inlineStr"/>
+    </row>
+    <row r="350">
+      <c r="A350" s="3" t="inlineStr">
+        <is>
+          <t>AIG Hospitals: Best Multi-Speciality Hospital in Hyderabad</t>
+        </is>
+      </c>
+      <c r="B350" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C350" s="3" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="D350" s="3" t="inlineStr">
+        <is>
+          <t>https://www.aighospitals.com/</t>
+        </is>
+      </c>
+      <c r="E350" s="3" t="inlineStr"/>
+      <c r="F350" s="3" t="inlineStr">
+        <is>
+          <t>+91 40 4244 4244</t>
+        </is>
+      </c>
+      <c r="G350" s="3" t="inlineStr"/>
+      <c r="H350" s="3" t="inlineStr"/>
+      <c r="I350" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J350" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:15</t>
+        </is>
+      </c>
+      <c r="K350" s="3" t="inlineStr"/>
+      <c r="L350" s="3" t="inlineStr">
+        <is>
+          <t>google_p1</t>
+        </is>
+      </c>
+      <c r="M350" s="3" t="inlineStr"/>
+      <c r="N350" s="3" t="inlineStr"/>
+    </row>
+    <row r="351">
+      <c r="A351" s="2" t="inlineStr">
+        <is>
+          <t>Best Hospital in Hyderabad | Multispecialty Healthcare</t>
+        </is>
+      </c>
+      <c r="B351" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C351" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="D351" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apollohospitals.com/hyderabad</t>
+        </is>
+      </c>
+      <c r="E351" s="2" t="inlineStr">
+        <is>
+          <t>dranjali_a@apollohospitals.com</t>
+        </is>
+      </c>
+      <c r="F351" s="2" t="inlineStr">
+        <is>
+          <t>+91 4043441066</t>
+        </is>
+      </c>
+      <c r="G351" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Prathap</t>
+        </is>
+      </c>
+      <c r="H351" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom Digital Solution for Streamlined Operations</t>
+        </is>
+      </c>
+      <c r="I351" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J351" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:15</t>
+        </is>
+      </c>
+      <c r="K351" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T12:17:33.064304</t>
+        </is>
+      </c>
+      <c r="L351" s="2" t="inlineStr">
+        <is>
+          <t>google_p1</t>
+        </is>
+      </c>
+      <c r="M351" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N351" s="2" t="inlineStr"/>
+    </row>
+    <row r="352">
+      <c r="A352" s="2" t="inlineStr">
+        <is>
+          <t>Best Hospital in Hyderabad, India | Multi-Super Speciality Care</t>
+        </is>
+      </c>
+      <c r="B352" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C352" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="D352" s="2" t="inlineStr">
+        <is>
+          <t>https://www.pacehospital.com/</t>
+        </is>
+      </c>
+      <c r="E352" s="2" t="inlineStr">
+        <is>
+          <t>customercare@pacehospital.com</t>
+        </is>
+      </c>
+      <c r="F352" s="2" t="inlineStr">
+        <is>
+          <t>040 4848 6868</t>
+        </is>
+      </c>
+      <c r="G352" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Govind Verma</t>
+        </is>
+      </c>
+      <c r="H352" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom Digital Solution for Streamlined Hospital Operations</t>
+        </is>
+      </c>
+      <c r="I352" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J352" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:18</t>
+        </is>
+      </c>
+      <c r="K352" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T12:20:07.864204</t>
+        </is>
+      </c>
+      <c r="L352" s="2" t="inlineStr">
+        <is>
+          <t>google_p1</t>
+        </is>
+      </c>
+      <c r="M352" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N352" s="2" t="inlineStr"/>
+    </row>
+    <row r="353">
+      <c r="A353" s="2" t="inlineStr">
+        <is>
+          <t>Best Cancer Care Multispecialty Hospital in Hyderabad | Near ...</t>
+        </is>
+      </c>
+      <c r="B353" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C353" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="D353" s="2" t="inlineStr">
+        <is>
+          <t>https://www.amorhospitals.com/</t>
+        </is>
+      </c>
+      <c r="E353" s="2" t="inlineStr">
+        <is>
+          <t>info@amorhospitals.in</t>
+        </is>
+      </c>
+      <c r="F353" s="2" t="inlineStr">
+        <is>
+          <t>+91 40 6606 9999</t>
+        </is>
+      </c>
+      <c r="G353" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Kishore</t>
+        </is>
+      </c>
+      <c r="H353" s="2" t="inlineStr">
+        <is>
+          <t>Transforming Operations at Best Cancer Care: Custom Digital Solution Proposal</t>
+        </is>
+      </c>
+      <c r="I353" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J353" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:20</t>
+        </is>
+      </c>
+      <c r="K353" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T12:22:40.469510</t>
+        </is>
+      </c>
+      <c r="L353" s="2" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M353" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N353" s="2" t="inlineStr"/>
+    </row>
+    <row r="354">
+      <c r="A354" s="2" t="inlineStr">
+        <is>
+          <t>Star Hospitals | Best Multispeciality Hospital in Hyderabad</t>
+        </is>
+      </c>
+      <c r="B354" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C354" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="D354" s="2" t="inlineStr">
+        <is>
+          <t>https://www.starhospitals.in/</t>
+        </is>
+      </c>
+      <c r="E354" s="2" t="inlineStr">
+        <is>
+          <t>cio@starhospitals.co.in</t>
+        </is>
+      </c>
+      <c r="F354" s="2" t="inlineStr">
+        <is>
+          <t>1800 102 7827</t>
+        </is>
+      </c>
+      <c r="G354" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Ramesh Gudapati</t>
+        </is>
+      </c>
+      <c r="H354" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom Digital Solution for Streamlined Operations @ Star Hospitals</t>
+        </is>
+      </c>
+      <c r="I354" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J354" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:23</t>
+        </is>
+      </c>
+      <c r="K354" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T12:25:15.241453</t>
+        </is>
+      </c>
+      <c r="L354" s="2" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M354" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N354" s="2" t="inlineStr"/>
+    </row>
+    <row r="355">
+      <c r="A355" s="2" t="inlineStr">
+        <is>
+          <t>Kingston Hospitals</t>
+        </is>
+      </c>
+      <c r="B355" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C355" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="D355" s="2" t="inlineStr">
+        <is>
+          <t>https://kingstonhospitals.in/</t>
+        </is>
+      </c>
+      <c r="E355" s="2" t="inlineStr">
+        <is>
+          <t>info@kingstonhospitals.in</t>
+        </is>
+      </c>
+      <c r="F355" s="2" t="inlineStr">
+        <is>
+          <t>+91 9100010007</t>
+        </is>
+      </c>
+      <c r="G355" s="2" t="inlineStr">
+        <is>
+          <t>Dr Mohammed</t>
+        </is>
+      </c>
+      <c r="H355" s="2" t="inlineStr">
+        <is>
+          <t>Revolutionize Operations: Custom Digital Solution Proposal</t>
+        </is>
+      </c>
+      <c r="I355" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J355" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:26</t>
+        </is>
+      </c>
+      <c r="K355" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T12:27:43.678430</t>
+        </is>
+      </c>
+      <c r="L355" s="2" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M355" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N355" s="2" t="inlineStr"/>
+    </row>
+    <row r="356">
+      <c r="A356" s="3" t="inlineStr">
+        <is>
+          <t>OMNI Hospitals: Best Multispeciality Hospital in Hyderabad ...</t>
+        </is>
+      </c>
+      <c r="B356" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C356" s="3" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="D356" s="3" t="inlineStr">
+        <is>
+          <t>https://omnihospitals.in/</t>
+        </is>
+      </c>
+      <c r="E356" s="3" t="inlineStr"/>
+      <c r="F356" s="3" t="inlineStr"/>
+      <c r="G356" s="3" t="inlineStr"/>
+      <c r="H356" s="3" t="inlineStr"/>
+      <c r="I356" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J356" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:28</t>
+        </is>
+      </c>
+      <c r="K356" s="3" t="inlineStr"/>
+      <c r="L356" s="3" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M356" s="3" t="inlineStr"/>
+      <c r="N356" s="3" t="inlineStr"/>
+    </row>
+    <row r="357">
+      <c r="A357" s="2" t="inlineStr">
+        <is>
+          <t>Best Hospital in Hyderabad | Multi-Specialty Hospital in ...</t>
+        </is>
+      </c>
+      <c r="B357" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C357" s="2" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="D357" s="2" t="inlineStr">
+        <is>
+          <t>https://vivekanandahospital.in/</t>
+        </is>
+      </c>
+      <c r="E357" s="2" t="inlineStr">
+        <is>
+          <t>info@vivekanandahospital.in</t>
+        </is>
+      </c>
+      <c r="F357" s="2" t="inlineStr">
+        <is>
+          <t>040 35261414</t>
+        </is>
+      </c>
+      <c r="G357" s="2" t="inlineStr">
+        <is>
+          <t>Dr. Shree Mukesh</t>
+        </is>
+      </c>
+      <c r="H357" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom Digital Solution for Efficient Hospital Operations</t>
+        </is>
+      </c>
+      <c r="I357" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J357" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:28</t>
+        </is>
+      </c>
+      <c r="K357" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T12:30:25.578378</t>
+        </is>
+      </c>
+      <c r="L357" s="2" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M357" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N357" s="2" t="inlineStr"/>
+    </row>
+    <row r="358">
+      <c r="A358" s="3" t="inlineStr">
+        <is>
+          <t>bbb health boutique | beste vrouwensportschool</t>
+        </is>
+      </c>
+      <c r="B358" s="3" t="inlineStr">
+        <is>
+          <t>gym</t>
+        </is>
+      </c>
+      <c r="C358" s="3" t="inlineStr">
+        <is>
+          <t>gyms Amsterdam</t>
+        </is>
+      </c>
+      <c r="D358" s="3" t="inlineStr">
+        <is>
+          <t>https://info.bbbhealthboutique.nl/proefles?studio=AMS01</t>
+        </is>
+      </c>
+      <c r="E358" s="3" t="inlineStr"/>
+      <c r="F358" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G358" s="3" t="inlineStr"/>
+      <c r="H358" s="3" t="inlineStr"/>
+      <c r="I358" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J358" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:31</t>
+        </is>
+      </c>
+      <c r="K358" s="3" t="inlineStr"/>
+      <c r="L358" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M358" s="3" t="inlineStr"/>
+      <c r="N358" s="3" t="inlineStr"/>
+    </row>
+    <row r="359">
+      <c r="A359" s="3" t="inlineStr">
+        <is>
+          <t>TrainMore Amsterdam Oost Black Label</t>
+        </is>
+      </c>
+      <c r="B359" s="3" t="inlineStr">
+        <is>
+          <t>gym</t>
+        </is>
+      </c>
+      <c r="C359" s="3" t="inlineStr">
+        <is>
+          <t>gyms Amsterdam</t>
+        </is>
+      </c>
+      <c r="D359" s="3" t="inlineStr">
+        <is>
+          <t>https://trainmore.com/nl-NL/clubs/amsterdam/oost/?utm_source=GMB-Amsterdam-Oost-Black-Label&amp;utm_medium=GMB&amp;utm_campaign=GMB-direct</t>
+        </is>
+      </c>
+      <c r="E359" s="3" t="inlineStr"/>
+      <c r="F359" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G359" s="3" t="inlineStr"/>
+      <c r="H359" s="3" t="inlineStr"/>
+      <c r="I359" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J359" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:31</t>
+        </is>
+      </c>
+      <c r="K359" s="3" t="inlineStr"/>
+      <c r="L359" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M359" s="3" t="inlineStr"/>
+      <c r="N359" s="3" t="inlineStr"/>
+    </row>
+    <row r="360">
+      <c r="A360" s="3" t="inlineStr">
+        <is>
+          <t>TrainMore Amsterdam Oosterdok</t>
+        </is>
+      </c>
+      <c r="B360" s="3" t="inlineStr">
+        <is>
+          <t>gym</t>
+        </is>
+      </c>
+      <c r="C360" s="3" t="inlineStr">
+        <is>
+          <t>gyms Amsterdam</t>
+        </is>
+      </c>
+      <c r="D360" s="3" t="inlineStr">
+        <is>
+          <t>https://trainmore.com/nl-NL/clubs/amsterdam/oosterdok/?utm_source=GMB-Amsterdam-Oosterdok&amp;utm_medium=GMB&amp;utm_campaign=GMB-direct</t>
+        </is>
+      </c>
+      <c r="E360" s="3" t="inlineStr"/>
+      <c r="F360" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G360" s="3" t="inlineStr"/>
+      <c r="H360" s="3" t="inlineStr"/>
+      <c r="I360" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J360" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:31</t>
+        </is>
+      </c>
+      <c r="K360" s="3" t="inlineStr"/>
+      <c r="L360" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M360" s="3" t="inlineStr"/>
+      <c r="N360" s="3" t="inlineStr"/>
+    </row>
+    <row r="361">
+      <c r="A361" s="3" t="inlineStr">
+        <is>
+          <t>TrainMore Amsterdam Singel Black Label</t>
+        </is>
+      </c>
+      <c r="B361" s="3" t="inlineStr">
+        <is>
+          <t>gym</t>
+        </is>
+      </c>
+      <c r="C361" s="3" t="inlineStr">
+        <is>
+          <t>gyms Amsterdam</t>
+        </is>
+      </c>
+      <c r="D361" s="3" t="inlineStr">
+        <is>
+          <t>https://trainmore.com/nl-NL/clubs/amsterdam/singel/?utm_source=GMB-Amsterdam-Singel-Black-Label&amp;utm_medium=GMB&amp;utm_campaign=GMB-direct</t>
+        </is>
+      </c>
+      <c r="E361" s="3" t="inlineStr"/>
+      <c r="F361" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G361" s="3" t="inlineStr"/>
+      <c r="H361" s="3" t="inlineStr"/>
+      <c r="I361" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J361" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:31</t>
+        </is>
+      </c>
+      <c r="K361" s="3" t="inlineStr"/>
+      <c r="L361" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M361" s="3" t="inlineStr"/>
+      <c r="N361" s="3" t="inlineStr"/>
+    </row>
+    <row r="362">
+      <c r="A362" s="3" t="inlineStr">
+        <is>
+          <t>TrainMore Amsterdam Noord</t>
+        </is>
+      </c>
+      <c r="B362" s="3" t="inlineStr">
+        <is>
+          <t>gym</t>
+        </is>
+      </c>
+      <c r="C362" s="3" t="inlineStr">
+        <is>
+          <t>gyms Amsterdam</t>
+        </is>
+      </c>
+      <c r="D362" s="3" t="inlineStr">
+        <is>
+          <t>https://trainmore.com/nl-NL/clubs/amsterdam/noord/?utm_source=GMB-Amsterdam-Noord&amp;utm_medium=GMB&amp;utm_campaign=GMB-direct</t>
+        </is>
+      </c>
+      <c r="E362" s="3" t="inlineStr"/>
+      <c r="F362" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G362" s="3" t="inlineStr"/>
+      <c r="H362" s="3" t="inlineStr"/>
+      <c r="I362" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J362" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:31</t>
+        </is>
+      </c>
+      <c r="K362" s="3" t="inlineStr"/>
+      <c r="L362" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M362" s="3" t="inlineStr"/>
+      <c r="N362" s="3" t="inlineStr"/>
+    </row>
+    <row r="363">
+      <c r="A363" s="2" t="inlineStr">
+        <is>
+          <t>The Gym</t>
+        </is>
+      </c>
+      <c r="B363" s="2" t="inlineStr">
+        <is>
+          <t>gym</t>
+        </is>
+      </c>
+      <c r="C363" s="2" t="inlineStr">
+        <is>
+          <t>gyms Amsterdam</t>
+        </is>
+      </c>
+      <c r="D363" s="2" t="inlineStr">
+        <is>
+          <t>http://www.thegym.amsterdam/</t>
+        </is>
+      </c>
+      <c r="E363" s="2" t="inlineStr">
+        <is>
+          <t>info@thegym.amsterdam</t>
+        </is>
+      </c>
+      <c r="F363" s="2" t="inlineStr">
+        <is>
+          <t>+31 651 68 36 38</t>
+        </is>
+      </c>
+      <c r="G363" s="2" t="inlineStr">
+        <is>
+          <t>Head Trainer</t>
+        </is>
+      </c>
+      <c r="H363" s="2" t="inlineStr">
+        <is>
+          <t>Streamline Gym Operations: Custom Digital Solution Proposal</t>
+        </is>
+      </c>
+      <c r="I363" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J363" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:32</t>
+        </is>
+      </c>
+      <c r="K363" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T12:33:32.464437</t>
+        </is>
+      </c>
+      <c r="L363" s="2" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M363" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N363" s="2" t="inlineStr"/>
+    </row>
+    <row r="364">
+      <c r="A364" s="3" t="inlineStr">
+        <is>
+          <t>TrainMore Amsterdam Van Wou</t>
+        </is>
+      </c>
+      <c r="B364" s="3" t="inlineStr">
+        <is>
+          <t>gym</t>
+        </is>
+      </c>
+      <c r="C364" s="3" t="inlineStr">
+        <is>
+          <t>gyms Amsterdam</t>
+        </is>
+      </c>
+      <c r="D364" s="3" t="inlineStr">
+        <is>
+          <t>https://trainmore.com/nl-NL/clubs/amsterdam/van-woustraat/?utm_source=GMB-Amsterdam-Van-Wou&amp;utm_medium=GMB&amp;utm_campaign=GMB-direct</t>
+        </is>
+      </c>
+      <c r="E364" s="3" t="inlineStr"/>
+      <c r="F364" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G364" s="3" t="inlineStr"/>
+      <c r="H364" s="3" t="inlineStr"/>
+      <c r="I364" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J364" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:34</t>
+        </is>
+      </c>
+      <c r="K364" s="3" t="inlineStr"/>
+      <c r="L364" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M364" s="3" t="inlineStr"/>
+      <c r="N364" s="3" t="inlineStr"/>
+    </row>
+    <row r="365">
+      <c r="A365" s="3" t="inlineStr">
+        <is>
+          <t>TrainMore Amsterdam West</t>
+        </is>
+      </c>
+      <c r="B365" s="3" t="inlineStr">
+        <is>
+          <t>gym</t>
+        </is>
+      </c>
+      <c r="C365" s="3" t="inlineStr">
+        <is>
+          <t>gyms Amsterdam</t>
+        </is>
+      </c>
+      <c r="D365" s="3" t="inlineStr">
+        <is>
+          <t>https://trainmore.com/nl-NL/clubs/amsterdam/west/?utm_source=GMB-Amsterdam-West&amp;utm_medium=GMB&amp;utm_campaign=GMB-direct</t>
+        </is>
+      </c>
+      <c r="E365" s="3" t="inlineStr"/>
+      <c r="F365" s="3" t="inlineStr">
+        <is>
+          <t>Send to phone</t>
+        </is>
+      </c>
+      <c r="G365" s="3" t="inlineStr"/>
+      <c r="H365" s="3" t="inlineStr"/>
+      <c r="I365" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J365" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:34</t>
+        </is>
+      </c>
+      <c r="K365" s="3" t="inlineStr"/>
+      <c r="L365" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M365" s="3" t="inlineStr"/>
+      <c r="N365" s="3" t="inlineStr"/>
+    </row>
+    <row r="366">
+      <c r="A366" s="3" t="inlineStr">
+        <is>
+          <t>BLESS Restaurant</t>
+        </is>
+      </c>
+      <c r="B366" s="3" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="C366" s="3" t="inlineStr">
+        <is>
+          <t>restaurants Berlin</t>
+        </is>
+      </c>
+      <c r="D366" s="3" t="inlineStr">
+        <is>
+          <t>https://bless-restaurants.com/berlin/speisekarte/</t>
+        </is>
+      </c>
+      <c r="E366" s="3" t="inlineStr"/>
+      <c r="F366" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="G366" s="3" t="inlineStr"/>
+      <c r="H366" s="3" t="inlineStr"/>
+      <c r="I366" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J366" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:34</t>
+        </is>
+      </c>
+      <c r="K366" s="3" t="inlineStr"/>
+      <c r="L366" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M366" s="3" t="inlineStr"/>
+      <c r="N366" s="3" t="inlineStr"/>
+    </row>
+    <row r="367">
+      <c r="A367" s="3" t="inlineStr">
+        <is>
+          <t>Nante-Eck | Restaurant Berlin Mitte</t>
+        </is>
+      </c>
+      <c r="B367" s="3" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="C367" s="3" t="inlineStr">
+        <is>
+          <t>restaurants Berlin</t>
+        </is>
+      </c>
+      <c r="D367" s="3" t="inlineStr">
+        <is>
+          <t>https://www.nante-eck.de/reservierung</t>
+        </is>
+      </c>
+      <c r="E367" s="3" t="inlineStr"/>
+      <c r="F367" s="3" t="inlineStr">
+        <is>
+          <t>+49 30 22487257</t>
+        </is>
+      </c>
+      <c r="G367" s="3" t="inlineStr"/>
+      <c r="H367" s="3" t="inlineStr"/>
+      <c r="I367" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J367" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:35</t>
+        </is>
+      </c>
+      <c r="K367" s="3" t="inlineStr"/>
+      <c r="L367" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M367" s="3" t="inlineStr"/>
+      <c r="N367" s="3" t="inlineStr"/>
+    </row>
+    <row r="368">
+      <c r="A368" s="2" t="inlineStr">
+        <is>
+          <t>Restaurant Facil</t>
+        </is>
+      </c>
+      <c r="B368" s="2" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="C368" s="2" t="inlineStr">
+        <is>
+          <t>restaurants Berlin</t>
+        </is>
+      </c>
+      <c r="D368" s="2" t="inlineStr">
+        <is>
+          <t>https://facil.de/de/menu/</t>
+        </is>
+      </c>
+      <c r="E368" s="2" t="inlineStr">
+        <is>
+          <t>welcome@facil.de</t>
+        </is>
+      </c>
+      <c r="F368" s="2" t="inlineStr">
+        <is>
+          <t>+49 30 5900 5 1234</t>
+        </is>
+      </c>
+      <c r="G368" s="2" t="inlineStr"/>
+      <c r="H368" s="2" t="inlineStr">
+        <is>
+          <t>Solve Operations Challenges: Custom Digital System for Your Restaurant</t>
+        </is>
+      </c>
+      <c r="I368" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J368" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:35</t>
+        </is>
+      </c>
+      <c r="K368" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T12:37:03.098094</t>
+        </is>
+      </c>
+      <c r="L368" s="2" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M368" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N368" s="2" t="inlineStr"/>
+    </row>
+    <row r="369">
+      <c r="A369" s="2" t="inlineStr">
+        <is>
+          <t>Restaurant Trattoria Portofino</t>
+        </is>
+      </c>
+      <c r="B369" s="2" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="C369" s="2" t="inlineStr">
+        <is>
+          <t>restaurants Berlin</t>
+        </is>
+      </c>
+      <c r="D369" s="2" t="inlineStr">
+        <is>
+          <t>http://www.portofino-trattoria.de/</t>
+        </is>
+      </c>
+      <c r="E369" s="2" t="inlineStr">
+        <is>
+          <t>info@portofino-trattoria.de</t>
+        </is>
+      </c>
+      <c r="F369" s="2" t="inlineStr">
+        <is>
+          <t>030 - 239 10 610</t>
+        </is>
+      </c>
+      <c r="G369" s="2" t="inlineStr"/>
+      <c r="H369" s="2" t="inlineStr">
+        <is>
+          <t>Streamline Operations: Custom Digital System Proposal</t>
+        </is>
+      </c>
+      <c r="I369" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J369" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:37</t>
+        </is>
+      </c>
+      <c r="K369" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T12:39:46.188220</t>
+        </is>
+      </c>
+      <c r="L369" s="2" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M369" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N369" s="2" t="inlineStr"/>
+    </row>
+    <row r="370">
+      <c r="A370" s="3" t="inlineStr">
+        <is>
+          <t>A Mano</t>
+        </is>
+      </c>
+      <c r="B370" s="3" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="C370" s="3" t="inlineStr">
+        <is>
+          <t>restaurants Berlin</t>
+        </is>
+      </c>
+      <c r="D370" s="3" t="inlineStr">
+        <is>
+          <t>https://www.amano-ristorante.de/reservierung/</t>
+        </is>
+      </c>
+      <c r="E370" s="3" t="inlineStr"/>
+      <c r="F370" s="3" t="inlineStr">
+        <is>
+          <t>95 59 82 43</t>
+        </is>
+      </c>
+      <c r="G370" s="3" t="inlineStr"/>
+      <c r="H370" s="3" t="inlineStr"/>
+      <c r="I370" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J370" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:40</t>
+        </is>
+      </c>
+      <c r="K370" s="3" t="inlineStr"/>
+      <c r="L370" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M370" s="3" t="inlineStr"/>
+      <c r="N370" s="3" t="inlineStr"/>
+    </row>
+    <row r="371">
+      <c r="A371" s="3" t="inlineStr">
+        <is>
+          <t>Restaurant Maximilians Berlin</t>
+        </is>
+      </c>
+      <c r="B371" s="3" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="C371" s="3" t="inlineStr">
+        <is>
+          <t>restaurants Berlin</t>
+        </is>
+      </c>
+      <c r="D371" s="3" t="inlineStr">
+        <is>
+          <t>https://www.maximilians-berlin.de/reservieren</t>
+        </is>
+      </c>
+      <c r="E371" s="3" t="inlineStr"/>
+      <c r="F371" s="3" t="inlineStr">
+        <is>
+          <t>190  10117</t>
+        </is>
+      </c>
+      <c r="G371" s="3" t="inlineStr"/>
+      <c r="H371" s="3" t="inlineStr"/>
+      <c r="I371" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J371" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:40</t>
+        </is>
+      </c>
+      <c r="K371" s="3" t="inlineStr"/>
+      <c r="L371" s="3" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M371" s="3" t="inlineStr"/>
+      <c r="N371" s="3" t="inlineStr"/>
+    </row>
+    <row r="372">
+      <c r="A372" s="4" t="inlineStr">
+        <is>
+          <t>Restaurant Dae Mon</t>
+        </is>
+      </c>
+      <c r="B372" s="4" t="inlineStr">
+        <is>
+          <t>restaurant</t>
+        </is>
+      </c>
+      <c r="C372" s="4" t="inlineStr">
+        <is>
+          <t>restaurants Berlin</t>
+        </is>
+      </c>
+      <c r="D372" s="4" t="inlineStr">
+        <is>
+          <t>https://dae-mon.com/#menu</t>
+        </is>
+      </c>
+      <c r="E372" s="4" t="inlineStr">
+        <is>
+          <t>mail@dae-mon.com</t>
+        </is>
+      </c>
+      <c r="F372" s="4" t="inlineStr">
+        <is>
+          <t>030 26 30 48 11</t>
+        </is>
+      </c>
+      <c r="G372" s="4" t="inlineStr"/>
+      <c r="H372" s="4" t="inlineStr"/>
+      <c r="I372" s="4" t="inlineStr">
         <is>
           <t>found</t>
         </is>
       </c>
-      <c r="J331" s="4" t="inlineStr">
-        <is>
-          <t>2026-05-08 11:44</t>
-        </is>
-      </c>
-      <c r="K331" s="4" t="inlineStr"/>
-      <c r="L331" s="4" t="inlineStr">
+      <c r="J372" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-08 12:41</t>
+        </is>
+      </c>
+      <c r="K372" s="4" t="inlineStr"/>
+      <c r="L372" s="4" t="inlineStr">
+        <is>
+          <t>google_maps</t>
+        </is>
+      </c>
+      <c r="M372" s="4" t="inlineStr"/>
+      <c r="N372" s="4" t="inlineStr"/>
+    </row>
+    <row r="373">
+      <c r="A373" s="3" t="inlineStr">
+        <is>
+          <t>St. Luke's International Hospital</t>
+        </is>
+      </c>
+      <c r="B373" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C373" s="3" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="D373" s="3" t="inlineStr">
+        <is>
+          <t>https://hospital.luke.ac.jp/eng/</t>
+        </is>
+      </c>
+      <c r="E373" s="3" t="inlineStr"/>
+      <c r="F373" s="3" t="inlineStr">
+        <is>
+          <t>03-3541-5151</t>
+        </is>
+      </c>
+      <c r="G373" s="3" t="inlineStr"/>
+      <c r="H373" s="3" t="inlineStr"/>
+      <c r="I373" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J373" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:07</t>
+        </is>
+      </c>
+      <c r="K373" s="3" t="inlineStr"/>
+      <c r="L373" s="3" t="inlineStr">
         <is>
           <t>google_p1</t>
         </is>
       </c>
-      <c r="M331" s="4" t="inlineStr"/>
-      <c r="N331" s="4" t="inlineStr"/>
+      <c r="M373" s="3" t="inlineStr"/>
+      <c r="N373" s="3" t="inlineStr"/>
+    </row>
+    <row r="374">
+      <c r="A374" s="2" t="inlineStr">
+        <is>
+          <t>NTT Medical Center Tokyo</t>
+        </is>
+      </c>
+      <c r="B374" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C374" s="2" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="D374" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nmct.ntt-east.co.jp/en/</t>
+        </is>
+      </c>
+      <c r="E374" s="2" t="inlineStr">
+        <is>
+          <t>nttihc-ml@east.ntt.co.jp</t>
+        </is>
+      </c>
+      <c r="F374" s="2" t="inlineStr">
+        <is>
+          <t>03-6721-6239</t>
+        </is>
+      </c>
+      <c r="G374" s="2" t="inlineStr"/>
+      <c r="H374" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom Digital Solution for Streamlined Hospital Operations</t>
+        </is>
+      </c>
+      <c r="I374" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J374" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:07</t>
+        </is>
+      </c>
+      <c r="K374" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T13:10:18.109490</t>
+        </is>
+      </c>
+      <c r="L374" s="2" t="inlineStr">
+        <is>
+          <t>google_p1</t>
+        </is>
+      </c>
+      <c r="M374" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N374" s="2" t="inlineStr"/>
+    </row>
+    <row r="375">
+      <c r="A375" s="3" t="inlineStr">
+        <is>
+          <t>Center Hospital of National Center for Global Health and ...</t>
+        </is>
+      </c>
+      <c r="B375" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C375" s="3" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="D375" s="3" t="inlineStr">
+        <is>
+          <t>https://www.hosp.jihs.go.jp/en/index.html</t>
+        </is>
+      </c>
+      <c r="E375" s="3" t="inlineStr"/>
+      <c r="F375" s="3" t="inlineStr">
+        <is>
+          <t>+81-3-3202-7181</t>
+        </is>
+      </c>
+      <c r="G375" s="3" t="inlineStr">
+        <is>
+          <t>Director 
+ Mission</t>
+        </is>
+      </c>
+      <c r="H375" s="3" t="inlineStr"/>
+      <c r="I375" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J375" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:11</t>
+        </is>
+      </c>
+      <c r="K375" s="3" t="inlineStr"/>
+      <c r="L375" s="3" t="inlineStr">
+        <is>
+          <t>google_p1</t>
+        </is>
+      </c>
+      <c r="M375" s="3" t="inlineStr"/>
+      <c r="N375" s="3" t="inlineStr"/>
+    </row>
+    <row r="376">
+      <c r="A376" s="2" t="inlineStr">
+        <is>
+          <t>Tokyo Station International Clinic【Official】English ...</t>
+        </is>
+      </c>
+      <c r="B376" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C376" s="2" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="D376" s="2" t="inlineStr">
+        <is>
+          <t>https://www.international-clinic.tokyo/</t>
+        </is>
+      </c>
+      <c r="E376" s="2" t="inlineStr">
+        <is>
+          <t>tsic@businessclinic.tokyo</t>
+        </is>
+      </c>
+      <c r="F376" s="2" t="inlineStr">
+        <is>
+          <t>03-6206-3070</t>
+        </is>
+      </c>
+      <c r="G376" s="2" t="inlineStr"/>
+      <c r="H376" s="2" t="inlineStr">
+        <is>
+          <t>Propose Custom Digital Solution for Operations Enhancement</t>
+        </is>
+      </c>
+      <c r="I376" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J376" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:11</t>
+        </is>
+      </c>
+      <c r="K376" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T13:18:40.176708</t>
+        </is>
+      </c>
+      <c r="L376" s="2" t="inlineStr">
+        <is>
+          <t>google_p1</t>
+        </is>
+      </c>
+      <c r="M376" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N376" s="2" t="inlineStr"/>
+    </row>
+    <row r="377">
+      <c r="A377" s="3" t="inlineStr">
+        <is>
+          <t>Medical Care / Affairs｜General Consulting Services</t>
+        </is>
+      </c>
+      <c r="B377" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C377" s="3" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="D377" s="3" t="inlineStr">
+        <is>
+          <t>https://www.hosp.med.osaka-u.ac.jp/english/inquiry/counter.html</t>
+        </is>
+      </c>
+      <c r="E377" s="3" t="inlineStr"/>
+      <c r="F377" s="3" t="inlineStr">
+        <is>
+          <t>06-6879-5111</t>
+        </is>
+      </c>
+      <c r="G377" s="3" t="inlineStr"/>
+      <c r="H377" s="3" t="inlineStr"/>
+      <c r="I377" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J377" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:19</t>
+        </is>
+      </c>
+      <c r="K377" s="3" t="inlineStr"/>
+      <c r="L377" s="3" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M377" s="3" t="inlineStr"/>
+      <c r="N377" s="3" t="inlineStr"/>
+    </row>
+    <row r="378">
+      <c r="A378" s="3" t="inlineStr">
+        <is>
+          <t>City of Osaka : When You Are Ill - 大阪市</t>
+        </is>
+      </c>
+      <c r="B378" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C378" s="3" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="D378" s="3" t="inlineStr">
+        <is>
+          <t>https://www.city.osaka.lg.jp/contents/wdu020/enjoy/en/content_i.html</t>
+        </is>
+      </c>
+      <c r="E378" s="3" t="inlineStr"/>
+      <c r="F378" s="3" t="inlineStr">
+        <is>
+          <t>0000549405</t>
+        </is>
+      </c>
+      <c r="G378" s="3" t="inlineStr"/>
+      <c r="H378" s="3" t="inlineStr"/>
+      <c r="I378" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J378" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:19</t>
+        </is>
+      </c>
+      <c r="K378" s="3" t="inlineStr"/>
+      <c r="L378" s="3" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M378" s="3" t="inlineStr"/>
+      <c r="N378" s="3" t="inlineStr"/>
+    </row>
+    <row r="379">
+      <c r="A379" s="3" t="inlineStr">
+        <is>
+          <t>Osaka Women's and Children's Hospital</t>
+        </is>
+      </c>
+      <c r="B379" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C379" s="3" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="D379" s="3" t="inlineStr">
+        <is>
+          <t>https://www.wch.opho.jp/english/hospital</t>
+        </is>
+      </c>
+      <c r="E379" s="3" t="inlineStr"/>
+      <c r="F379" s="3" t="inlineStr">
+        <is>
+          <t>+81-725-56-1220</t>
+        </is>
+      </c>
+      <c r="G379" s="3" t="inlineStr"/>
+      <c r="H379" s="3" t="inlineStr"/>
+      <c r="I379" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J379" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:19</t>
+        </is>
+      </c>
+      <c r="K379" s="3" t="inlineStr"/>
+      <c r="L379" s="3" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M379" s="3" t="inlineStr"/>
+      <c r="N379" s="3" t="inlineStr"/>
+    </row>
+    <row r="380">
+      <c r="A380" s="3" t="inlineStr">
+        <is>
+          <t>English-Speaking Hospitals in Osaka</t>
+        </is>
+      </c>
+      <c r="B380" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C380" s="3" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="D380" s="3" t="inlineStr">
+        <is>
+          <t>https://www.japanlivingguide.com/expatinfo/healthcaresystem/hospitals-in-osaka/</t>
+        </is>
+      </c>
+      <c r="E380" s="3" t="inlineStr"/>
+      <c r="F380" s="3" t="inlineStr">
+        <is>
+          <t>03-3583-6941</t>
+        </is>
+      </c>
+      <c r="G380" s="3" t="inlineStr"/>
+      <c r="H380" s="3" t="inlineStr"/>
+      <c r="I380" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J380" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:20</t>
+        </is>
+      </c>
+      <c r="K380" s="3" t="inlineStr"/>
+      <c r="L380" s="3" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M380" s="3" t="inlineStr"/>
+      <c r="N380" s="3" t="inlineStr"/>
+    </row>
+    <row r="381">
+      <c r="A381" s="2" t="inlineStr">
+        <is>
+          <t>Sumitomo Hospital</t>
+        </is>
+      </c>
+      <c r="B381" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C381" s="2" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="D381" s="2" t="inlineStr">
+        <is>
+          <t>https://www.myhospitalnow.com/hospitals/sumitomo-hospital</t>
+        </is>
+      </c>
+      <c r="E381" s="2" t="inlineStr">
+        <is>
+          <t>contact@myhospitalnow.com</t>
+        </is>
+      </c>
+      <c r="F381" s="2" t="inlineStr">
+        <is>
+          <t>664431261</t>
+        </is>
+      </c>
+      <c r="G381" s="2" t="inlineStr"/>
+      <c r="H381" s="2" t="inlineStr">
+        <is>
+          <t>A digital system that could save Sumitomo Hospital hours every week</t>
+        </is>
+      </c>
+      <c r="I381" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J381" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:20</t>
+        </is>
+      </c>
+      <c r="K381" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T13:27:25.164018</t>
+        </is>
+      </c>
+      <c r="L381" s="2" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M381" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="N381" s="2" t="inlineStr"/>
+    </row>
+    <row r="382">
+      <c r="A382" s="2" t="inlineStr">
+        <is>
+          <t>Hospitals in Japan</t>
+        </is>
+      </c>
+      <c r="B382" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C382" s="2" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="D382" s="2" t="inlineStr">
+        <is>
+          <t>https://www.internationalinsurance.com/countries/japan/hospitals/?srsltid=AfmBOooEciibu0MzXarxTvPwUR7AGXR5eiLT2CveqfBw8plYwUEeVn7C</t>
+        </is>
+      </c>
+      <c r="E382" s="2" t="inlineStr">
+        <is>
+          <t>info@internationalinsurance.com</t>
+        </is>
+      </c>
+      <c r="F382" s="2" t="inlineStr">
+        <is>
+          <t>+1 617 500 6738</t>
+        </is>
+      </c>
+      <c r="G382" s="2" t="inlineStr"/>
+      <c r="H382" s="2" t="inlineStr">
+        <is>
+          <t>A digital system that could save Hospitals in Japan hours every week</t>
+        </is>
+      </c>
+      <c r="I382" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J382" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:28</t>
+        </is>
+      </c>
+      <c r="K382" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T13:35:11.487615</t>
+        </is>
+      </c>
+      <c r="L382" s="2" t="inlineStr">
+        <is>
+          <t>google_p3</t>
+        </is>
+      </c>
+      <c r="M382" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="N382" s="2" t="inlineStr"/>
+    </row>
+    <row r="383">
+      <c r="A383" s="3" t="inlineStr">
+        <is>
+          <t>ALL JAPAN HOSPITAL ASSOCIATION</t>
+        </is>
+      </c>
+      <c r="B383" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C383" s="3" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="D383" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ajha.or.jp/eng/index.pdf</t>
+        </is>
+      </c>
+      <c r="E383" s="3" t="inlineStr"/>
+      <c r="F383" s="3" t="inlineStr">
+        <is>
+          <t>2009-04-14</t>
+        </is>
+      </c>
+      <c r="G383" s="3" t="inlineStr"/>
+      <c r="H383" s="3" t="inlineStr"/>
+      <c r="I383" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J383" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:35</t>
+        </is>
+      </c>
+      <c r="K383" s="3" t="inlineStr"/>
+      <c r="L383" s="3" t="inlineStr">
+        <is>
+          <t>google_p3</t>
+        </is>
+      </c>
+      <c r="M383" s="3" t="inlineStr"/>
+      <c r="N383" s="3" t="inlineStr"/>
+    </row>
+    <row r="384">
+      <c r="A384" s="3" t="inlineStr">
+        <is>
+          <t>NHO Osaka National Hospital - Overview, News &amp; Similar ...</t>
+        </is>
+      </c>
+      <c r="B384" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C384" s="3" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="D384" s="3" t="inlineStr">
+        <is>
+          <t>https://www.zoominfo.com/c/national-hospital-organization-osaka-national-hospital/1338580265</t>
+        </is>
+      </c>
+      <c r="E384" s="3" t="inlineStr"/>
+      <c r="F384" s="3" t="inlineStr">
+        <is>
+          <t>+1 866-904-9666</t>
+        </is>
+      </c>
+      <c r="G384" s="3" t="inlineStr"/>
+      <c r="H384" s="3" t="inlineStr"/>
+      <c r="I384" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J384" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:37</t>
+        </is>
+      </c>
+      <c r="K384" s="3" t="inlineStr"/>
+      <c r="L384" s="3" t="inlineStr">
+        <is>
+          <t>google_p3</t>
+        </is>
+      </c>
+      <c r="M384" s="3" t="inlineStr"/>
+      <c r="N384" s="3" t="inlineStr"/>
+    </row>
+    <row r="385">
+      <c r="A385" s="3" t="inlineStr">
+        <is>
+          <t>Sakai Heisei Hospital - Japan Travel by NAVITIME</t>
+        </is>
+      </c>
+      <c r="B385" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C385" s="3" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="D385" s="3" t="inlineStr">
+        <is>
+          <t>https://japantravel.navitime.com/en/area/jp/spot/01127-00001083609/</t>
+        </is>
+      </c>
+      <c r="E385" s="3" t="inlineStr"/>
+      <c r="F385" s="3" t="inlineStr">
+        <is>
+          <t>0722782461</t>
+        </is>
+      </c>
+      <c r="G385" s="3" t="inlineStr"/>
+      <c r="H385" s="3" t="inlineStr"/>
+      <c r="I385" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J385" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:37</t>
+        </is>
+      </c>
+      <c r="K385" s="3" t="inlineStr"/>
+      <c r="L385" s="3" t="inlineStr">
+        <is>
+          <t>google_p3</t>
+        </is>
+      </c>
+      <c r="M385" s="3" t="inlineStr"/>
+      <c r="N385" s="3" t="inlineStr"/>
+    </row>
+    <row r="386">
+      <c r="A386" s="2" t="inlineStr">
+        <is>
+          <t>Hospital Overview | Osaka Red Cross Hospital</t>
+        </is>
+      </c>
+      <c r="B386" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C386" s="2" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="D386" s="2" t="inlineStr">
+        <is>
+          <t>https://www.osaka-med.jrc.or.jp/english/overview/index.html</t>
+        </is>
+      </c>
+      <c r="E386" s="2" t="inlineStr">
+        <is>
+          <t>hospital@osaka-med.jrc.or.jp</t>
+        </is>
+      </c>
+      <c r="F386" s="2" t="inlineStr">
+        <is>
+          <t>06-6774-5111</t>
+        </is>
+      </c>
+      <c r="G386" s="2" t="inlineStr">
+        <is>
+          <t>Director 
+ Yoshiharu Sakai</t>
+        </is>
+      </c>
+      <c r="H386" s="2" t="inlineStr">
+        <is>
+          <t>Streamline Operations: Custom Digital Solution Proposal</t>
+        </is>
+      </c>
+      <c r="I386" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J386" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:38</t>
+        </is>
+      </c>
+      <c r="K386" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T13:41:43.001158</t>
+        </is>
+      </c>
+      <c r="L386" s="2" t="inlineStr">
+        <is>
+          <t>google_p3</t>
+        </is>
+      </c>
+      <c r="M386" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N386" s="2" t="inlineStr"/>
+    </row>
+    <row r="387">
+      <c r="A387" s="3" t="inlineStr">
+        <is>
+          <t>NCT05321082 | A Study to Find Out Whether BI 1015550 ...</t>
+        </is>
+      </c>
+      <c r="B387" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C387" s="3" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="D387" s="3" t="inlineStr">
+        <is>
+          <t>https://clinicaltrials.gov/study/NCT05321082</t>
+        </is>
+      </c>
+      <c r="E387" s="3" t="inlineStr"/>
+      <c r="F387" s="3" t="inlineStr"/>
+      <c r="G387" s="3" t="inlineStr"/>
+      <c r="H387" s="3" t="inlineStr"/>
+      <c r="I387" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J387" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:42</t>
+        </is>
+      </c>
+      <c r="K387" s="3" t="inlineStr"/>
+      <c r="L387" s="3" t="inlineStr">
+        <is>
+          <t>google_p4</t>
+        </is>
+      </c>
+      <c r="M387" s="3" t="inlineStr"/>
+      <c r="N387" s="3" t="inlineStr"/>
+    </row>
+    <row r="388">
+      <c r="A388" s="3" t="inlineStr">
+        <is>
+          <t>Healthcare in Japan: A guide to the Japanese ...</t>
+        </is>
+      </c>
+      <c r="B388" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C388" s="3" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="D388" s="3" t="inlineStr">
+        <is>
+          <t>https://wise.com/us/blog/healthcare-system-in-japan</t>
+        </is>
+      </c>
+      <c r="E388" s="3" t="inlineStr"/>
+      <c r="F388" s="3" t="inlineStr"/>
+      <c r="G388" s="3" t="inlineStr"/>
+      <c r="H388" s="3" t="inlineStr"/>
+      <c r="I388" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J388" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:42</t>
+        </is>
+      </c>
+      <c r="K388" s="3" t="inlineStr"/>
+      <c r="L388" s="3" t="inlineStr">
+        <is>
+          <t>google_p4</t>
+        </is>
+      </c>
+      <c r="M388" s="3" t="inlineStr"/>
+      <c r="N388" s="3" t="inlineStr"/>
+    </row>
+    <row r="389">
+      <c r="A389" s="3" t="inlineStr">
+        <is>
+          <t>About us | Osaka City Juso Hospital</t>
+        </is>
+      </c>
+      <c r="B389" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C389" s="3" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="D389" s="3" t="inlineStr">
+        <is>
+          <t>https://www.osakacity-hp.or.jp/juso/en/about.html</t>
+        </is>
+      </c>
+      <c r="E389" s="3" t="inlineStr"/>
+      <c r="F389" s="3" t="inlineStr">
+        <is>
+          <t>06-6150-8000</t>
+        </is>
+      </c>
+      <c r="G389" s="3" t="inlineStr"/>
+      <c r="H389" s="3" t="inlineStr"/>
+      <c r="I389" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J389" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:43</t>
+        </is>
+      </c>
+      <c r="K389" s="3" t="inlineStr"/>
+      <c r="L389" s="3" t="inlineStr">
+        <is>
+          <t>google_p4</t>
+        </is>
+      </c>
+      <c r="M389" s="3" t="inlineStr"/>
+      <c r="N389" s="3" t="inlineStr"/>
+    </row>
+    <row r="390">
+      <c r="A390" s="3" t="inlineStr">
+        <is>
+          <t>Find JCI-accredited organizations</t>
+        </is>
+      </c>
+      <c r="B390" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C390" s="3" t="inlineStr">
+        <is>
+          <t>Osaka</t>
+        </is>
+      </c>
+      <c r="D390" s="3" t="inlineStr">
+        <is>
+          <t>https://www.jointcommission.org/en/about-us/recognizing-excellence/find-accredited-international-organizations</t>
+        </is>
+      </c>
+      <c r="E390" s="3" t="inlineStr"/>
+      <c r="F390" s="3" t="inlineStr"/>
+      <c r="G390" s="3" t="inlineStr"/>
+      <c r="H390" s="3" t="inlineStr"/>
+      <c r="I390" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J390" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:43</t>
+        </is>
+      </c>
+      <c r="K390" s="3" t="inlineStr"/>
+      <c r="L390" s="3" t="inlineStr">
+        <is>
+          <t>google_p4</t>
+        </is>
+      </c>
+      <c r="M390" s="3" t="inlineStr"/>
+      <c r="N390" s="3" t="inlineStr"/>
+    </row>
+    <row r="391">
+      <c r="A391" s="3" t="inlineStr">
+        <is>
+          <t>Welcome To The Sydney Private Hospital - The Sydney ...</t>
+        </is>
+      </c>
+      <c r="B391" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C391" s="3" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D391" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sydneyprivate.com.au/</t>
+        </is>
+      </c>
+      <c r="E391" s="3" t="inlineStr"/>
+      <c r="F391" s="3" t="inlineStr">
+        <is>
+          <t>02) 9797 0555</t>
+        </is>
+      </c>
+      <c r="G391" s="3" t="inlineStr"/>
+      <c r="H391" s="3" t="inlineStr"/>
+      <c r="I391" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J391" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:43</t>
+        </is>
+      </c>
+      <c r="K391" s="3" t="inlineStr"/>
+      <c r="L391" s="3" t="inlineStr">
+        <is>
+          <t>google_p1</t>
+        </is>
+      </c>
+      <c r="M391" s="3" t="inlineStr"/>
+      <c r="N391" s="3" t="inlineStr"/>
+    </row>
+    <row r="392">
+      <c r="A392" s="2" t="inlineStr">
+        <is>
+          <t>East Sydney Private Hospital - Home</t>
+        </is>
+      </c>
+      <c r="B392" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C392" s="2" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D392" s="2" t="inlineStr">
+        <is>
+          <t>https://www.eastsydneyprivatehospital.com/</t>
+        </is>
+      </c>
+      <c r="E392" s="2" t="inlineStr">
+        <is>
+          <t>Credentialing@esphospital.com</t>
+        </is>
+      </c>
+      <c r="F392" s="2" t="inlineStr">
+        <is>
+          <t>02)  9001 2000</t>
+        </is>
+      </c>
+      <c r="G392" s="2" t="inlineStr"/>
+      <c r="H392" s="2" t="inlineStr">
+        <is>
+          <t>Streamline Operations: Custom Digital Solution Proposal</t>
+        </is>
+      </c>
+      <c r="I392" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J392" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:43</t>
+        </is>
+      </c>
+      <c r="K392" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T13:51:10.041085</t>
+        </is>
+      </c>
+      <c r="L392" s="2" t="inlineStr">
+        <is>
+          <t>google_p1</t>
+        </is>
+      </c>
+      <c r="M392" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N392" s="2" t="inlineStr"/>
+    </row>
+    <row r="393">
+      <c r="A393" s="3" t="inlineStr">
+        <is>
+          <t>Sydney Southwest Private Hospital: Home</t>
+        </is>
+      </c>
+      <c r="B393" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C393" s="3" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D393" s="3" t="inlineStr">
+        <is>
+          <t>https://sydneysouthwestprivatehospital.com.au/</t>
+        </is>
+      </c>
+      <c r="E393" s="3" t="inlineStr"/>
+      <c r="F393" s="3" t="inlineStr">
+        <is>
+          <t>02 9600 4000</t>
+        </is>
+      </c>
+      <c r="G393" s="3" t="inlineStr">
+        <is>
+          <t>Head Neck Surgery</t>
+        </is>
+      </c>
+      <c r="H393" s="3" t="inlineStr"/>
+      <c r="I393" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J393" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:52</t>
+        </is>
+      </c>
+      <c r="K393" s="3" t="inlineStr"/>
+      <c r="L393" s="3" t="inlineStr">
+        <is>
+          <t>google_p1</t>
+        </is>
+      </c>
+      <c r="M393" s="3" t="inlineStr"/>
+      <c r="N393" s="3" t="inlineStr"/>
+    </row>
+    <row r="394">
+      <c r="A394" s="3" t="inlineStr">
+        <is>
+          <t>St Vincent's Private Hospital, Sydney</t>
+        </is>
+      </c>
+      <c r="B394" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C394" s="3" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D394" s="3" t="inlineStr">
+        <is>
+          <t>https://www.svph.org.au/hospitals/sydney</t>
+        </is>
+      </c>
+      <c r="E394" s="3" t="inlineStr"/>
+      <c r="F394" s="3" t="inlineStr"/>
+      <c r="G394" s="3" t="inlineStr"/>
+      <c r="H394" s="3" t="inlineStr"/>
+      <c r="I394" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J394" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:52</t>
+        </is>
+      </c>
+      <c r="K394" s="3" t="inlineStr"/>
+      <c r="L394" s="3" t="inlineStr">
+        <is>
+          <t>google_p1</t>
+        </is>
+      </c>
+      <c r="M394" s="3" t="inlineStr"/>
+      <c r="N394" s="3" t="inlineStr"/>
+    </row>
+    <row r="395">
+      <c r="A395" s="3" t="inlineStr">
+        <is>
+          <t>Welcome to Strathfield Private Hospital</t>
+        </is>
+      </c>
+      <c r="B395" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C395" s="3" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D395" s="3" t="inlineStr">
+        <is>
+          <t>https://www.strathfieldprivate.com.au/</t>
+        </is>
+      </c>
+      <c r="E395" s="3" t="inlineStr"/>
+      <c r="F395" s="3" t="inlineStr">
+        <is>
+          <t>02 9745 7444</t>
+        </is>
+      </c>
+      <c r="G395" s="3" t="inlineStr"/>
+      <c r="H395" s="3" t="inlineStr"/>
+      <c r="I395" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J395" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:52</t>
+        </is>
+      </c>
+      <c r="K395" s="3" t="inlineStr"/>
+      <c r="L395" s="3" t="inlineStr">
+        <is>
+          <t>google_p1</t>
+        </is>
+      </c>
+      <c r="M395" s="3" t="inlineStr"/>
+      <c r="N395" s="3" t="inlineStr"/>
+    </row>
+    <row r="396">
+      <c r="A396" s="3" t="inlineStr">
+        <is>
+          <t>Welcome to Westmead Private Hospital</t>
+        </is>
+      </c>
+      <c r="B396" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C396" s="3" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D396" s="3" t="inlineStr">
+        <is>
+          <t>https://www.westmeadprivate.com.au/</t>
+        </is>
+      </c>
+      <c r="E396" s="3" t="inlineStr"/>
+      <c r="F396" s="3" t="inlineStr">
+        <is>
+          <t>02 8837 9000</t>
+        </is>
+      </c>
+      <c r="G396" s="3" t="inlineStr"/>
+      <c r="H396" s="3" t="inlineStr"/>
+      <c r="I396" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J396" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:53</t>
+        </is>
+      </c>
+      <c r="K396" s="3" t="inlineStr"/>
+      <c r="L396" s="3" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M396" s="3" t="inlineStr"/>
+      <c r="N396" s="3" t="inlineStr"/>
+    </row>
+    <row r="397">
+      <c r="A397" s="3" t="inlineStr">
+        <is>
+          <t>Sydney Adventist Hospital "The San" - Sydney north shore ...</t>
+        </is>
+      </c>
+      <c r="B397" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C397" s="3" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D397" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sah.org.au/</t>
+        </is>
+      </c>
+      <c r="E397" s="3" t="inlineStr"/>
+      <c r="F397" s="3" t="inlineStr"/>
+      <c r="G397" s="3" t="inlineStr"/>
+      <c r="H397" s="3" t="inlineStr"/>
+      <c r="I397" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J397" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:53</t>
+        </is>
+      </c>
+      <c r="K397" s="3" t="inlineStr"/>
+      <c r="L397" s="3" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M397" s="3" t="inlineStr"/>
+      <c r="N397" s="3" t="inlineStr"/>
+    </row>
+    <row r="398">
+      <c r="A398" s="3" t="inlineStr">
+        <is>
+          <t>Welcome to North Shore Private Hospital</t>
+        </is>
+      </c>
+      <c r="B398" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C398" s="3" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D398" s="3" t="inlineStr">
+        <is>
+          <t>https://www.northshoreprivate.com.au/</t>
+        </is>
+      </c>
+      <c r="E398" s="3" t="inlineStr"/>
+      <c r="F398" s="3" t="inlineStr">
+        <is>
+          <t>02 8425 3000</t>
+        </is>
+      </c>
+      <c r="G398" s="3" t="inlineStr"/>
+      <c r="H398" s="3" t="inlineStr"/>
+      <c r="I398" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J398" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:53</t>
+        </is>
+      </c>
+      <c r="K398" s="3" t="inlineStr"/>
+      <c r="L398" s="3" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M398" s="3" t="inlineStr"/>
+      <c r="N398" s="3" t="inlineStr"/>
+    </row>
+    <row r="399">
+      <c r="A399" s="3" t="inlineStr">
+        <is>
+          <t>Ramsay Health Care: People Caring for People</t>
+        </is>
+      </c>
+      <c r="B399" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C399" s="3" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D399" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ramsayhealth.com.au/</t>
+        </is>
+      </c>
+      <c r="E399" s="3" t="inlineStr"/>
+      <c r="F399" s="3" t="inlineStr"/>
+      <c r="G399" s="3" t="inlineStr"/>
+      <c r="H399" s="3" t="inlineStr"/>
+      <c r="I399" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J399" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:54</t>
+        </is>
+      </c>
+      <c r="K399" s="3" t="inlineStr"/>
+      <c r="L399" s="3" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M399" s="3" t="inlineStr"/>
+      <c r="N399" s="3" t="inlineStr"/>
+    </row>
+    <row r="400">
+      <c r="A400" s="3" t="inlineStr">
+        <is>
+          <t>Contact Us - The Sydney Private Hospital Surgical ...</t>
+        </is>
+      </c>
+      <c r="B400" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C400" s="3" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D400" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sydneyprivate.com.au/the-sydney-private-hospital/</t>
+        </is>
+      </c>
+      <c r="E400" s="3" t="inlineStr"/>
+      <c r="F400" s="3" t="inlineStr">
+        <is>
+          <t>02) 8775 1100</t>
+        </is>
+      </c>
+      <c r="G400" s="3" t="inlineStr"/>
+      <c r="H400" s="3" t="inlineStr"/>
+      <c r="I400" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J400" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:54</t>
+        </is>
+      </c>
+      <c r="K400" s="3" t="inlineStr"/>
+      <c r="L400" s="3" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M400" s="3" t="inlineStr"/>
+      <c r="N400" s="3" t="inlineStr"/>
+    </row>
+    <row r="401">
+      <c r="A401" s="3" t="inlineStr">
+        <is>
+          <t>Lakeview Private Hospital: Private Hospital Norwest Sydney</t>
+        </is>
+      </c>
+      <c r="B401" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C401" s="3" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D401" s="3" t="inlineStr">
+        <is>
+          <t>https://lakeviewprivate.com.au/</t>
+        </is>
+      </c>
+      <c r="E401" s="3" t="inlineStr"/>
+      <c r="F401" s="3" t="inlineStr">
+        <is>
+          <t>02 8624 5000</t>
+        </is>
+      </c>
+      <c r="G401" s="3" t="inlineStr"/>
+      <c r="H401" s="3" t="inlineStr"/>
+      <c r="I401" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J401" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:54</t>
+        </is>
+      </c>
+      <c r="K401" s="3" t="inlineStr"/>
+      <c r="L401" s="3" t="inlineStr">
+        <is>
+          <t>google_p3</t>
+        </is>
+      </c>
+      <c r="M401" s="3" t="inlineStr"/>
+      <c r="N401" s="3" t="inlineStr"/>
+    </row>
+    <row r="402">
+      <c r="A402" s="3" t="inlineStr">
+        <is>
+          <t>Prince of Wales Private Hospital</t>
+        </is>
+      </c>
+      <c r="B402" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C402" s="3" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D402" s="3" t="inlineStr">
+        <is>
+          <t>https://princeofwalesprivatehospital.com.au/</t>
+        </is>
+      </c>
+      <c r="E402" s="3" t="inlineStr"/>
+      <c r="F402" s="3" t="inlineStr">
+        <is>
+          <t>02 9650 4000</t>
+        </is>
+      </c>
+      <c r="G402" s="3" t="inlineStr"/>
+      <c r="H402" s="3" t="inlineStr"/>
+      <c r="I402" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J402" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:55</t>
+        </is>
+      </c>
+      <c r="K402" s="3" t="inlineStr"/>
+      <c r="L402" s="3" t="inlineStr">
+        <is>
+          <t>google_p3</t>
+        </is>
+      </c>
+      <c r="M402" s="3" t="inlineStr"/>
+      <c r="N402" s="3" t="inlineStr"/>
+    </row>
+    <row r="403">
+      <c r="A403" s="3" t="inlineStr">
+        <is>
+          <t>Somerset Private Hospital</t>
+        </is>
+      </c>
+      <c r="B403" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C403" s="3" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D403" s="3" t="inlineStr">
+        <is>
+          <t>https://curagroup.com.au/hospital/somerset-private-hospital/</t>
+        </is>
+      </c>
+      <c r="E403" s="3" t="inlineStr"/>
+      <c r="F403" s="3" t="inlineStr"/>
+      <c r="G403" s="3" t="inlineStr"/>
+      <c r="H403" s="3" t="inlineStr"/>
+      <c r="I403" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J403" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:56</t>
+        </is>
+      </c>
+      <c r="K403" s="3" t="inlineStr"/>
+      <c r="L403" s="3" t="inlineStr">
+        <is>
+          <t>google_p3</t>
+        </is>
+      </c>
+      <c r="M403" s="3" t="inlineStr"/>
+      <c r="N403" s="3" t="inlineStr"/>
+    </row>
+    <row r="404">
+      <c r="A404" s="3" t="inlineStr">
+        <is>
+          <t>Waratah Private Hospital – A Healthe Care hospital</t>
+        </is>
+      </c>
+      <c r="B404" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C404" s="3" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D404" s="3" t="inlineStr">
+        <is>
+          <t>https://waratahprivate.com.au/</t>
+        </is>
+      </c>
+      <c r="E404" s="3" t="inlineStr"/>
+      <c r="F404" s="3" t="inlineStr">
+        <is>
+          <t>+61 2 9598 0000</t>
+        </is>
+      </c>
+      <c r="G404" s="3" t="inlineStr"/>
+      <c r="H404" s="3" t="inlineStr"/>
+      <c r="I404" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J404" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:56</t>
+        </is>
+      </c>
+      <c r="K404" s="3" t="inlineStr"/>
+      <c r="L404" s="3" t="inlineStr">
+        <is>
+          <t>google_p3</t>
+        </is>
+      </c>
+      <c r="M404" s="3" t="inlineStr"/>
+      <c r="N404" s="3" t="inlineStr"/>
+    </row>
+    <row r="405">
+      <c r="A405" s="3" t="inlineStr">
+        <is>
+          <t>Nepean Private Hospital – Nepean Private Maternity ...</t>
+        </is>
+      </c>
+      <c r="B405" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C405" s="3" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D405" s="3" t="inlineStr">
+        <is>
+          <t>https://nepeanprivatehospital.com.au/</t>
+        </is>
+      </c>
+      <c r="E405" s="3" t="inlineStr"/>
+      <c r="F405" s="3" t="inlineStr">
+        <is>
+          <t>02 4732 7333</t>
+        </is>
+      </c>
+      <c r="G405" s="3" t="inlineStr"/>
+      <c r="H405" s="3" t="inlineStr"/>
+      <c r="I405" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J405" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:57</t>
+        </is>
+      </c>
+      <c r="K405" s="3" t="inlineStr"/>
+      <c r="L405" s="3" t="inlineStr">
+        <is>
+          <t>google_p3</t>
+        </is>
+      </c>
+      <c r="M405" s="3" t="inlineStr"/>
+      <c r="N405" s="3" t="inlineStr"/>
+    </row>
+    <row r="406">
+      <c r="A406" s="3" t="inlineStr">
+        <is>
+          <t>Longueville Private Rehabilitation and Medical Hospital ...</t>
+        </is>
+      </c>
+      <c r="B406" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C406" s="3" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D406" s="3" t="inlineStr">
+        <is>
+          <t>https://www.longuevilleprivate.com.au/</t>
+        </is>
+      </c>
+      <c r="E406" s="3" t="inlineStr"/>
+      <c r="F406" s="3" t="inlineStr">
+        <is>
+          <t>02) 9427 0844</t>
+        </is>
+      </c>
+      <c r="G406" s="3" t="inlineStr"/>
+      <c r="H406" s="3" t="inlineStr"/>
+      <c r="I406" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J406" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:57</t>
+        </is>
+      </c>
+      <c r="K406" s="3" t="inlineStr"/>
+      <c r="L406" s="3" t="inlineStr">
+        <is>
+          <t>google_p4</t>
+        </is>
+      </c>
+      <c r="M406" s="3" t="inlineStr"/>
+      <c r="N406" s="3" t="inlineStr"/>
+    </row>
+    <row r="407">
+      <c r="A407" s="3" t="inlineStr">
+        <is>
+          <t>St John of God Health Care</t>
+        </is>
+      </c>
+      <c r="B407" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C407" s="3" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D407" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sjog.org.au/</t>
+        </is>
+      </c>
+      <c r="E407" s="3" t="inlineStr"/>
+      <c r="F407" s="3" t="inlineStr">
+        <is>
+          <t>1300 863 566</t>
+        </is>
+      </c>
+      <c r="G407" s="3" t="inlineStr">
+        <is>
+          <t>Dr David Borshoff</t>
+        </is>
+      </c>
+      <c r="H407" s="3" t="inlineStr"/>
+      <c r="I407" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J407" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:58</t>
+        </is>
+      </c>
+      <c r="K407" s="3" t="inlineStr"/>
+      <c r="L407" s="3" t="inlineStr">
+        <is>
+          <t>google_p4</t>
+        </is>
+      </c>
+      <c r="M407" s="3" t="inlineStr"/>
+      <c r="N407" s="3" t="inlineStr"/>
+    </row>
+    <row r="408">
+      <c r="A408" s="3" t="inlineStr">
+        <is>
+          <t>Homepage — Forster Private Hospital</t>
+        </is>
+      </c>
+      <c r="B408" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C408" s="3" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D408" s="3" t="inlineStr">
+        <is>
+          <t>https://forsterprivate.com.au/</t>
+        </is>
+      </c>
+      <c r="E408" s="3" t="inlineStr"/>
+      <c r="F408" s="3" t="inlineStr">
+        <is>
+          <t>02 6555 1333</t>
+        </is>
+      </c>
+      <c r="G408" s="3" t="inlineStr"/>
+      <c r="H408" s="3" t="inlineStr"/>
+      <c r="I408" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J408" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:58</t>
+        </is>
+      </c>
+      <c r="K408" s="3" t="inlineStr"/>
+      <c r="L408" s="3" t="inlineStr">
+        <is>
+          <t>google_p4</t>
+        </is>
+      </c>
+      <c r="M408" s="3" t="inlineStr"/>
+      <c r="N408" s="3" t="inlineStr"/>
+    </row>
+    <row r="409">
+      <c r="A409" s="2" t="inlineStr">
+        <is>
+          <t>Evolution Healthcare: Home</t>
+        </is>
+      </c>
+      <c r="B409" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C409" s="2" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D409" s="2" t="inlineStr">
+        <is>
+          <t>https://evolutioncare.com/</t>
+        </is>
+      </c>
+      <c r="E409" s="2" t="inlineStr">
+        <is>
+          <t>enquiries@evolutioncare.com</t>
+        </is>
+      </c>
+      <c r="F409" s="2" t="inlineStr">
+        <is>
+          <t>+64 4 381 8100</t>
+        </is>
+      </c>
+      <c r="G409" s="2" t="inlineStr">
+        <is>
+          <t>Mr Rodney Studd</t>
+        </is>
+      </c>
+      <c r="H409" s="2" t="inlineStr">
+        <is>
+          <t>A digital system that could save Evolution Healthcare: Home hours every week</t>
+        </is>
+      </c>
+      <c r="I409" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J409" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 13:59</t>
+        </is>
+      </c>
+      <c r="K409" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T14:06:05.621167</t>
+        </is>
+      </c>
+      <c r="L409" s="2" t="inlineStr">
+        <is>
+          <t>google_p4</t>
+        </is>
+      </c>
+      <c r="M409" s="2" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="N409" s="2" t="inlineStr"/>
+    </row>
+    <row r="410">
+      <c r="A410" s="2" t="inlineStr">
+        <is>
+          <t>Contact Us</t>
+        </is>
+      </c>
+      <c r="B410" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C410" s="2" t="inlineStr">
+        <is>
+          <t>Sydney</t>
+        </is>
+      </c>
+      <c r="D410" s="2" t="inlineStr">
+        <is>
+          <t>https://www.eastsydneyprivatehospital.com/contact-us/</t>
+        </is>
+      </c>
+      <c r="E410" s="2" t="inlineStr">
+        <is>
+          <t>Credentialing@esphospital.com</t>
+        </is>
+      </c>
+      <c r="F410" s="2" t="inlineStr">
+        <is>
+          <t>02)  9001 2000</t>
+        </is>
+      </c>
+      <c r="G410" s="2" t="inlineStr"/>
+      <c r="H410" s="2" t="inlineStr">
+        <is>
+          <t>Streamline Hospital Operations with Custom Digital Solution</t>
+        </is>
+      </c>
+      <c r="I410" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J410" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 14:06</t>
+        </is>
+      </c>
+      <c r="K410" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T14:11:45.561192</t>
+        </is>
+      </c>
+      <c r="L410" s="2" t="inlineStr">
+        <is>
+          <t>google_p4</t>
+        </is>
+      </c>
+      <c r="M410" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N410" s="2" t="inlineStr"/>
+    </row>
+    <row r="411">
+      <c r="A411" s="3" t="inlineStr">
+        <is>
+          <t>Melbourne Private Hospital: Home</t>
+        </is>
+      </c>
+      <c r="B411" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C411" s="3" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="D411" s="3" t="inlineStr">
+        <is>
+          <t>https://melbourneprivatehospital.com.au/</t>
+        </is>
+      </c>
+      <c r="E411" s="3" t="inlineStr"/>
+      <c r="F411" s="3" t="inlineStr">
+        <is>
+          <t>03 8341 3400</t>
+        </is>
+      </c>
+      <c r="G411" s="3" t="inlineStr"/>
+      <c r="H411" s="3" t="inlineStr"/>
+      <c r="I411" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J411" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 14:12</t>
+        </is>
+      </c>
+      <c r="K411" s="3" t="inlineStr"/>
+      <c r="L411" s="3" t="inlineStr">
+        <is>
+          <t>google_p1</t>
+        </is>
+      </c>
+      <c r="M411" s="3" t="inlineStr"/>
+      <c r="N411" s="3" t="inlineStr"/>
+    </row>
+    <row r="412">
+      <c r="A412" s="3" t="inlineStr">
+        <is>
+          <t>General Information :: Melbourne Private Hospital</t>
+        </is>
+      </c>
+      <c r="B412" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C412" s="3" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="D412" s="3" t="inlineStr">
+        <is>
+          <t>https://melbourneprivatehospital.com.au/patients/general-information</t>
+        </is>
+      </c>
+      <c r="E412" s="3" t="inlineStr"/>
+      <c r="F412" s="3" t="inlineStr">
+        <is>
+          <t>03 8341 3400</t>
+        </is>
+      </c>
+      <c r="G412" s="3" t="inlineStr"/>
+      <c r="H412" s="3" t="inlineStr"/>
+      <c r="I412" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J412" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 14:13</t>
+        </is>
+      </c>
+      <c r="K412" s="3" t="inlineStr"/>
+      <c r="L412" s="3" t="inlineStr">
+        <is>
+          <t>google_p1</t>
+        </is>
+      </c>
+      <c r="M412" s="3" t="inlineStr"/>
+      <c r="N412" s="3" t="inlineStr"/>
+    </row>
+    <row r="413">
+      <c r="A413" s="3" t="inlineStr">
+        <is>
+          <t>St Vincent's Hospital Melbourne: Welcome To St Vincent's ...</t>
+        </is>
+      </c>
+      <c r="B413" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C413" s="3" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="D413" s="3" t="inlineStr">
+        <is>
+          <t>https://www.svhm.org.au/</t>
+        </is>
+      </c>
+      <c r="E413" s="3" t="inlineStr"/>
+      <c r="F413" s="3" t="inlineStr">
+        <is>
+          <t>03 9231 2211</t>
+        </is>
+      </c>
+      <c r="G413" s="3" t="inlineStr">
+        <is>
+          <t>CEO 
+ Hello</t>
+        </is>
+      </c>
+      <c r="H413" s="3" t="inlineStr"/>
+      <c r="I413" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J413" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 14:13</t>
+        </is>
+      </c>
+      <c r="K413" s="3" t="inlineStr"/>
+      <c r="L413" s="3" t="inlineStr">
+        <is>
+          <t>google_p1</t>
+        </is>
+      </c>
+      <c r="M413" s="3" t="inlineStr"/>
+      <c r="N413" s="3" t="inlineStr"/>
+    </row>
+    <row r="414">
+      <c r="A414" s="3" t="inlineStr">
+        <is>
+          <t>Melbourne Private Hospital</t>
+        </is>
+      </c>
+      <c r="B414" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C414" s="3" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="D414" s="3" t="inlineStr">
+        <is>
+          <t>https://vahi.vic.gov.au/hospital-and-health-services/melbourne-private-hospital</t>
+        </is>
+      </c>
+      <c r="E414" s="3" t="inlineStr"/>
+      <c r="F414" s="3" t="inlineStr"/>
+      <c r="G414" s="3" t="inlineStr"/>
+      <c r="H414" s="3" t="inlineStr"/>
+      <c r="I414" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J414" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 14:13</t>
+        </is>
+      </c>
+      <c r="K414" s="3" t="inlineStr"/>
+      <c r="L414" s="3" t="inlineStr">
+        <is>
+          <t>google_p1</t>
+        </is>
+      </c>
+      <c r="M414" s="3" t="inlineStr"/>
+      <c r="N414" s="3" t="inlineStr"/>
+    </row>
+    <row r="415">
+      <c r="A415" s="3" t="inlineStr">
+        <is>
+          <t>Melbourne Eastern Private Hospital</t>
+        </is>
+      </c>
+      <c r="B415" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C415" s="3" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="D415" s="3" t="inlineStr">
+        <is>
+          <t>https://www.melbourneeastern.com.au/</t>
+        </is>
+      </c>
+      <c r="E415" s="3" t="inlineStr"/>
+      <c r="F415" s="3" t="inlineStr">
+        <is>
+          <t>03) 9720 3388</t>
+        </is>
+      </c>
+      <c r="G415" s="3" t="inlineStr"/>
+      <c r="H415" s="3" t="inlineStr"/>
+      <c r="I415" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J415" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 14:14</t>
+        </is>
+      </c>
+      <c r="K415" s="3" t="inlineStr"/>
+      <c r="L415" s="3" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M415" s="3" t="inlineStr"/>
+      <c r="N415" s="3" t="inlineStr"/>
+    </row>
+    <row r="416">
+      <c r="A416" s="3" t="inlineStr">
+        <is>
+          <t>Austin Health: Home</t>
+        </is>
+      </c>
+      <c r="B416" s="3" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C416" s="3" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="D416" s="3" t="inlineStr">
+        <is>
+          <t>https://www.austin.org.au/</t>
+        </is>
+      </c>
+      <c r="E416" s="3" t="inlineStr"/>
+      <c r="F416" s="3" t="inlineStr">
+        <is>
+          <t>03 9496 5000</t>
+        </is>
+      </c>
+      <c r="G416" s="3" t="inlineStr"/>
+      <c r="H416" s="3" t="inlineStr"/>
+      <c r="I416" s="3" t="inlineStr">
+        <is>
+          <t>no_email</t>
+        </is>
+      </c>
+      <c r="J416" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 14:14</t>
+        </is>
+      </c>
+      <c r="K416" s="3" t="inlineStr"/>
+      <c r="L416" s="3" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M416" s="3" t="inlineStr"/>
+      <c r="N416" s="3" t="inlineStr"/>
+    </row>
+    <row r="417">
+      <c r="A417" s="2" t="inlineStr">
+        <is>
+          <t>eAdmissions :: Melbourne Private Hospital</t>
+        </is>
+      </c>
+      <c r="B417" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C417" s="2" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="D417" s="2" t="inlineStr">
+        <is>
+          <t>https://melbourneprivatehospital.com.au/patients/eadmissions-registration</t>
+        </is>
+      </c>
+      <c r="E417" s="2" t="inlineStr">
+        <is>
+          <t>melbookings@healthscope.com.au</t>
+        </is>
+      </c>
+      <c r="F417" s="2" t="inlineStr">
+        <is>
+          <t>03 8341 3400</t>
+        </is>
+      </c>
+      <c r="G417" s="2" t="inlineStr"/>
+      <c r="H417" s="2" t="inlineStr">
+        <is>
+          <t>Streamline Operations: Custom Digital Solution Proposal</t>
+        </is>
+      </c>
+      <c r="I417" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J417" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 14:14</t>
+        </is>
+      </c>
+      <c r="K417" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T14:17:08.228134</t>
+        </is>
+      </c>
+      <c r="L417" s="2" t="inlineStr">
+        <is>
+          <t>google_p2</t>
+        </is>
+      </c>
+      <c r="M417" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N417" s="2" t="inlineStr"/>
+    </row>
+    <row r="418">
+      <c r="A418" s="2" t="inlineStr">
+        <is>
+          <t>Private Hospital Melbourne | Adeney Private Hospital, Kew</t>
+        </is>
+      </c>
+      <c r="B418" s="2" t="inlineStr">
+        <is>
+          <t>hospital</t>
+        </is>
+      </c>
+      <c r="C418" s="2" t="inlineStr">
+        <is>
+          <t>Melbourne</t>
+        </is>
+      </c>
+      <c r="D418" s="2" t="inlineStr">
+        <is>
+          <t>https://adeneyprivate.com.au/</t>
+        </is>
+      </c>
+      <c r="E418" s="2" t="inlineStr">
+        <is>
+          <t>care@adeneyprivate.com.au</t>
+        </is>
+      </c>
+      <c r="F418" s="2" t="inlineStr">
+        <is>
+          <t>03) 7049 5000</t>
+        </is>
+      </c>
+      <c r="G418" s="2" t="inlineStr"/>
+      <c r="H418" s="2" t="inlineStr">
+        <is>
+          <t>Transform Operations: Tailored Digital Solution Proposal</t>
+        </is>
+      </c>
+      <c r="I418" s="2" t="inlineStr">
+        <is>
+          <t>email_sent</t>
+        </is>
+      </c>
+      <c r="J418" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08 14:17</t>
+        </is>
+      </c>
+      <c r="K418" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-08T14:20:36.204106</t>
+        </is>
+      </c>
+      <c r="L418" s="2" t="inlineStr">
+        <is>
+          <t>google_p3</t>
+        </is>
+      </c>
+      <c r="M418" s="2" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="N418" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>